<commit_message>
Yayın: elektrik birim fiyatı kitabın kendi kuruluşuna çevrildi
Metraj cetveli, keşif özetleri ve teklif cetvelleri ELEKTRİK-BF revizyon
koduyla işaretlendi: birim fiyat = malzeme rayici x 1,25 + pozun kendi
montaj bedeli (işçilik rayicinden kurulur, oran değildir).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -2278,11 +2278,11 @@
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>48908.37</v>
+        <v>49741.82</v>
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F25" s="20">
@@ -2298,7 +2298,7 @@
         <v/>
       </c>
       <c r="I25" s="13" t="n">
-        <v>41083.03</v>
+        <v>41783.13</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
@@ -2318,11 +2318,11 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>10963.58</v>
+        <v>12003.52</v>
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F26" s="20">
@@ -2338,7 +2338,7 @@
         <v/>
       </c>
       <c r="I26" s="13" t="n">
-        <v>9209.41</v>
+        <v>10082.96</v>
       </c>
     </row>
     <row r="27" ht="14" customHeight="1">
@@ -2358,11 +2358,11 @@
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>12658.36</v>
+        <v>13847.2</v>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F27" s="20">
@@ -2378,7 +2378,7 @@
         <v/>
       </c>
       <c r="I27" s="13" t="n">
-        <v>10633.02</v>
+        <v>11631.65</v>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
@@ -2398,11 +2398,11 @@
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>5460.08</v>
+        <v>5280.06</v>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F28" s="20">
@@ -2418,7 +2418,7 @@
         <v/>
       </c>
       <c r="I28" s="13" t="n">
-        <v>4586.47</v>
+        <v>4435.25</v>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
@@ -2438,11 +2438,11 @@
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>7356.08</v>
+        <v>7048.52</v>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F29" s="20">
@@ -2458,7 +2458,7 @@
         <v/>
       </c>
       <c r="I29" s="13" t="n">
-        <v>6179.11</v>
+        <v>5920.76</v>
       </c>
     </row>
     <row r="30" ht="14" customHeight="1">
@@ -2478,11 +2478,11 @@
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>1670.19</v>
+        <v>1709.76</v>
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F30" s="20">
@@ -2498,7 +2498,7 @@
         <v/>
       </c>
       <c r="I30" s="13" t="n">
-        <v>1402.96</v>
+        <v>1436.2</v>
       </c>
     </row>
     <row r="31" ht="14" customHeight="1">
@@ -2518,11 +2518,11 @@
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>59651.77</v>
+        <v>53225.97</v>
       </c>
       <c r="E31" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F31" s="20">
@@ -2538,7 +2538,7 @@
         <v/>
       </c>
       <c r="I31" s="13" t="n">
-        <v>50107.49</v>
+        <v>44709.81</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -2558,11 +2558,11 @@
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>2327.86</v>
+        <v>2640.66</v>
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F32" s="20">
@@ -2578,7 +2578,7 @@
         <v/>
       </c>
       <c r="I32" s="13" t="n">
-        <v>1955.4</v>
+        <v>2218.15</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -2598,11 +2598,11 @@
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>243.05</v>
+        <v>223.96</v>
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F33" s="20">
@@ -2618,7 +2618,7 @@
         <v/>
       </c>
       <c r="I33" s="13" t="n">
-        <v>204.16</v>
+        <v>188.13</v>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
@@ -2638,11 +2638,11 @@
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>79.31999999999999</v>
+        <v>84.91</v>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F34" s="20">
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="I34" s="13" t="n">
-        <v>66.63</v>
+        <v>71.31999999999999</v>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
@@ -2678,11 +2678,11 @@
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>309.53</v>
+        <v>290.5</v>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F35" s="20">
@@ -2698,7 +2698,7 @@
         <v/>
       </c>
       <c r="I35" s="13" t="n">
-        <v>260.01</v>
+        <v>244.02</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
@@ -2718,11 +2718,11 @@
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>428.92</v>
+        <v>395.44</v>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F36" s="20">
@@ -2738,7 +2738,7 @@
         <v/>
       </c>
       <c r="I36" s="13" t="n">
-        <v>360.29</v>
+        <v>332.17</v>
       </c>
     </row>
     <row r="37" ht="14" customHeight="1">
@@ -2758,11 +2758,11 @@
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>18.91</v>
+        <v>28.05</v>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F37" s="20">
@@ -2778,7 +2778,7 @@
         <v/>
       </c>
       <c r="I37" s="13" t="n">
-        <v>15.88</v>
+        <v>23.56</v>
       </c>
     </row>
     <row r="38" ht="14" customHeight="1">
@@ -2798,11 +2798,11 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>30.18</v>
+        <v>39.41</v>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F38" s="20">
@@ -2818,7 +2818,7 @@
         <v/>
       </c>
       <c r="I38" s="13" t="n">
-        <v>25.35</v>
+        <v>33.1</v>
       </c>
     </row>
     <row r="39" ht="14" customHeight="1">
@@ -2838,11 +2838,11 @@
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>44.96</v>
+        <v>88.59</v>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F39" s="20">
@@ -2858,7 +2858,7 @@
         <v/>
       </c>
       <c r="I39" s="13" t="n">
-        <v>37.77</v>
+        <v>74.42</v>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
@@ -2878,11 +2878,11 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>2121.73</v>
+        <v>1848.1</v>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F40" s="20">
@@ -2898,7 +2898,7 @@
         <v/>
       </c>
       <c r="I40" s="13" t="n">
-        <v>1782.25</v>
+        <v>1552.4</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
@@ -2918,11 +2918,11 @@
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>3089.16</v>
+        <v>2646.28</v>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F41" s="20">
@@ -2938,7 +2938,7 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
-        <v>2594.89</v>
+        <v>2222.88</v>
       </c>
     </row>
     <row r="42" ht="14" customHeight="1">
@@ -2958,11 +2958,11 @@
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>11812.61</v>
+        <v>9896.620000000001</v>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F42" s="20">
@@ -2978,7 +2978,7 @@
         <v/>
       </c>
       <c r="I42" s="13" t="n">
-        <v>9922.59</v>
+        <v>8313.16</v>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
@@ -2998,11 +2998,11 @@
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>9640.309999999999</v>
+        <v>9265.620000000001</v>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F43" s="20">
@@ -3018,7 +3018,7 @@
         <v/>
       </c>
       <c r="I43" s="13" t="n">
-        <v>8097.86</v>
+        <v>7783.12</v>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
@@ -3038,11 +3038,11 @@
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>723278.66</v>
+        <v>576288.2</v>
       </c>
       <c r="E44" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F44" s="20">
@@ -3058,7 +3058,7 @@
         <v/>
       </c>
       <c r="I44" s="13" t="n">
-        <v>607554.0699999999</v>
+        <v>484082.09</v>
       </c>
     </row>
     <row r="45" ht="14" customHeight="1">
@@ -3078,11 +3078,11 @@
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>123273.35</v>
+        <v>99145.64999999999</v>
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F45" s="20">
@@ -3098,7 +3098,7 @@
         <v/>
       </c>
       <c r="I45" s="13" t="n">
-        <v>103549.61</v>
+        <v>83282.35000000001</v>
       </c>
     </row>
     <row r="46" ht="14" customHeight="1">
@@ -3118,11 +3118,11 @@
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>24136.06</v>
+        <v>20726.2</v>
       </c>
       <c r="E46" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F46" s="20">
@@ -3138,7 +3138,7 @@
         <v/>
       </c>
       <c r="I46" s="13" t="n">
-        <v>20274.29</v>
+        <v>17410.01</v>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
@@ -3158,11 +3158,11 @@
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>660.4</v>
+        <v>572.8</v>
       </c>
       <c r="E47" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F47" s="20">
@@ -3178,7 +3178,7 @@
         <v/>
       </c>
       <c r="I47" s="13" t="n">
-        <v>554.74</v>
+        <v>481.15</v>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
@@ -3198,11 +3198,11 @@
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>179.47</v>
+        <v>185.85</v>
       </c>
       <c r="E48" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,625</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
         </is>
       </c>
       <c r="F48" s="20">
@@ -3218,7 +3218,7 @@
         <v/>
       </c>
       <c r="I48" s="13" t="n">
-        <v>150.75</v>
+        <v>156.11</v>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Yayın: yüklenici unvanı MAHMUT TARI - MARFEN, antet yer tutucuları kaldırıldı
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -791,7 +791,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -3538,7 +3538,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -6534,7 +6534,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6885,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7174,7 +7174,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7463,7 +7463,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7752,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: yüklenici künyesi ticaret sicili kaydına göre düzeltildi
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -530,7 +530,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TEKLİF İCMALİ — MARFEN</t>
+          <t>TEKLİF İCMALİ — MAFREN</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -3538,7 +3538,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -6534,7 +6534,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6885,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7174,7 +7174,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7463,7 +7463,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7752,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI - MARFEN MÜHENDİSLİK TASARIM VE DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: firma künyesi (sicil, Mersis, telefon, e-posta) bütün belgelerde
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -791,7 +791,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -3538,7 +3538,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -6534,7 +6534,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6885,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7174,7 +7174,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7463,7 +7463,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7752,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: teklif geçerlilik tarihi 26.12.2027
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -791,7 +791,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.12.2027 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -3538,7 +3538,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.12.2027 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.12.2027 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -6534,7 +6534,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.12.2027 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -6885,7 +6885,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.12.2027 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7174,7 +7174,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.12.2027 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7463,7 +7463,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.12.2027 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7752,7 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.11.2026 · KDV hariç fiyatlar</t>
+          <t>MAHMUT TARI MAFREN MÜHENDİSLİK DANIŞMANLIK HİZMETLERİ · MAHMUT TARI · Ticaret sicil no Gölcük/6196 · Mersis 4943840532200001 · Tel 0541 553 66 86 · mahmuttari@gmail.com · 26.08.2026 · geçerlilik 26.12.2027 · KDV hariç fiyatlar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: elektrik pozlarından montaj bedeli çıkarıldı
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -1442,11 +1442,11 @@
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>12003.52</v>
+        <v>8433.52</v>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F23" s="20">
@@ -1462,7 +1462,7 @@
         <v/>
       </c>
       <c r="I23" s="13" t="n">
-        <v>10082.96</v>
+        <v>7084.16</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
@@ -1482,11 +1482,11 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>5280.06</v>
+        <v>4200.06</v>
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F24" s="20">
@@ -1502,7 +1502,7 @@
         <v/>
       </c>
       <c r="I24" s="13" t="n">
-        <v>4435.25</v>
+        <v>3528.05</v>
       </c>
     </row>
     <row r="25" ht="14" customHeight="1">
@@ -1522,11 +1522,11 @@
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1709.76</v>
+        <v>1284.76</v>
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F25" s="20">
@@ -1542,7 +1542,7 @@
         <v/>
       </c>
       <c r="I25" s="13" t="n">
-        <v>1436.2</v>
+        <v>1079.2</v>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
@@ -1562,11 +1562,11 @@
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>223.96</v>
+        <v>186.96</v>
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F26" s="20">
@@ -1582,7 +1582,7 @@
         <v/>
       </c>
       <c r="I26" s="13" t="n">
-        <v>188.13</v>
+        <v>157.05</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
@@ -1602,11 +1602,11 @@
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>290.5</v>
+        <v>238.1</v>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F27" s="20">
@@ -1622,7 +1622,7 @@
         <v/>
       </c>
       <c r="I27" s="13" t="n">
-        <v>244.02</v>
+        <v>200</v>
       </c>
     </row>
     <row r="28" ht="14" customHeight="1">
@@ -1642,11 +1642,11 @@
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>28.05</v>
+        <v>14.55</v>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F28" s="20">
@@ -1662,7 +1662,7 @@
         <v/>
       </c>
       <c r="I28" s="13" t="n">
-        <v>23.56</v>
+        <v>12.22</v>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
@@ -1682,11 +1682,11 @@
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>39.41</v>
+        <v>23.21</v>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F29" s="20">
@@ -1702,7 +1702,7 @@
         <v/>
       </c>
       <c r="I29" s="13" t="n">
-        <v>33.1</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="30" ht="14" customHeight="1">
@@ -1722,11 +1722,11 @@
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>88.59</v>
+        <v>34.59</v>
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F30" s="20">
@@ -1742,7 +1742,7 @@
         <v/>
       </c>
       <c r="I30" s="13" t="n">
-        <v>74.42</v>
+        <v>29.06</v>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
@@ -1762,11 +1762,11 @@
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>1848.1</v>
+        <v>1632.1</v>
       </c>
       <c r="E31" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F31" s="20">
@@ -1782,7 +1782,7 @@
         <v/>
       </c>
       <c r="I31" s="13" t="n">
-        <v>1552.4</v>
+        <v>1370.96</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
@@ -1802,11 +1802,11 @@
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>2646.28</v>
+        <v>2376.28</v>
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F32" s="20">
@@ -1822,7 +1822,7 @@
         <v/>
       </c>
       <c r="I32" s="13" t="n">
-        <v>2222.88</v>
+        <v>1996.08</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
@@ -1842,11 +1842,11 @@
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>576288.2</v>
+        <v>556368.2</v>
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F33" s="20">
@@ -1862,7 +1862,7 @@
         <v/>
       </c>
       <c r="I33" s="13" t="n">
-        <v>484082.09</v>
+        <v>467349.29</v>
       </c>
     </row>
     <row r="34" ht="14" customHeight="1">
@@ -1882,11 +1882,11 @@
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>99145.64999999999</v>
+        <v>94825.64999999999</v>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F34" s="20">
@@ -1902,7 +1902,7 @@
         <v/>
       </c>
       <c r="I34" s="13" t="n">
-        <v>83282.35000000001</v>
+        <v>79653.55</v>
       </c>
     </row>
     <row r="35" ht="14" customHeight="1">
@@ -1922,11 +1922,11 @@
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>20726.2</v>
+        <v>18566.2</v>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F35" s="20">
@@ -1942,7 +1942,7 @@
         <v/>
       </c>
       <c r="I35" s="13" t="n">
-        <v>17410.01</v>
+        <v>15595.61</v>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
@@ -1962,11 +1962,11 @@
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>572.8</v>
+        <v>508</v>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F36" s="20">
@@ -1982,7 +1982,7 @@
         <v/>
       </c>
       <c r="I36" s="13" t="n">
-        <v>481.15</v>
+        <v>426.72</v>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
@@ -2002,11 +2002,11 @@
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>185.85</v>
+        <v>138.05</v>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25 + montaj</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F37" s="20">
@@ -2022,7 +2022,7 @@
         <v/>
       </c>
       <c r="I37" s="13" t="n">
-        <v>156.11</v>
+        <v>115.96</v>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">

</xml_diff>

<commit_message>
Yayın: yağmur suyu iniş borusu Ø70 sert PVC
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1265,24 +1265,24 @@
         <v>381.49</v>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
+    <row r="19" ht="14" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
-          <t>15.540.1537</t>
+          <t>15.315.1001</t>
         </is>
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası</t>
+          <t>Ø70 sert PVC yağmur suyu iniş borusu temini ve yerine tesbiti</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D19" s="5" t="n">
-        <v>296.13</v>
+        <v>207.41</v>
       </c>
       <c r="E19" s="19" t="inlineStr">
         <is>
@@ -1302,18 +1302,18 @@
         <v/>
       </c>
       <c r="I19" s="13" t="n">
-        <v>248.75</v>
+        <v>174.22</v>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="17" t="inlineStr">
         <is>
-          <t>15.540.1606</t>
+          <t>15.540.1537</t>
         </is>
       </c>
       <c r="B20" s="18" t="inlineStr">
         <is>
-          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası</t>
+          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="D20" s="5" t="n">
-        <v>386.03</v>
+        <v>296.13</v>
       </c>
       <c r="E20" s="19" t="inlineStr">
         <is>
@@ -1342,27 +1342,27 @@
         <v/>
       </c>
       <c r="I20" s="13" t="n">
-        <v>324.27</v>
+        <v>248.75</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>15.550.1002</t>
+          <t>15.540.1606</t>
         </is>
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>1,50 mm sacdan bükme kapı kasası yapılması ve yerine konulması — servis bölümü iç kapıları</t>
+          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>218.54</v>
+        <v>386.03</v>
       </c>
       <c r="E21" s="19" t="inlineStr">
         <is>
@@ -1382,18 +1382,18 @@
         <v/>
       </c>
       <c r="I21" s="13" t="n">
-        <v>183.57</v>
+        <v>324.27</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>15.550.1202</t>
+          <t>15.550.1002</t>
         </is>
       </c>
       <c r="B22" s="18" t="inlineStr">
         <is>
-          <t>Lama ve profil demirlerden mahya, saçak ve köşe kapama profilleri</t>
+          <t>1,50 mm sacdan bükme kapı kasası yapılması ve yerine konulması — servis bölümü iç kapıları</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1402,7 +1402,7 @@
         </is>
       </c>
       <c r="D22" s="5" t="n">
-        <v>175.8</v>
+        <v>218.54</v>
       </c>
       <c r="E22" s="19" t="inlineStr">
         <is>
@@ -1422,31 +1422,31 @@
         <v/>
       </c>
       <c r="I22" s="13" t="n">
-        <v>147.67</v>
+        <v>183.57</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>30.100.2105</t>
+          <t>15.550.1202</t>
         </is>
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>Kümes dağıtım panosu (sıva üstü galvanizli sac tablo, 0,40-0,50 m²)</t>
+          <t>Lama ve profil demirlerden mahya, saçak ve köşe kapama profilleri</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D23" s="5" t="n">
-        <v>8433.52</v>
+        <v>175.8</v>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>ÇŞB 2026 birim fiyat kitabı</t>
         </is>
       </c>
       <c r="F23" s="20">
@@ -1462,18 +1462,18 @@
         <v/>
       </c>
       <c r="I23" s="13" t="n">
-        <v>7084.16</v>
+        <v>147.67</v>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>30.110.1102</t>
+          <t>30.100.2105</t>
         </is>
       </c>
       <c r="B24" s="18" t="inlineStr">
         <is>
-          <t>Termik-manyetik kompakt şalter 3x100 A, Icu 35 kA — kümes besleme</t>
+          <t>Kümes dağıtım panosu (sıva üstü galvanizli sac tablo, 0,40-0,50 m²)</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1482,7 +1482,7 @@
         </is>
       </c>
       <c r="D24" s="5" t="n">
-        <v>4200.06</v>
+        <v>8433.52</v>
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
@@ -1502,18 +1502,18 @@
         <v/>
       </c>
       <c r="I24" s="13" t="n">
-        <v>3528.05</v>
-      </c>
-    </row>
-    <row r="25" ht="14" customHeight="1">
+        <v>7084.16</v>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>30.115.1003</t>
+          <t>30.110.1102</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA</t>
+          <t>Termik-manyetik kompakt şalter 3x100 A, Icu 35 kA — kümes besleme</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1522,7 +1522,7 @@
         </is>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1284.76</v>
+        <v>4200.06</v>
       </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
@@ -1542,27 +1542,27 @@
         <v/>
       </c>
       <c r="I25" s="13" t="n">
-        <v>1079.2</v>
-      </c>
-    </row>
-    <row r="26" ht="22" customHeight="1">
+        <v>3528.05</v>
+      </c>
+    </row>
+    <row r="26" ht="14" customHeight="1">
       <c r="A26" s="17" t="inlineStr">
         <is>
-          <t>30.140.1105</t>
+          <t>30.115.1003</t>
         </is>
       </c>
       <c r="B26" s="18" t="inlineStr">
         <is>
-          <t>Çıplak bakır tel 25 mm² — eşpotansiyel bara ve topraklama iletkeni</t>
+          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D26" s="5" t="n">
-        <v>186.96</v>
+        <v>1284.76</v>
       </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
@@ -1582,18 +1582,18 @@
         <v/>
       </c>
       <c r="I26" s="13" t="n">
-        <v>157.05</v>
+        <v>1079.2</v>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>30.140.3104</t>
+          <t>30.140.1105</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>YVV (NYY) 1 kV yeraltı kablosu ile kolon hattı tesisi — 1x25 mm²</t>
+          <t>Çıplak bakır tel 25 mm² — eşpotansiyel bara ve topraklama iletkeni</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1602,7 +1602,7 @@
         </is>
       </c>
       <c r="D27" s="5" t="n">
-        <v>238.1</v>
+        <v>186.96</v>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
@@ -1622,18 +1622,18 @@
         <v/>
       </c>
       <c r="I27" s="13" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="28" ht="14" customHeight="1">
+        <v>157.05</v>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
         <is>
-          <t>30.150.1401</t>
+          <t>30.140.3104</t>
         </is>
       </c>
       <c r="B28" s="18" t="inlineStr">
         <is>
-          <t>Halojensiz H07Z tipi iletken 1x1,5 mm² ile kumanda tesisatı</t>
+          <t>YVV (NYY) 1 kV yeraltı kablosu ile kolon hattı tesisi — 1x25 mm²</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1642,7 +1642,7 @@
         </is>
       </c>
       <c r="D28" s="5" t="n">
-        <v>14.55</v>
+        <v>238.1</v>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
@@ -1662,18 +1662,18 @@
         <v/>
       </c>
       <c r="I28" s="13" t="n">
-        <v>12.22</v>
+        <v>200</v>
       </c>
     </row>
     <row r="29" ht="14" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>30.150.1402</t>
+          <t>30.150.1401</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>Halojensiz H07Z tipi iletken 1x2,5 mm² ile tesisat</t>
+          <t>Halojensiz H07Z tipi iletken 1x1,5 mm² ile kumanda tesisatı</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1682,7 +1682,7 @@
         </is>
       </c>
       <c r="D29" s="5" t="n">
-        <v>23.21</v>
+        <v>14.55</v>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
@@ -1702,18 +1702,18 @@
         <v/>
       </c>
       <c r="I29" s="13" t="n">
-        <v>19.5</v>
+        <v>12.22</v>
       </c>
     </row>
     <row r="30" ht="14" customHeight="1">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>30.160.6102</t>
+          <t>30.150.1402</t>
         </is>
       </c>
       <c r="B30" s="18" t="inlineStr">
         <is>
-          <t>Boş boru döşemesi — 25-32 mm PVC boru</t>
+          <t>Halojensiz H07Z tipi iletken 1x2,5 mm² ile tesisat</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1722,7 +1722,7 @@
         </is>
       </c>
       <c r="D30" s="5" t="n">
-        <v>34.59</v>
+        <v>23.21</v>
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
@@ -1742,27 +1742,27 @@
         <v/>
       </c>
       <c r="I30" s="13" t="n">
-        <v>29.06</v>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="31" ht="14" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>30.170.1601</t>
+          <t>30.160.6102</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 1800 lm — servis bölümü</t>
+          <t>Boş boru döşemesi — 25-32 mm PVC boru</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>1632.1</v>
+        <v>34.59</v>
       </c>
       <c r="E31" s="19" t="inlineStr">
         <is>
@@ -1782,18 +1782,18 @@
         <v/>
       </c>
       <c r="I31" s="13" t="n">
-        <v>1370.96</v>
+        <v>29.06</v>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>30.170.1602</t>
+          <t>30.170.1601</t>
         </is>
       </c>
       <c r="B32" s="18" t="inlineStr">
         <is>
-          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 2700 lm — kümes genel aydınlatması</t>
+          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 1800 lm — servis bölümü</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1802,7 +1802,7 @@
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>2376.28</v>
+        <v>1632.1</v>
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
@@ -1822,18 +1822,18 @@
         <v/>
       </c>
       <c r="I32" s="13" t="n">
-        <v>1996.08</v>
+        <v>1370.96</v>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>30.740.1106</t>
+          <t>30.170.1602</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
+          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 2700 lm — kümes genel aydınlatması</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1842,7 +1842,7 @@
         </is>
       </c>
       <c r="D33" s="5" t="n">
-        <v>556368.2</v>
+        <v>2376.28</v>
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
@@ -1862,18 +1862,18 @@
         <v/>
       </c>
       <c r="I33" s="13" t="n">
-        <v>467349.29</v>
-      </c>
-    </row>
-    <row r="34" ht="14" customHeight="1">
+        <v>1996.08</v>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>30.740.5406</t>
+          <t>30.740.1106</t>
         </is>
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>94825.64999999999</v>
+        <v>556368.2</v>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
@@ -1902,18 +1902,18 @@
         <v/>
       </c>
       <c r="I34" s="13" t="n">
-        <v>79653.55</v>
+        <v>467349.29</v>
       </c>
     </row>
     <row r="35" ht="14" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>30.750.1502</t>
+          <t>30.740.5406</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>18566.2</v>
+        <v>94825.64999999999</v>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
@@ -1942,27 +1942,27 @@
         <v/>
       </c>
       <c r="I35" s="13" t="n">
-        <v>15595.61</v>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
+        <v>79653.55</v>
+      </c>
+    </row>
+    <row r="36" ht="14" customHeight="1">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>30.750.2001</t>
+          <t>30.750.1502</t>
         </is>
       </c>
       <c r="B36" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>508</v>
+        <v>18566.2</v>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
@@ -1982,18 +1982,18 @@
         <v/>
       </c>
       <c r="I36" s="13" t="n">
-        <v>426.72</v>
+        <v>15595.61</v>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>30.750.3002</t>
+          <t>30.750.2001</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>138.05</v>
+        <v>508</v>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
@@ -2022,18 +2022,18 @@
         <v/>
       </c>
       <c r="I37" s="13" t="n">
-        <v>115.96</v>
+        <v>426.72</v>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>30.750.3002</t>
         </is>
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2042,11 +2042,11 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>393.69</v>
+        <v>138.05</v>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F38" s="20">
@@ -2062,27 +2062,27 @@
         <v/>
       </c>
       <c r="I38" s="13" t="n">
-        <v>330.7</v>
-      </c>
-    </row>
-    <row r="39" ht="14" customHeight="1">
+        <v>115.96</v>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>43.527.1001</t>
         </is>
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
+          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>271.25</v>
+        <v>393.69</v>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
@@ -2102,27 +2102,27 @@
         <v/>
       </c>
       <c r="I39" s="13" t="n">
-        <v>227.85</v>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1">
+        <v>330.7</v>
+      </c>
+    </row>
+    <row r="40" ht="14" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
+          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>1035.88</v>
+        <v>271.25</v>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
@@ -2142,18 +2142,18 @@
         <v/>
       </c>
       <c r="I40" s="13" t="n">
-        <v>870.14</v>
+        <v>227.85</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0175</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>3199.68</v>
+        <v>1035.88</v>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
@@ -2182,18 +2182,18 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
-        <v>2687.73</v>
+        <v>870.14</v>
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0177</t>
+          <t>TKDK-0175</t>
         </is>
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2202,7 +2202,7 @@
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>835.1</v>
+        <v>3199.68</v>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
@@ -2222,6 +2222,46 @@
         <v/>
       </c>
       <c r="I42" s="13" t="n">
+        <v>2687.73</v>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0177</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>835.1</v>
+      </c>
+      <c r="E43" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F43" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G43" s="5">
+        <f>D43*(1-F43)</f>
+        <v/>
+      </c>
+      <c r="H43" s="5">
+        <f>D43*$D$3</f>
+        <v/>
+      </c>
+      <c r="I43" s="13" t="n">
         <v>701.48</v>
       </c>
     </row>
@@ -2843,21 +2883,21 @@
       </c>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>15.315.1001</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan iniş borusu yapılması — ø100</t>
+          <t>Ø70 sert PVC yağmur suyu iniş borusu temini ve yerine tesbiti</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>40.96</v>
+        <v>51.2</v>
       </c>
       <c r="F23" s="23">
         <f>IFERROR(VLOOKUP($B23,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4279,21 +4319,21 @@
       </c>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>15.315.1001</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan iniş borusu yapılması — ø100</t>
+          <t>Ø70 sert PVC yağmur suyu iniş borusu temini ve yerine tesbiti</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>40.96</v>
+        <v>51.2</v>
       </c>
       <c r="F23" s="23">
         <f>IFERROR(VLOOKUP($B23,'Fiyatlar'!$A:$I,9,FALSE),0)</f>

</xml_diff>

<commit_message>
Yayın: jeneratör tesisatı hibe dışına alındı
Jeneratör grubu, ses izolasyon kabini ve otomatik transfer şalteri
MARFEN proformasına (36) girdi. Uygun harcama 290.859'dan 270.123
Avro'ya indi; kriter 1 kademesi ve 5 puan aynı, eşiğe kalan pay
29.877 Avro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>'01 Kümes A Blok'!$G$48</f>
+        <f>'01 Kümes A Blok'!$G$46</f>
         <v/>
       </c>
       <c r="D4" s="6">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>'02 Kümes B Blok'!$G$48</f>
+        <f>'02 Kümes B Blok'!$G$46</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1865,15 +1865,15 @@
         <v>1996.08</v>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
+    <row r="34" ht="14" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>30.740.1106</t>
+          <t>30.750.1502</t>
         </is>
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>556368.2</v>
+        <v>18566.2</v>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
@@ -1902,27 +1902,27 @@
         <v/>
       </c>
       <c r="I34" s="13" t="n">
-        <v>467349.29</v>
-      </c>
-    </row>
-    <row r="35" ht="14" customHeight="1">
+        <v>15595.61</v>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>30.740.5406</t>
+          <t>30.750.2001</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>94825.64999999999</v>
+        <v>508</v>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
@@ -1942,27 +1942,27 @@
         <v/>
       </c>
       <c r="I35" s="13" t="n">
-        <v>79653.55</v>
-      </c>
-    </row>
-    <row r="36" ht="14" customHeight="1">
+        <v>426.72</v>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>30.750.1502</t>
+          <t>30.750.3002</t>
         </is>
       </c>
       <c r="B36" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
+          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>18566.2</v>
+        <v>138.05</v>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
@@ -1982,18 +1982,18 @@
         <v/>
       </c>
       <c r="I36" s="13" t="n">
-        <v>15595.61</v>
+        <v>115.96</v>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>30.750.2001</t>
+          <t>43.527.1001</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
+          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2002,11 +2002,11 @@
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>508</v>
+        <v>393.69</v>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F37" s="20">
@@ -2022,31 +2022,31 @@
         <v/>
       </c>
       <c r="I37" s="13" t="n">
-        <v>426.72</v>
-      </c>
-    </row>
-    <row r="38" ht="22" customHeight="1">
+        <v>330.7</v>
+      </c>
+    </row>
+    <row r="38" ht="14" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>30.750.3002</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
+          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>138.05</v>
+        <v>271.25</v>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F38" s="20">
@@ -2062,27 +2062,27 @@
         <v/>
       </c>
       <c r="I38" s="13" t="n">
-        <v>115.96</v>
+        <v>227.85</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>393.69</v>
+        <v>1035.88</v>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
@@ -2102,27 +2102,27 @@
         <v/>
       </c>
       <c r="I39" s="13" t="n">
-        <v>330.7</v>
-      </c>
-    </row>
-    <row r="40" ht="14" customHeight="1">
+        <v>870.14</v>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>TKDK-0175</t>
         </is>
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
+          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>271.25</v>
+        <v>3199.68</v>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
@@ -2142,18 +2142,18 @@
         <v/>
       </c>
       <c r="I40" s="13" t="n">
-        <v>227.85</v>
+        <v>2687.73</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>TKDK-0177</t>
         </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
+          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>1035.88</v>
+        <v>835.1</v>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
@@ -2182,86 +2182,6 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
-        <v>870.14</v>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="17" t="inlineStr">
-        <is>
-          <t>TKDK-0175</t>
-        </is>
-      </c>
-      <c r="B42" s="18" t="inlineStr">
-        <is>
-          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="n">
-        <v>3199.68</v>
-      </c>
-      <c r="E42" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F42" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G42" s="5">
-        <f>D42*(1-F42)</f>
-        <v/>
-      </c>
-      <c r="H42" s="5">
-        <f>D42*$D$3</f>
-        <v/>
-      </c>
-      <c r="I42" s="13" t="n">
-        <v>2687.73</v>
-      </c>
-    </row>
-    <row r="43" ht="22" customHeight="1">
-      <c r="A43" s="17" t="inlineStr">
-        <is>
-          <t>TKDK-0177</t>
-        </is>
-      </c>
-      <c r="B43" s="18" t="inlineStr">
-        <is>
-          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="n">
-        <v>835.1</v>
-      </c>
-      <c r="E43" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F43" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G43" s="5">
-        <f>D43*(1-F43)</f>
-        <v/>
-      </c>
-      <c r="H43" s="5">
-        <f>D43*$D$3</f>
-        <v/>
-      </c>
-      <c r="I43" s="13" t="n">
         <v>701.48</v>
       </c>
     </row>
@@ -2280,7 +2200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3590,113 +3510,51 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="3" t="n">
-        <v>41</v>
-      </c>
-      <c r="B46" s="21" t="inlineStr">
-        <is>
-          <t>30.740.1106</t>
-        </is>
-      </c>
-      <c r="C46" s="18" t="inlineStr">
-        <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E46" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" s="23">
-        <f>IFERROR(VLOOKUP($B46,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G46" s="5">
-        <f>E46*F46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" ht="14" customHeight="1">
-      <c r="A47" s="3" t="n">
-        <v>42</v>
-      </c>
-      <c r="B47" s="21" t="inlineStr">
-        <is>
-          <t>30.740.5406</t>
-        </is>
-      </c>
-      <c r="C47" s="18" t="inlineStr">
-        <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E47" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="23">
-        <f>IFERROR(VLOOKUP($B47,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
+    <row r="46">
+      <c r="A46" s="7" t="n"/>
+      <c r="B46" s="7" t="n"/>
+      <c r="C46" s="24" t="inlineStr">
+        <is>
+          <t>ARA TOPLAM (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="n"/>
+      <c r="E46" s="7" t="n"/>
+      <c r="F46" s="7" t="n"/>
+      <c r="G46" s="9">
+        <f>SUM(G6:G45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n"/>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="25" t="inlineStr">
+        <is>
+          <t>KDV</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="4" t="n"/>
+      <c r="F47" s="4" t="n"/>
       <c r="G47" s="5">
-        <f>E47*F47</f>
+        <f>G46*'Fiyatlar'!$F$3</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="n"/>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="24" t="inlineStr">
-        <is>
-          <t>ARA TOPLAM (KDV hariç)</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="n"/>
-      <c r="E48" s="7" t="n"/>
-      <c r="F48" s="7" t="n"/>
-      <c r="G48" s="9">
-        <f>SUM(G6:G47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="25" t="inlineStr">
-        <is>
-          <t>KDV</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="5">
-        <f>G48*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="11" t="n"/>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="26" t="inlineStr">
+      <c r="A48" s="11" t="n"/>
+      <c r="B48" s="11" t="n"/>
+      <c r="C48" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="13">
-        <f>G48+G49</f>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="11" t="n"/>
+      <c r="F48" s="11" t="n"/>
+      <c r="G48" s="13">
+        <f>G46+G47</f>
         <v/>
       </c>
     </row>
@@ -3716,7 +3574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5026,113 +4884,51 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="3" t="n">
-        <v>41</v>
-      </c>
-      <c r="B46" s="21" t="inlineStr">
-        <is>
-          <t>30.740.1106</t>
-        </is>
-      </c>
-      <c r="C46" s="18" t="inlineStr">
-        <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E46" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" s="23">
-        <f>IFERROR(VLOOKUP($B46,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G46" s="5">
-        <f>E46*F46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" ht="14" customHeight="1">
-      <c r="A47" s="3" t="n">
-        <v>42</v>
-      </c>
-      <c r="B47" s="21" t="inlineStr">
-        <is>
-          <t>30.740.5406</t>
-        </is>
-      </c>
-      <c r="C47" s="18" t="inlineStr">
-        <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>ad</t>
-        </is>
-      </c>
-      <c r="E47" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="23">
-        <f>IFERROR(VLOOKUP($B47,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
+    <row r="46">
+      <c r="A46" s="7" t="n"/>
+      <c r="B46" s="7" t="n"/>
+      <c r="C46" s="24" t="inlineStr">
+        <is>
+          <t>ARA TOPLAM (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="n"/>
+      <c r="E46" s="7" t="n"/>
+      <c r="F46" s="7" t="n"/>
+      <c r="G46" s="9">
+        <f>SUM(G6:G45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n"/>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="25" t="inlineStr">
+        <is>
+          <t>KDV</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="n"/>
+      <c r="E47" s="4" t="n"/>
+      <c r="F47" s="4" t="n"/>
       <c r="G47" s="5">
-        <f>E47*F47</f>
+        <f>G46*'Fiyatlar'!$F$3</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="n"/>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="24" t="inlineStr">
-        <is>
-          <t>ARA TOPLAM (KDV hariç)</t>
-        </is>
-      </c>
-      <c r="D48" s="7" t="n"/>
-      <c r="E48" s="7" t="n"/>
-      <c r="F48" s="7" t="n"/>
-      <c r="G48" s="9">
-        <f>SUM(G6:G47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="25" t="inlineStr">
-        <is>
-          <t>KDV</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="5">
-        <f>G48*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="11" t="n"/>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="26" t="inlineStr">
+      <c r="A48" s="11" t="n"/>
+      <c r="B48" s="11" t="n"/>
+      <c r="C48" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="13">
-        <f>G48+G49</f>
+      <c r="D48" s="11" t="n"/>
+      <c r="E48" s="11" t="n"/>
+      <c r="F48" s="11" t="n"/>
+      <c r="G48" s="13">
+        <f>G46+G47</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: cetvellerde tutar yazan üç haneli miktardan hesaplanıyor
Yapı bazında teklifler (13, 14), keşif Excel'i (15) ve A3.1.1, teklif
sunum formuyla (28) kuruşuna kadar aynı toplamı veriyor:
14.251.205,62 TL. Cetveldeki miktarla birim fiyatın çarpımı yazan tutarı
veriyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -2321,7 +2321,7 @@
         </is>
       </c>
       <c r="E7" s="22" t="n">
-        <v>31.4285</v>
+        <v>31.428</v>
       </c>
       <c r="F7" s="23">
         <f>IFERROR(VLOOKUP($B7,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2445,7 +2445,7 @@
         </is>
       </c>
       <c r="E11" s="22" t="n">
-        <v>4.1599</v>
+        <v>4.16</v>
       </c>
       <c r="F11" s="23">
         <f>IFERROR(VLOOKUP($B11,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="E12" s="22" t="n">
-        <v>7.2875</v>
+        <v>7.287</v>
       </c>
       <c r="F12" s="23">
         <f>IFERROR(VLOOKUP($B12,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2507,7 +2507,7 @@
         </is>
       </c>
       <c r="E13" s="22" t="n">
-        <v>3.6375</v>
+        <v>3.637</v>
       </c>
       <c r="F13" s="23">
         <f>IFERROR(VLOOKUP($B13,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2538,7 +2538,7 @@
         </is>
       </c>
       <c r="E14" s="22" t="n">
-        <v>44.0481</v>
+        <v>44.048</v>
       </c>
       <c r="F14" s="23">
         <f>IFERROR(VLOOKUP($B14,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3695,7 +3695,7 @@
         </is>
       </c>
       <c r="E7" s="22" t="n">
-        <v>31.4285</v>
+        <v>31.428</v>
       </c>
       <c r="F7" s="23">
         <f>IFERROR(VLOOKUP($B7,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3819,7 +3819,7 @@
         </is>
       </c>
       <c r="E11" s="22" t="n">
-        <v>4.1599</v>
+        <v>4.16</v>
       </c>
       <c r="F11" s="23">
         <f>IFERROR(VLOOKUP($B11,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3850,7 +3850,7 @@
         </is>
       </c>
       <c r="E12" s="22" t="n">
-        <v>7.2875</v>
+        <v>7.287</v>
       </c>
       <c r="F12" s="23">
         <f>IFERROR(VLOOKUP($B12,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3881,7 +3881,7 @@
         </is>
       </c>
       <c r="E13" s="22" t="n">
-        <v>3.6375</v>
+        <v>3.637</v>
       </c>
       <c r="F13" s="23">
         <f>IFERROR(VLOOKUP($B13,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="E14" s="22" t="n">
-        <v>44.0481</v>
+        <v>44.048</v>
       </c>
       <c r="F14" s="23">
         <f>IFERROR(VLOOKUP($B14,'Fiyatlar'!$A:$I,9,FALSE),0)</f>

</xml_diff>

<commit_message>
Yayın: jeneratör grubu ve kabini hibe kapsamına geri alındı
Uygun harcama 270.122 -> 290.858 Avro; 300.000 kademesi altında, 5 puan
duruyor. Transfer şalteri hibe dışında kalmaya devam ediyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>'01 Kümes A Blok'!$G$46</f>
+        <f>'01 Kümes A Blok'!$G$48</f>
         <v/>
       </c>
       <c r="D4" s="6">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>'02 Kümes B Blok'!$G$46</f>
+        <f>'02 Kümes B Blok'!$G$48</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1865,15 +1865,15 @@
         <v>1996.08</v>
       </c>
     </row>
-    <row r="34" ht="14" customHeight="1">
+    <row r="34" ht="22" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>30.750.1502</t>
+          <t>30.740.1106</t>
         </is>
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>18566.2</v>
+        <v>556368.2</v>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
@@ -1902,27 +1902,27 @@
         <v/>
       </c>
       <c r="I34" s="13" t="n">
-        <v>15595.61</v>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
+        <v>467349.29</v>
+      </c>
+    </row>
+    <row r="35" ht="14" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>30.750.2001</t>
+          <t>30.740.5406</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>508</v>
+        <v>94825.64999999999</v>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
@@ -1942,27 +1942,27 @@
         <v/>
       </c>
       <c r="I35" s="13" t="n">
-        <v>426.72</v>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
+        <v>79653.55</v>
+      </c>
+    </row>
+    <row r="36" ht="14" customHeight="1">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>30.750.3002</t>
+          <t>30.750.1502</t>
         </is>
       </c>
       <c r="B36" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>138.05</v>
+        <v>18566.2</v>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
@@ -1982,18 +1982,18 @@
         <v/>
       </c>
       <c r="I36" s="13" t="n">
-        <v>115.96</v>
+        <v>15595.61</v>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>30.750.2001</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2002,11 +2002,11 @@
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>393.69</v>
+        <v>508</v>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F37" s="20">
@@ -2022,31 +2022,31 @@
         <v/>
       </c>
       <c r="I37" s="13" t="n">
-        <v>330.7</v>
-      </c>
-    </row>
-    <row r="38" ht="14" customHeight="1">
+        <v>426.72</v>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>30.750.3002</t>
         </is>
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
+          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>271.25</v>
+        <v>138.05</v>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F38" s="20">
@@ -2062,27 +2062,27 @@
         <v/>
       </c>
       <c r="I38" s="13" t="n">
-        <v>227.85</v>
+        <v>115.96</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>43.527.1001</t>
         </is>
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
+          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>1035.88</v>
+        <v>393.69</v>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
@@ -2102,27 +2102,27 @@
         <v/>
       </c>
       <c r="I39" s="13" t="n">
-        <v>870.14</v>
-      </c>
-    </row>
-    <row r="40" ht="22" customHeight="1">
+        <v>330.7</v>
+      </c>
+    </row>
+    <row r="40" ht="14" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0175</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>3199.68</v>
+        <v>271.25</v>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
@@ -2142,18 +2142,18 @@
         <v/>
       </c>
       <c r="I40" s="13" t="n">
-        <v>2687.73</v>
+        <v>227.85</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0177</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>835.1</v>
+        <v>1035.88</v>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
@@ -2182,6 +2182,86 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
+        <v>870.14</v>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0175</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>3199.68</v>
+      </c>
+      <c r="E42" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F42" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G42" s="5">
+        <f>D42*(1-F42)</f>
+        <v/>
+      </c>
+      <c r="H42" s="5">
+        <f>D42*$D$3</f>
+        <v/>
+      </c>
+      <c r="I42" s="13" t="n">
+        <v>2687.73</v>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0177</t>
+        </is>
+      </c>
+      <c r="B43" s="18" t="inlineStr">
+        <is>
+          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>835.1</v>
+      </c>
+      <c r="E43" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F43" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G43" s="5">
+        <f>D43*(1-F43)</f>
+        <v/>
+      </c>
+      <c r="H43" s="5">
+        <f>D43*$D$3</f>
+        <v/>
+      </c>
+      <c r="I43" s="13" t="n">
         <v>701.48</v>
       </c>
     </row>
@@ -2200,7 +2280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3510,51 +3590,113 @@
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="7" t="n"/>
-      <c r="B46" s="7" t="n"/>
-      <c r="C46" s="24" t="inlineStr">
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" s="21" t="inlineStr">
+        <is>
+          <t>30.740.1106</t>
+        </is>
+      </c>
+      <c r="C46" s="18" t="inlineStr">
+        <is>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="23">
+        <f>IFERROR(VLOOKUP($B46,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G46" s="5">
+        <f>E46*F46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="14" customHeight="1">
+      <c r="A47" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>30.740.5406</t>
+        </is>
+      </c>
+      <c r="C47" s="18" t="inlineStr">
+        <is>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="23">
+        <f>IFERROR(VLOOKUP($B47,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G47" s="5">
+        <f>E47*F47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="n"/>
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="24" t="inlineStr">
         <is>
           <t>ARA TOPLAM (KDV hariç)</t>
         </is>
       </c>
-      <c r="D46" s="7" t="n"/>
-      <c r="E46" s="7" t="n"/>
-      <c r="F46" s="7" t="n"/>
-      <c r="G46" s="9">
-        <f>SUM(G6:G45)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n"/>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="25" t="inlineStr">
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="9">
+        <f>SUM(G6:G47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n"/>
+      <c r="B49" s="4" t="n"/>
+      <c r="C49" s="25" t="inlineStr">
         <is>
           <t>KDV</t>
         </is>
       </c>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="5">
-        <f>G46*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="11" t="n"/>
-      <c r="B48" s="11" t="n"/>
-      <c r="C48" s="26" t="inlineStr">
+      <c r="D49" s="4" t="n"/>
+      <c r="E49" s="4" t="n"/>
+      <c r="F49" s="4" t="n"/>
+      <c r="G49" s="5">
+        <f>G48*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="n"/>
+      <c r="B50" s="11" t="n"/>
+      <c r="C50" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D48" s="11" t="n"/>
-      <c r="E48" s="11" t="n"/>
-      <c r="F48" s="11" t="n"/>
-      <c r="G48" s="13">
-        <f>G46+G47</f>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="11" t="n"/>
+      <c r="F50" s="11" t="n"/>
+      <c r="G50" s="13">
+        <f>G48+G49</f>
         <v/>
       </c>
     </row>
@@ -3574,7 +3716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4884,51 +5026,113 @@
         <v/>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="7" t="n"/>
-      <c r="B46" s="7" t="n"/>
-      <c r="C46" s="24" t="inlineStr">
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" s="21" t="inlineStr">
+        <is>
+          <t>30.740.1106</t>
+        </is>
+      </c>
+      <c r="C46" s="18" t="inlineStr">
+        <is>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="23">
+        <f>IFERROR(VLOOKUP($B46,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G46" s="5">
+        <f>E46*F46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="14" customHeight="1">
+      <c r="A47" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" s="21" t="inlineStr">
+        <is>
+          <t>30.740.5406</t>
+        </is>
+      </c>
+      <c r="C47" s="18" t="inlineStr">
+        <is>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="23">
+        <f>IFERROR(VLOOKUP($B47,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G47" s="5">
+        <f>E47*F47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="n"/>
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="24" t="inlineStr">
         <is>
           <t>ARA TOPLAM (KDV hariç)</t>
         </is>
       </c>
-      <c r="D46" s="7" t="n"/>
-      <c r="E46" s="7" t="n"/>
-      <c r="F46" s="7" t="n"/>
-      <c r="G46" s="9">
-        <f>SUM(G6:G45)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n"/>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="25" t="inlineStr">
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="9">
+        <f>SUM(G6:G47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n"/>
+      <c r="B49" s="4" t="n"/>
+      <c r="C49" s="25" t="inlineStr">
         <is>
           <t>KDV</t>
         </is>
       </c>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="5">
-        <f>G46*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="11" t="n"/>
-      <c r="B48" s="11" t="n"/>
-      <c r="C48" s="26" t="inlineStr">
+      <c r="D49" s="4" t="n"/>
+      <c r="E49" s="4" t="n"/>
+      <c r="F49" s="4" t="n"/>
+      <c r="G49" s="5">
+        <f>G48*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="n"/>
+      <c r="B50" s="11" t="n"/>
+      <c r="C50" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D48" s="11" t="n"/>
-      <c r="E48" s="11" t="n"/>
-      <c r="F48" s="11" t="n"/>
-      <c r="G48" s="13">
-        <f>G46+G47</f>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="11" t="n"/>
+      <c r="F50" s="11" t="n"/>
+      <c r="G50" s="13">
+        <f>G48+G49</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: metraj yuvarlaması yarım değerde yukarı
31,4285 -> 31,429 ve 7,2875 -> 7,288. Uygun harcama 290.859 Avro;
kademe, puan ve pay değişmedi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -2401,7 +2401,7 @@
         </is>
       </c>
       <c r="E7" s="22" t="n">
-        <v>31.428</v>
+        <v>31.429</v>
       </c>
       <c r="F7" s="23">
         <f>IFERROR(VLOOKUP($B7,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2556,7 +2556,7 @@
         </is>
       </c>
       <c r="E12" s="22" t="n">
-        <v>7.287</v>
+        <v>7.288</v>
       </c>
       <c r="F12" s="23">
         <f>IFERROR(VLOOKUP($B12,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3837,7 +3837,7 @@
         </is>
       </c>
       <c r="E7" s="22" t="n">
-        <v>31.428</v>
+        <v>31.429</v>
       </c>
       <c r="F7" s="23">
         <f>IFERROR(VLOOKUP($B7,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3992,7 +3992,7 @@
         </is>
       </c>
       <c r="E12" s="22" t="n">
-        <v>7.287</v>
+        <v>7.288</v>
       </c>
       <c r="F12" s="23">
         <f>IFERROR(VLOOKUP($B12,'Fiyatlar'!$A:$I,9,FALSE),0)</f>

</xml_diff>

<commit_message>
Yayın: kümes başına 200 m kablo tavası (ÇŞB 35.190.1100)
Malzeme ve montaj ayrı poz satırı. Uygun harcama 295.391 Avro, eşiğe
kalan pay 4.609 Avro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>'01 Kümes A Blok'!$G$48</f>
+        <f>'01 Kümes A Blok'!$G$50</f>
         <v/>
       </c>
       <c r="D4" s="6">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>'02 Kümes B Blok'!$G$48</f>
+        <f>'02 Kümes B Blok'!$G$50</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2068,25 +2068,25 @@
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>35.190.1100</t>
         </is>
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>393.69</v>
+        <v>237.4</v>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F39" s="20">
@@ -2102,18 +2102,18 @@
         <v/>
       </c>
       <c r="I39" s="13" t="n">
-        <v>330.7</v>
+        <v>199.42</v>
       </c>
     </row>
     <row r="40" ht="14" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>35.190.1100 (montaj)</t>
         </is>
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
+          <t>Kablo tava sisteminin montajı — askı ve konsollarla tespiti</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2122,11 +2122,11 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>271.25</v>
+        <v>46.09</v>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 35.190.1100 pozunun 01.06.2026 tarihli MONTAJ fiyatı 46,09 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 189,92 x 1,25 + montaj 46,09 = 283,49 TL</t>
         </is>
       </c>
       <c r="F40" s="20">
@@ -2142,27 +2142,27 @@
         <v/>
       </c>
       <c r="I40" s="13" t="n">
-        <v>227.85</v>
+        <v>38.72</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>43.527.1001</t>
         </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
+          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>1035.88</v>
+        <v>393.69</v>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
@@ -2182,27 +2182,27 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
-        <v>870.14</v>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
+        <v>330.7</v>
+      </c>
+    </row>
+    <row r="42" ht="14" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0175</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>3199.68</v>
+        <v>271.25</v>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
@@ -2222,18 +2222,18 @@
         <v/>
       </c>
       <c r="I42" s="13" t="n">
-        <v>2687.73</v>
+        <v>227.85</v>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0177</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2242,7 +2242,7 @@
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>835.1</v>
+        <v>1035.88</v>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
@@ -2262,6 +2262,86 @@
         <v/>
       </c>
       <c r="I43" s="13" t="n">
+        <v>870.14</v>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0175</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="inlineStr">
+        <is>
+          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>3199.68</v>
+      </c>
+      <c r="E44" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F44" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G44" s="5">
+        <f>D44*(1-F44)</f>
+        <v/>
+      </c>
+      <c r="H44" s="5">
+        <f>D44*$D$3</f>
+        <v/>
+      </c>
+      <c r="I44" s="13" t="n">
+        <v>2687.73</v>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0177</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="inlineStr">
+        <is>
+          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>835.1</v>
+      </c>
+      <c r="E45" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F45" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G45" s="5">
+        <f>D45*(1-F45)</f>
+        <v/>
+      </c>
+      <c r="H45" s="5">
+        <f>D45*$D$3</f>
+        <v/>
+      </c>
+      <c r="I45" s="13" t="n">
         <v>701.48</v>
       </c>
     </row>
@@ -2280,7 +2360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3652,51 +3732,113 @@
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="7" t="n"/>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="24" t="inlineStr">
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100</t>
+        </is>
+      </c>
+      <c r="C48" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F48" s="23">
+        <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G48" s="5">
+        <f>E48*F48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="14" customHeight="1">
+      <c r="A49" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100 (montaj)</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sisteminin montajı — askı ve konsollarla tespiti</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F49" s="23">
+        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="5">
+        <f>E49*F49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="n"/>
+      <c r="B50" s="7" t="n"/>
+      <c r="C50" s="24" t="inlineStr">
         <is>
           <t>ARA TOPLAM (KDV hariç)</t>
         </is>
       </c>
-      <c r="D48" s="7" t="n"/>
-      <c r="E48" s="7" t="n"/>
-      <c r="F48" s="7" t="n"/>
-      <c r="G48" s="9">
-        <f>SUM(G6:G47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="25" t="inlineStr">
+      <c r="D50" s="7" t="n"/>
+      <c r="E50" s="7" t="n"/>
+      <c r="F50" s="7" t="n"/>
+      <c r="G50" s="9">
+        <f>SUM(G6:G49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n"/>
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="25" t="inlineStr">
         <is>
           <t>KDV</t>
         </is>
       </c>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="5">
-        <f>G48*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="11" t="n"/>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="26" t="inlineStr">
+      <c r="D51" s="4" t="n"/>
+      <c r="E51" s="4" t="n"/>
+      <c r="F51" s="4" t="n"/>
+      <c r="G51" s="5">
+        <f>G50*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="n"/>
+      <c r="B52" s="11" t="n"/>
+      <c r="C52" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="13">
-        <f>G48+G49</f>
+      <c r="D52" s="11" t="n"/>
+      <c r="E52" s="11" t="n"/>
+      <c r="F52" s="11" t="n"/>
+      <c r="G52" s="13">
+        <f>G50+G51</f>
         <v/>
       </c>
     </row>
@@ -3716,7 +3858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5088,51 +5230,113 @@
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="7" t="n"/>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="24" t="inlineStr">
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100</t>
+        </is>
+      </c>
+      <c r="C48" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F48" s="23">
+        <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G48" s="5">
+        <f>E48*F48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="14" customHeight="1">
+      <c r="A49" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100 (montaj)</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sisteminin montajı — askı ve konsollarla tespiti</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F49" s="23">
+        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="5">
+        <f>E49*F49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="n"/>
+      <c r="B50" s="7" t="n"/>
+      <c r="C50" s="24" t="inlineStr">
         <is>
           <t>ARA TOPLAM (KDV hariç)</t>
         </is>
       </c>
-      <c r="D48" s="7" t="n"/>
-      <c r="E48" s="7" t="n"/>
-      <c r="F48" s="7" t="n"/>
-      <c r="G48" s="9">
-        <f>SUM(G6:G47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="25" t="inlineStr">
+      <c r="D50" s="7" t="n"/>
+      <c r="E50" s="7" t="n"/>
+      <c r="F50" s="7" t="n"/>
+      <c r="G50" s="9">
+        <f>SUM(G6:G49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n"/>
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="25" t="inlineStr">
         <is>
           <t>KDV</t>
         </is>
       </c>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="5">
-        <f>G48*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="11" t="n"/>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="26" t="inlineStr">
+      <c r="D51" s="4" t="n"/>
+      <c r="E51" s="4" t="n"/>
+      <c r="F51" s="4" t="n"/>
+      <c r="G51" s="5">
+        <f>G50*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="11" t="n"/>
+      <c r="B52" s="11" t="n"/>
+      <c r="C52" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="13">
-        <f>G48+G49</f>
+      <c r="D52" s="11" t="n"/>
+      <c r="E52" s="11" t="n"/>
+      <c r="F52" s="11" t="n"/>
+      <c r="G52" s="13">
+        <f>G50+G51</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: kablo tavası kapak sacı (ÇŞB 35.190.1101)
Malzeme 193,30 + montaj 25,36 = 218,66 TL/kg, blok başına 361,200 kg.
Uygun harcama 297.906 Avro; eşiğe kalan pay 2.094 Avro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>'01 Kümes A Blok'!$G$50</f>
+        <f>'01 Kümes A Blok'!$G$52</f>
         <v/>
       </c>
       <c r="D4" s="6">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>'02 Kümes B Blok'!$G$50</f>
+        <f>'02 Kümes B Blok'!$G$52</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2105,7 +2105,7 @@
         <v>199.42</v>
       </c>
     </row>
-    <row r="40" ht="14" customHeight="1">
+    <row r="40" ht="33" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
           <t>35.190.1100 (montaj)</t>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sisteminin montajı — askı ve konsollarla tespiti</t>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2148,25 +2148,25 @@
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>35.190.1101</t>
         </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>393.69</v>
+        <v>193.3</v>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F41" s="20">
@@ -2182,18 +2182,18 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
-        <v>330.7</v>
-      </c>
-    </row>
-    <row r="42" ht="14" customHeight="1">
+        <v>162.37</v>
+      </c>
+    </row>
+    <row r="42" ht="33" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>35.190.1101 (montaj)</t>
         </is>
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2202,11 +2202,11 @@
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>271.25</v>
+        <v>25.36</v>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 35.190.1101 pozunun 01.06.2026 tarihli MONTAJ fiyatı 25,36 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 154,64 x 1,25 + montaj 25,36 = 218,66 TL</t>
         </is>
       </c>
       <c r="F42" s="20">
@@ -2222,27 +2222,27 @@
         <v/>
       </c>
       <c r="I42" s="13" t="n">
-        <v>227.85</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>43.527.1001</t>
         </is>
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
+          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>1035.88</v>
+        <v>393.69</v>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
@@ -2262,27 +2262,27 @@
         <v/>
       </c>
       <c r="I43" s="13" t="n">
-        <v>870.14</v>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1">
+        <v>330.7</v>
+      </c>
+    </row>
+    <row r="44" ht="14" customHeight="1">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0175</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="B44" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>3199.68</v>
+        <v>271.25</v>
       </c>
       <c r="E44" s="19" t="inlineStr">
         <is>
@@ -2302,18 +2302,18 @@
         <v/>
       </c>
       <c r="I44" s="13" t="n">
-        <v>2687.73</v>
+        <v>227.85</v>
       </c>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0177</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>835.1</v>
+        <v>1035.88</v>
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
@@ -2342,6 +2342,86 @@
         <v/>
       </c>
       <c r="I45" s="13" t="n">
+        <v>870.14</v>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0175</t>
+        </is>
+      </c>
+      <c r="B46" s="18" t="inlineStr">
+        <is>
+          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>3199.68</v>
+      </c>
+      <c r="E46" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F46" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G46" s="5">
+        <f>D46*(1-F46)</f>
+        <v/>
+      </c>
+      <c r="H46" s="5">
+        <f>D46*$D$3</f>
+        <v/>
+      </c>
+      <c r="I46" s="13" t="n">
+        <v>2687.73</v>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0177</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="n">
+        <v>835.1</v>
+      </c>
+      <c r="E47" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F47" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G47" s="5">
+        <f>D47*(1-F47)</f>
+        <v/>
+      </c>
+      <c r="H47" s="5">
+        <f>D47*$D$3</f>
+        <v/>
+      </c>
+      <c r="I47" s="13" t="n">
         <v>701.48</v>
       </c>
     </row>
@@ -2360,7 +2440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2457,7 +2537,7 @@
         <v/>
       </c>
       <c r="G6" s="5">
-        <f>E6*F6</f>
+        <f>ROUND(E6*F6,2)</f>
         <v/>
       </c>
     </row>
@@ -2488,7 +2568,7 @@
         <v/>
       </c>
       <c r="G7" s="5">
-        <f>E7*F7</f>
+        <f>ROUND(E7*F7,2)</f>
         <v/>
       </c>
     </row>
@@ -2519,7 +2599,7 @@
         <v/>
       </c>
       <c r="G8" s="5">
-        <f>E8*F8</f>
+        <f>ROUND(E8*F8,2)</f>
         <v/>
       </c>
     </row>
@@ -2550,7 +2630,7 @@
         <v/>
       </c>
       <c r="G9" s="5">
-        <f>E9*F9</f>
+        <f>ROUND(E9*F9,2)</f>
         <v/>
       </c>
     </row>
@@ -2581,7 +2661,7 @@
         <v/>
       </c>
       <c r="G10" s="5">
-        <f>E10*F10</f>
+        <f>ROUND(E10*F10,2)</f>
         <v/>
       </c>
     </row>
@@ -2612,7 +2692,7 @@
         <v/>
       </c>
       <c r="G11" s="5">
-        <f>E11*F11</f>
+        <f>ROUND(E11*F11,2)</f>
         <v/>
       </c>
     </row>
@@ -2643,7 +2723,7 @@
         <v/>
       </c>
       <c r="G12" s="5">
-        <f>E12*F12</f>
+        <f>ROUND(E12*F12,2)</f>
         <v/>
       </c>
     </row>
@@ -2674,7 +2754,7 @@
         <v/>
       </c>
       <c r="G13" s="5">
-        <f>E13*F13</f>
+        <f>ROUND(E13*F13,2)</f>
         <v/>
       </c>
     </row>
@@ -2705,7 +2785,7 @@
         <v/>
       </c>
       <c r="G14" s="5">
-        <f>E14*F14</f>
+        <f>ROUND(E14*F14,2)</f>
         <v/>
       </c>
     </row>
@@ -2736,7 +2816,7 @@
         <v/>
       </c>
       <c r="G15" s="5">
-        <f>E15*F15</f>
+        <f>ROUND(E15*F15,2)</f>
         <v/>
       </c>
     </row>
@@ -2767,7 +2847,7 @@
         <v/>
       </c>
       <c r="G16" s="5">
-        <f>E16*F16</f>
+        <f>ROUND(E16*F16,2)</f>
         <v/>
       </c>
     </row>
@@ -2798,7 +2878,7 @@
         <v/>
       </c>
       <c r="G17" s="5">
-        <f>E17*F17</f>
+        <f>ROUND(E17*F17,2)</f>
         <v/>
       </c>
     </row>
@@ -2829,7 +2909,7 @@
         <v/>
       </c>
       <c r="G18" s="5">
-        <f>E18*F18</f>
+        <f>ROUND(E18*F18,2)</f>
         <v/>
       </c>
     </row>
@@ -2860,7 +2940,7 @@
         <v/>
       </c>
       <c r="G19" s="5">
-        <f>E19*F19</f>
+        <f>ROUND(E19*F19,2)</f>
         <v/>
       </c>
     </row>
@@ -2891,7 +2971,7 @@
         <v/>
       </c>
       <c r="G20" s="5">
-        <f>E20*F20</f>
+        <f>ROUND(E20*F20,2)</f>
         <v/>
       </c>
     </row>
@@ -2922,7 +3002,7 @@
         <v/>
       </c>
       <c r="G21" s="5">
-        <f>E21*F21</f>
+        <f>ROUND(E21*F21,2)</f>
         <v/>
       </c>
     </row>
@@ -2953,7 +3033,7 @@
         <v/>
       </c>
       <c r="G22" s="5">
-        <f>E22*F22</f>
+        <f>ROUND(E22*F22,2)</f>
         <v/>
       </c>
     </row>
@@ -2984,7 +3064,7 @@
         <v/>
       </c>
       <c r="G23" s="5">
-        <f>E23*F23</f>
+        <f>ROUND(E23*F23,2)</f>
         <v/>
       </c>
     </row>
@@ -3015,7 +3095,7 @@
         <v/>
       </c>
       <c r="G24" s="5">
-        <f>E24*F24</f>
+        <f>ROUND(E24*F24,2)</f>
         <v/>
       </c>
     </row>
@@ -3046,7 +3126,7 @@
         <v/>
       </c>
       <c r="G25" s="5">
-        <f>E25*F25</f>
+        <f>ROUND(E25*F25,2)</f>
         <v/>
       </c>
     </row>
@@ -3077,7 +3157,7 @@
         <v/>
       </c>
       <c r="G26" s="5">
-        <f>E26*F26</f>
+        <f>ROUND(E26*F26,2)</f>
         <v/>
       </c>
     </row>
@@ -3108,7 +3188,7 @@
         <v/>
       </c>
       <c r="G27" s="5">
-        <f>E27*F27</f>
+        <f>ROUND(E27*F27,2)</f>
         <v/>
       </c>
     </row>
@@ -3139,7 +3219,7 @@
         <v/>
       </c>
       <c r="G28" s="5">
-        <f>E28*F28</f>
+        <f>ROUND(E28*F28,2)</f>
         <v/>
       </c>
     </row>
@@ -3170,7 +3250,7 @@
         <v/>
       </c>
       <c r="G29" s="5">
-        <f>E29*F29</f>
+        <f>ROUND(E29*F29,2)</f>
         <v/>
       </c>
     </row>
@@ -3201,7 +3281,7 @@
         <v/>
       </c>
       <c r="G30" s="5">
-        <f>E30*F30</f>
+        <f>ROUND(E30*F30,2)</f>
         <v/>
       </c>
     </row>
@@ -3232,7 +3312,7 @@
         <v/>
       </c>
       <c r="G31" s="5">
-        <f>E31*F31</f>
+        <f>ROUND(E31*F31,2)</f>
         <v/>
       </c>
     </row>
@@ -3263,7 +3343,7 @@
         <v/>
       </c>
       <c r="G32" s="5">
-        <f>E32*F32</f>
+        <f>ROUND(E32*F32,2)</f>
         <v/>
       </c>
     </row>
@@ -3294,7 +3374,7 @@
         <v/>
       </c>
       <c r="G33" s="5">
-        <f>E33*F33</f>
+        <f>ROUND(E33*F33,2)</f>
         <v/>
       </c>
     </row>
@@ -3325,7 +3405,7 @@
         <v/>
       </c>
       <c r="G34" s="5">
-        <f>E34*F34</f>
+        <f>ROUND(E34*F34,2)</f>
         <v/>
       </c>
     </row>
@@ -3356,7 +3436,7 @@
         <v/>
       </c>
       <c r="G35" s="5">
-        <f>E35*F35</f>
+        <f>ROUND(E35*F35,2)</f>
         <v/>
       </c>
     </row>
@@ -3387,7 +3467,7 @@
         <v/>
       </c>
       <c r="G36" s="5">
-        <f>E36*F36</f>
+        <f>ROUND(E36*F36,2)</f>
         <v/>
       </c>
     </row>
@@ -3418,7 +3498,7 @@
         <v/>
       </c>
       <c r="G37" s="5">
-        <f>E37*F37</f>
+        <f>ROUND(E37*F37,2)</f>
         <v/>
       </c>
     </row>
@@ -3449,7 +3529,7 @@
         <v/>
       </c>
       <c r="G38" s="5">
-        <f>E38*F38</f>
+        <f>ROUND(E38*F38,2)</f>
         <v/>
       </c>
     </row>
@@ -3480,7 +3560,7 @@
         <v/>
       </c>
       <c r="G39" s="5">
-        <f>E39*F39</f>
+        <f>ROUND(E39*F39,2)</f>
         <v/>
       </c>
     </row>
@@ -3511,7 +3591,7 @@
         <v/>
       </c>
       <c r="G40" s="5">
-        <f>E40*F40</f>
+        <f>ROUND(E40*F40,2)</f>
         <v/>
       </c>
     </row>
@@ -3542,7 +3622,7 @@
         <v/>
       </c>
       <c r="G41" s="5">
-        <f>E41*F41</f>
+        <f>ROUND(E41*F41,2)</f>
         <v/>
       </c>
     </row>
@@ -3573,7 +3653,7 @@
         <v/>
       </c>
       <c r="G42" s="5">
-        <f>E42*F42</f>
+        <f>ROUND(E42*F42,2)</f>
         <v/>
       </c>
     </row>
@@ -3604,7 +3684,7 @@
         <v/>
       </c>
       <c r="G43" s="5">
-        <f>E43*F43</f>
+        <f>ROUND(E43*F43,2)</f>
         <v/>
       </c>
     </row>
@@ -3635,7 +3715,7 @@
         <v/>
       </c>
       <c r="G44" s="5">
-        <f>E44*F44</f>
+        <f>ROUND(E44*F44,2)</f>
         <v/>
       </c>
     </row>
@@ -3666,7 +3746,7 @@
         <v/>
       </c>
       <c r="G45" s="5">
-        <f>E45*F45</f>
+        <f>ROUND(E45*F45,2)</f>
         <v/>
       </c>
     </row>
@@ -3697,7 +3777,7 @@
         <v/>
       </c>
       <c r="G46" s="5">
-        <f>E46*F46</f>
+        <f>ROUND(E46*F46,2)</f>
         <v/>
       </c>
     </row>
@@ -3728,7 +3808,7 @@
         <v/>
       </c>
       <c r="G47" s="5">
-        <f>E47*F47</f>
+        <f>ROUND(E47*F47,2)</f>
         <v/>
       </c>
     </row>
@@ -3759,11 +3839,11 @@
         <v/>
       </c>
       <c r="G48" s="5">
-        <f>E48*F48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="14" customHeight="1">
+        <f>ROUND(E48*F48,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
       <c r="A49" s="3" t="n">
         <v>44</v>
       </c>
@@ -3774,7 +3854,7 @@
       </c>
       <c r="C49" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sisteminin montajı — askı ve konsollarla tespiti</t>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -3790,55 +3870,117 @@
         <v/>
       </c>
       <c r="G49" s="5">
-        <f>E49*F49</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="n"/>
-      <c r="B50" s="7" t="n"/>
-      <c r="C50" s="24" t="inlineStr">
+        <f>ROUND(E49*F49,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="14" customHeight="1">
+      <c r="A50" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F50" s="23">
+        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="5">
+        <f>ROUND(E50*F50,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101 (montaj)</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F51" s="23">
+        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="5">
+        <f>ROUND(E51*F51,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="n"/>
+      <c r="B52" s="7" t="n"/>
+      <c r="C52" s="24" t="inlineStr">
         <is>
           <t>ARA TOPLAM (KDV hariç)</t>
         </is>
       </c>
-      <c r="D50" s="7" t="n"/>
-      <c r="E50" s="7" t="n"/>
-      <c r="F50" s="7" t="n"/>
-      <c r="G50" s="9">
-        <f>SUM(G6:G49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="n"/>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="25" t="inlineStr">
+      <c r="D52" s="7" t="n"/>
+      <c r="E52" s="7" t="n"/>
+      <c r="F52" s="7" t="n"/>
+      <c r="G52" s="9">
+        <f>SUM(G6:G51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n"/>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="25" t="inlineStr">
         <is>
           <t>KDV</t>
         </is>
       </c>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="5">
-        <f>G50*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="11" t="n"/>
-      <c r="B52" s="11" t="n"/>
-      <c r="C52" s="26" t="inlineStr">
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="5">
+        <f>G52*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="n"/>
+      <c r="B54" s="11" t="n"/>
+      <c r="C54" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D52" s="11" t="n"/>
-      <c r="E52" s="11" t="n"/>
-      <c r="F52" s="11" t="n"/>
-      <c r="G52" s="13">
-        <f>G50+G51</f>
+      <c r="D54" s="11" t="n"/>
+      <c r="E54" s="11" t="n"/>
+      <c r="F54" s="11" t="n"/>
+      <c r="G54" s="13">
+        <f>G52+G53</f>
         <v/>
       </c>
     </row>
@@ -3858,7 +4000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3955,7 +4097,7 @@
         <v/>
       </c>
       <c r="G6" s="5">
-        <f>E6*F6</f>
+        <f>ROUND(E6*F6,2)</f>
         <v/>
       </c>
     </row>
@@ -3986,7 +4128,7 @@
         <v/>
       </c>
       <c r="G7" s="5">
-        <f>E7*F7</f>
+        <f>ROUND(E7*F7,2)</f>
         <v/>
       </c>
     </row>
@@ -4017,7 +4159,7 @@
         <v/>
       </c>
       <c r="G8" s="5">
-        <f>E8*F8</f>
+        <f>ROUND(E8*F8,2)</f>
         <v/>
       </c>
     </row>
@@ -4048,7 +4190,7 @@
         <v/>
       </c>
       <c r="G9" s="5">
-        <f>E9*F9</f>
+        <f>ROUND(E9*F9,2)</f>
         <v/>
       </c>
     </row>
@@ -4079,7 +4221,7 @@
         <v/>
       </c>
       <c r="G10" s="5">
-        <f>E10*F10</f>
+        <f>ROUND(E10*F10,2)</f>
         <v/>
       </c>
     </row>
@@ -4110,7 +4252,7 @@
         <v/>
       </c>
       <c r="G11" s="5">
-        <f>E11*F11</f>
+        <f>ROUND(E11*F11,2)</f>
         <v/>
       </c>
     </row>
@@ -4141,7 +4283,7 @@
         <v/>
       </c>
       <c r="G12" s="5">
-        <f>E12*F12</f>
+        <f>ROUND(E12*F12,2)</f>
         <v/>
       </c>
     </row>
@@ -4172,7 +4314,7 @@
         <v/>
       </c>
       <c r="G13" s="5">
-        <f>E13*F13</f>
+        <f>ROUND(E13*F13,2)</f>
         <v/>
       </c>
     </row>
@@ -4203,7 +4345,7 @@
         <v/>
       </c>
       <c r="G14" s="5">
-        <f>E14*F14</f>
+        <f>ROUND(E14*F14,2)</f>
         <v/>
       </c>
     </row>
@@ -4234,7 +4376,7 @@
         <v/>
       </c>
       <c r="G15" s="5">
-        <f>E15*F15</f>
+        <f>ROUND(E15*F15,2)</f>
         <v/>
       </c>
     </row>
@@ -4265,7 +4407,7 @@
         <v/>
       </c>
       <c r="G16" s="5">
-        <f>E16*F16</f>
+        <f>ROUND(E16*F16,2)</f>
         <v/>
       </c>
     </row>
@@ -4296,7 +4438,7 @@
         <v/>
       </c>
       <c r="G17" s="5">
-        <f>E17*F17</f>
+        <f>ROUND(E17*F17,2)</f>
         <v/>
       </c>
     </row>
@@ -4327,7 +4469,7 @@
         <v/>
       </c>
       <c r="G18" s="5">
-        <f>E18*F18</f>
+        <f>ROUND(E18*F18,2)</f>
         <v/>
       </c>
     </row>
@@ -4358,7 +4500,7 @@
         <v/>
       </c>
       <c r="G19" s="5">
-        <f>E19*F19</f>
+        <f>ROUND(E19*F19,2)</f>
         <v/>
       </c>
     </row>
@@ -4389,7 +4531,7 @@
         <v/>
       </c>
       <c r="G20" s="5">
-        <f>E20*F20</f>
+        <f>ROUND(E20*F20,2)</f>
         <v/>
       </c>
     </row>
@@ -4420,7 +4562,7 @@
         <v/>
       </c>
       <c r="G21" s="5">
-        <f>E21*F21</f>
+        <f>ROUND(E21*F21,2)</f>
         <v/>
       </c>
     </row>
@@ -4451,7 +4593,7 @@
         <v/>
       </c>
       <c r="G22" s="5">
-        <f>E22*F22</f>
+        <f>ROUND(E22*F22,2)</f>
         <v/>
       </c>
     </row>
@@ -4482,7 +4624,7 @@
         <v/>
       </c>
       <c r="G23" s="5">
-        <f>E23*F23</f>
+        <f>ROUND(E23*F23,2)</f>
         <v/>
       </c>
     </row>
@@ -4513,7 +4655,7 @@
         <v/>
       </c>
       <c r="G24" s="5">
-        <f>E24*F24</f>
+        <f>ROUND(E24*F24,2)</f>
         <v/>
       </c>
     </row>
@@ -4544,7 +4686,7 @@
         <v/>
       </c>
       <c r="G25" s="5">
-        <f>E25*F25</f>
+        <f>ROUND(E25*F25,2)</f>
         <v/>
       </c>
     </row>
@@ -4575,7 +4717,7 @@
         <v/>
       </c>
       <c r="G26" s="5">
-        <f>E26*F26</f>
+        <f>ROUND(E26*F26,2)</f>
         <v/>
       </c>
     </row>
@@ -4606,7 +4748,7 @@
         <v/>
       </c>
       <c r="G27" s="5">
-        <f>E27*F27</f>
+        <f>ROUND(E27*F27,2)</f>
         <v/>
       </c>
     </row>
@@ -4637,7 +4779,7 @@
         <v/>
       </c>
       <c r="G28" s="5">
-        <f>E28*F28</f>
+        <f>ROUND(E28*F28,2)</f>
         <v/>
       </c>
     </row>
@@ -4668,7 +4810,7 @@
         <v/>
       </c>
       <c r="G29" s="5">
-        <f>E29*F29</f>
+        <f>ROUND(E29*F29,2)</f>
         <v/>
       </c>
     </row>
@@ -4699,7 +4841,7 @@
         <v/>
       </c>
       <c r="G30" s="5">
-        <f>E30*F30</f>
+        <f>ROUND(E30*F30,2)</f>
         <v/>
       </c>
     </row>
@@ -4730,7 +4872,7 @@
         <v/>
       </c>
       <c r="G31" s="5">
-        <f>E31*F31</f>
+        <f>ROUND(E31*F31,2)</f>
         <v/>
       </c>
     </row>
@@ -4761,7 +4903,7 @@
         <v/>
       </c>
       <c r="G32" s="5">
-        <f>E32*F32</f>
+        <f>ROUND(E32*F32,2)</f>
         <v/>
       </c>
     </row>
@@ -4792,7 +4934,7 @@
         <v/>
       </c>
       <c r="G33" s="5">
-        <f>E33*F33</f>
+        <f>ROUND(E33*F33,2)</f>
         <v/>
       </c>
     </row>
@@ -4823,7 +4965,7 @@
         <v/>
       </c>
       <c r="G34" s="5">
-        <f>E34*F34</f>
+        <f>ROUND(E34*F34,2)</f>
         <v/>
       </c>
     </row>
@@ -4854,7 +4996,7 @@
         <v/>
       </c>
       <c r="G35" s="5">
-        <f>E35*F35</f>
+        <f>ROUND(E35*F35,2)</f>
         <v/>
       </c>
     </row>
@@ -4885,7 +5027,7 @@
         <v/>
       </c>
       <c r="G36" s="5">
-        <f>E36*F36</f>
+        <f>ROUND(E36*F36,2)</f>
         <v/>
       </c>
     </row>
@@ -4916,7 +5058,7 @@
         <v/>
       </c>
       <c r="G37" s="5">
-        <f>E37*F37</f>
+        <f>ROUND(E37*F37,2)</f>
         <v/>
       </c>
     </row>
@@ -4947,7 +5089,7 @@
         <v/>
       </c>
       <c r="G38" s="5">
-        <f>E38*F38</f>
+        <f>ROUND(E38*F38,2)</f>
         <v/>
       </c>
     </row>
@@ -4978,7 +5120,7 @@
         <v/>
       </c>
       <c r="G39" s="5">
-        <f>E39*F39</f>
+        <f>ROUND(E39*F39,2)</f>
         <v/>
       </c>
     </row>
@@ -5009,7 +5151,7 @@
         <v/>
       </c>
       <c r="G40" s="5">
-        <f>E40*F40</f>
+        <f>ROUND(E40*F40,2)</f>
         <v/>
       </c>
     </row>
@@ -5040,7 +5182,7 @@
         <v/>
       </c>
       <c r="G41" s="5">
-        <f>E41*F41</f>
+        <f>ROUND(E41*F41,2)</f>
         <v/>
       </c>
     </row>
@@ -5071,7 +5213,7 @@
         <v/>
       </c>
       <c r="G42" s="5">
-        <f>E42*F42</f>
+        <f>ROUND(E42*F42,2)</f>
         <v/>
       </c>
     </row>
@@ -5102,7 +5244,7 @@
         <v/>
       </c>
       <c r="G43" s="5">
-        <f>E43*F43</f>
+        <f>ROUND(E43*F43,2)</f>
         <v/>
       </c>
     </row>
@@ -5133,7 +5275,7 @@
         <v/>
       </c>
       <c r="G44" s="5">
-        <f>E44*F44</f>
+        <f>ROUND(E44*F44,2)</f>
         <v/>
       </c>
     </row>
@@ -5164,7 +5306,7 @@
         <v/>
       </c>
       <c r="G45" s="5">
-        <f>E45*F45</f>
+        <f>ROUND(E45*F45,2)</f>
         <v/>
       </c>
     </row>
@@ -5195,7 +5337,7 @@
         <v/>
       </c>
       <c r="G46" s="5">
-        <f>E46*F46</f>
+        <f>ROUND(E46*F46,2)</f>
         <v/>
       </c>
     </row>
@@ -5226,7 +5368,7 @@
         <v/>
       </c>
       <c r="G47" s="5">
-        <f>E47*F47</f>
+        <f>ROUND(E47*F47,2)</f>
         <v/>
       </c>
     </row>
@@ -5257,11 +5399,11 @@
         <v/>
       </c>
       <c r="G48" s="5">
-        <f>E48*F48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="14" customHeight="1">
+        <f>ROUND(E48*F48,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
       <c r="A49" s="3" t="n">
         <v>44</v>
       </c>
@@ -5272,7 +5414,7 @@
       </c>
       <c r="C49" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sisteminin montajı — askı ve konsollarla tespiti</t>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -5288,55 +5430,117 @@
         <v/>
       </c>
       <c r="G49" s="5">
-        <f>E49*F49</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="n"/>
-      <c r="B50" s="7" t="n"/>
-      <c r="C50" s="24" t="inlineStr">
+        <f>ROUND(E49*F49,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="14" customHeight="1">
+      <c r="A50" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F50" s="23">
+        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="5">
+        <f>ROUND(E50*F50,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101 (montaj)</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F51" s="23">
+        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="5">
+        <f>ROUND(E51*F51,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="n"/>
+      <c r="B52" s="7" t="n"/>
+      <c r="C52" s="24" t="inlineStr">
         <is>
           <t>ARA TOPLAM (KDV hariç)</t>
         </is>
       </c>
-      <c r="D50" s="7" t="n"/>
-      <c r="E50" s="7" t="n"/>
-      <c r="F50" s="7" t="n"/>
-      <c r="G50" s="9">
-        <f>SUM(G6:G49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="n"/>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="25" t="inlineStr">
+      <c r="D52" s="7" t="n"/>
+      <c r="E52" s="7" t="n"/>
+      <c r="F52" s="7" t="n"/>
+      <c r="G52" s="9">
+        <f>SUM(G6:G51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n"/>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="25" t="inlineStr">
         <is>
           <t>KDV</t>
         </is>
       </c>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="n"/>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="5">
-        <f>G50*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="11" t="n"/>
-      <c r="B52" s="11" t="n"/>
-      <c r="C52" s="26" t="inlineStr">
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="5">
+        <f>G52*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="11" t="n"/>
+      <c r="B54" s="11" t="n"/>
+      <c r="C54" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D52" s="11" t="n"/>
-      <c r="E52" s="11" t="n"/>
-      <c r="F52" s="11" t="n"/>
-      <c r="G52" s="13">
-        <f>G50+G51</f>
+      <c r="D54" s="11" t="n"/>
+      <c r="E54" s="11" t="n"/>
+      <c r="F54" s="11" t="n"/>
+      <c r="G54" s="13">
+        <f>G52+G53</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: kablo tava sistemi hibe dışına alındı
Uygun harcama 290.859 Avro, eşiğe kalan pay 9.141 Avro (%3,05).
Tava projede duruyor, proforma 36 ile beyan ediliyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>'01 Kümes A Blok'!$G$52</f>
+        <f>'01 Kümes A Blok'!$G$48</f>
         <v/>
       </c>
       <c r="D4" s="6">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>'02 Kümes B Blok'!$G$52</f>
+        <f>'02 Kümes B Blok'!$G$48</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2068,25 +2068,25 @@
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>35.190.1100</t>
+          <t>43.527.1001</t>
         </is>
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
+          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>237.4</v>
+        <v>393.69</v>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F39" s="20">
@@ -2102,18 +2102,18 @@
         <v/>
       </c>
       <c r="I39" s="13" t="n">
-        <v>199.42</v>
-      </c>
-    </row>
-    <row r="40" ht="33" customHeight="1">
+        <v>330.7</v>
+      </c>
+    </row>
+    <row r="40" ht="14" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>35.190.1100 (montaj)</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
+          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2122,11 +2122,11 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>46.09</v>
+        <v>271.25</v>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 35.190.1100 pozunun 01.06.2026 tarihli MONTAJ fiyatı 46,09 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 189,92 x 1,25 + montaj 46,09 = 283,49 TL</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F40" s="20">
@@ -2142,31 +2142,31 @@
         <v/>
       </c>
       <c r="I40" s="13" t="n">
-        <v>38.72</v>
+        <v>227.85</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>35.190.1101</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
+          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>193.3</v>
+        <v>1035.88</v>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F41" s="20">
@@ -2182,31 +2182,31 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
-        <v>162.37</v>
-      </c>
-    </row>
-    <row r="42" ht="33" customHeight="1">
+        <v>870.14</v>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>35.190.1101 (montaj)</t>
+          <t>TKDK-0175</t>
         </is>
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
+          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>25.36</v>
+        <v>3199.68</v>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 35.190.1101 pozunun 01.06.2026 tarihli MONTAJ fiyatı 25,36 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 154,64 x 1,25 + montaj 25,36 = 218,66 TL</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F42" s="20">
@@ -2222,27 +2222,27 @@
         <v/>
       </c>
       <c r="I42" s="13" t="n">
-        <v>21.3</v>
+        <v>2687.73</v>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>TKDK-0177</t>
         </is>
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>393.69</v>
+        <v>835.1</v>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
@@ -2262,166 +2262,6 @@
         <v/>
       </c>
       <c r="I43" s="13" t="n">
-        <v>330.7</v>
-      </c>
-    </row>
-    <row r="44" ht="14" customHeight="1">
-      <c r="A44" s="17" t="inlineStr">
-        <is>
-          <t>TKDK-0115</t>
-        </is>
-      </c>
-      <c r="B44" s="18" t="inlineStr">
-        <is>
-          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="n">
-        <v>271.25</v>
-      </c>
-      <c r="E44" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F44" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G44" s="5">
-        <f>D44*(1-F44)</f>
-        <v/>
-      </c>
-      <c r="H44" s="5">
-        <f>D44*$D$3</f>
-        <v/>
-      </c>
-      <c r="I44" s="13" t="n">
-        <v>227.85</v>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1">
-      <c r="A45" s="17" t="inlineStr">
-        <is>
-          <t>TKDK-0151</t>
-        </is>
-      </c>
-      <c r="B45" s="18" t="inlineStr">
-        <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="n">
-        <v>1035.88</v>
-      </c>
-      <c r="E45" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F45" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G45" s="5">
-        <f>D45*(1-F45)</f>
-        <v/>
-      </c>
-      <c r="H45" s="5">
-        <f>D45*$D$3</f>
-        <v/>
-      </c>
-      <c r="I45" s="13" t="n">
-        <v>870.14</v>
-      </c>
-    </row>
-    <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="17" t="inlineStr">
-        <is>
-          <t>TKDK-0175</t>
-        </is>
-      </c>
-      <c r="B46" s="18" t="inlineStr">
-        <is>
-          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="n">
-        <v>3199.68</v>
-      </c>
-      <c r="E46" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F46" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G46" s="5">
-        <f>D46*(1-F46)</f>
-        <v/>
-      </c>
-      <c r="H46" s="5">
-        <f>D46*$D$3</f>
-        <v/>
-      </c>
-      <c r="I46" s="13" t="n">
-        <v>2687.73</v>
-      </c>
-    </row>
-    <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="17" t="inlineStr">
-        <is>
-          <t>TKDK-0177</t>
-        </is>
-      </c>
-      <c r="B47" s="18" t="inlineStr">
-        <is>
-          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="n">
-        <v>835.1</v>
-      </c>
-      <c r="E47" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F47" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G47" s="5">
-        <f>D47*(1-F47)</f>
-        <v/>
-      </c>
-      <c r="H47" s="5">
-        <f>D47*$D$3</f>
-        <v/>
-      </c>
-      <c r="I47" s="13" t="n">
         <v>701.48</v>
       </c>
     </row>
@@ -2440,7 +2280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3812,175 +3652,51 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="3" t="n">
-        <v>43</v>
-      </c>
-      <c r="B48" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1100</t>
-        </is>
-      </c>
-      <c r="C48" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E48" s="22" t="n">
-        <v>502</v>
-      </c>
-      <c r="F48" s="23">
-        <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G48" s="5">
-        <f>ROUND(E48*F48,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="3" t="n">
-        <v>44</v>
-      </c>
-      <c r="B49" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1100 (montaj)</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E49" s="22" t="n">
-        <v>502</v>
-      </c>
-      <c r="F49" s="23">
-        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
+    <row r="48">
+      <c r="A48" s="7" t="n"/>
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="24" t="inlineStr">
+        <is>
+          <t>ARA TOPLAM (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="9">
+        <f>SUM(G6:G47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n"/>
+      <c r="B49" s="4" t="n"/>
+      <c r="C49" s="25" t="inlineStr">
+        <is>
+          <t>KDV</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="n"/>
+      <c r="E49" s="4" t="n"/>
+      <c r="F49" s="4" t="n"/>
       <c r="G49" s="5">
-        <f>ROUND(E49*F49,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="14" customHeight="1">
-      <c r="A50" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="B50" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101</t>
-        </is>
-      </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E50" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F50" s="23">
-        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G50" s="5">
-        <f>ROUND(E50*F50,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="B51" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101 (montaj)</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E51" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F51" s="23">
-        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G51" s="5">
-        <f>ROUND(E51*F51,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="7" t="n"/>
-      <c r="B52" s="7" t="n"/>
-      <c r="C52" s="24" t="inlineStr">
-        <is>
-          <t>ARA TOPLAM (KDV hariç)</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="n"/>
-      <c r="E52" s="7" t="n"/>
-      <c r="F52" s="7" t="n"/>
-      <c r="G52" s="9">
-        <f>SUM(G6:G51)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="n"/>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="25" t="inlineStr">
-        <is>
-          <t>KDV</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="4" t="n"/>
-      <c r="G53" s="5">
-        <f>G52*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="11" t="n"/>
-      <c r="B54" s="11" t="n"/>
-      <c r="C54" s="26" t="inlineStr">
+        <f>G48*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="n"/>
+      <c r="B50" s="11" t="n"/>
+      <c r="C50" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D54" s="11" t="n"/>
-      <c r="E54" s="11" t="n"/>
-      <c r="F54" s="11" t="n"/>
-      <c r="G54" s="13">
-        <f>G52+G53</f>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="11" t="n"/>
+      <c r="F50" s="11" t="n"/>
+      <c r="G50" s="13">
+        <f>G48+G49</f>
         <v/>
       </c>
     </row>
@@ -4000,7 +3716,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5372,175 +5088,51 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="3" t="n">
-        <v>43</v>
-      </c>
-      <c r="B48" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1100</t>
-        </is>
-      </c>
-      <c r="C48" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E48" s="22" t="n">
-        <v>502</v>
-      </c>
-      <c r="F48" s="23">
-        <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G48" s="5">
-        <f>ROUND(E48*F48,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="3" t="n">
-        <v>44</v>
-      </c>
-      <c r="B49" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1100 (montaj)</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E49" s="22" t="n">
-        <v>502</v>
-      </c>
-      <c r="F49" s="23">
-        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
+    <row r="48">
+      <c r="A48" s="7" t="n"/>
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="24" t="inlineStr">
+        <is>
+          <t>ARA TOPLAM (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="9">
+        <f>SUM(G6:G47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n"/>
+      <c r="B49" s="4" t="n"/>
+      <c r="C49" s="25" t="inlineStr">
+        <is>
+          <t>KDV</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="n"/>
+      <c r="E49" s="4" t="n"/>
+      <c r="F49" s="4" t="n"/>
       <c r="G49" s="5">
-        <f>ROUND(E49*F49,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="14" customHeight="1">
-      <c r="A50" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="B50" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101</t>
-        </is>
-      </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E50" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F50" s="23">
-        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G50" s="5">
-        <f>ROUND(E50*F50,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="B51" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101 (montaj)</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E51" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F51" s="23">
-        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G51" s="5">
-        <f>ROUND(E51*F51,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="7" t="n"/>
-      <c r="B52" s="7" t="n"/>
-      <c r="C52" s="24" t="inlineStr">
-        <is>
-          <t>ARA TOPLAM (KDV hariç)</t>
-        </is>
-      </c>
-      <c r="D52" s="7" t="n"/>
-      <c r="E52" s="7" t="n"/>
-      <c r="F52" s="7" t="n"/>
-      <c r="G52" s="9">
-        <f>SUM(G6:G51)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="n"/>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="25" t="inlineStr">
-        <is>
-          <t>KDV</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="n"/>
-      <c r="E53" s="4" t="n"/>
-      <c r="F53" s="4" t="n"/>
-      <c r="G53" s="5">
-        <f>G52*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="11" t="n"/>
-      <c r="B54" s="11" t="n"/>
-      <c r="C54" s="26" t="inlineStr">
+        <f>G48*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="n"/>
+      <c r="B50" s="11" t="n"/>
+      <c r="C50" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D54" s="11" t="n"/>
-      <c r="E54" s="11" t="n"/>
-      <c r="F54" s="11" t="n"/>
-      <c r="G54" s="13">
-        <f>G52+G53</f>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="11" t="n"/>
+      <c r="F50" s="11" t="n"/>
+      <c r="G50" s="13">
+        <f>G48+G49</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: uygun harcama 298.994 Avro — kablo kanalı eklendi
Tava sistemi kapsama geri alındı, sıva üstü PVC kablo kanalı
(30.190.1304, 123 m/blok) eklendi. Eşiğe kalan pay 1.006 Avro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>'01 Kümes A Blok'!$G$48</f>
+        <f>'01 Kümes A Blok'!$G$53</f>
         <v/>
       </c>
       <c r="D4" s="6">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>'02 Kümes B Blok'!$G$48</f>
+        <f>'02 Kümes B Blok'!$G$53</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1865,24 +1865,24 @@
         <v>1996.08</v>
       </c>
     </row>
-    <row r="34" ht="22" customHeight="1">
+    <row r="34" ht="14" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>30.740.1106</t>
+          <t>30.190.1304</t>
         </is>
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>556368.2</v>
+        <v>277.71</v>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
@@ -1902,18 +1902,18 @@
         <v/>
       </c>
       <c r="I34" s="13" t="n">
-        <v>467349.29</v>
-      </c>
-    </row>
-    <row r="35" ht="14" customHeight="1">
+        <v>233.28</v>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>30.740.5406</t>
+          <t>30.740.1106</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -1922,7 +1922,7 @@
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>94825.64999999999</v>
+        <v>556368.2</v>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
@@ -1942,18 +1942,18 @@
         <v/>
       </c>
       <c r="I35" s="13" t="n">
-        <v>79653.55</v>
+        <v>467349.29</v>
       </c>
     </row>
     <row r="36" ht="14" customHeight="1">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>30.750.1502</t>
+          <t>30.740.5406</t>
         </is>
       </c>
       <c r="B36" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>18566.2</v>
+        <v>94825.64999999999</v>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
@@ -1982,27 +1982,27 @@
         <v/>
       </c>
       <c r="I36" s="13" t="n">
-        <v>15595.61</v>
-      </c>
-    </row>
-    <row r="37" ht="22" customHeight="1">
+        <v>79653.55</v>
+      </c>
+    </row>
+    <row r="37" ht="14" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>30.750.2001</t>
+          <t>30.750.1502</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>508</v>
+        <v>18566.2</v>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
@@ -2022,18 +2022,18 @@
         <v/>
       </c>
       <c r="I37" s="13" t="n">
-        <v>426.72</v>
+        <v>15595.61</v>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>30.750.3002</t>
+          <t>30.750.2001</t>
         </is>
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>138.05</v>
+        <v>508</v>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
@@ -2062,18 +2062,18 @@
         <v/>
       </c>
       <c r="I38" s="13" t="n">
-        <v>115.96</v>
+        <v>426.72</v>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>30.750.3002</t>
         </is>
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2082,11 +2082,11 @@
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>393.69</v>
+        <v>138.05</v>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F39" s="20">
@@ -2102,18 +2102,18 @@
         <v/>
       </c>
       <c r="I39" s="13" t="n">
-        <v>330.7</v>
-      </c>
-    </row>
-    <row r="40" ht="14" customHeight="1">
+        <v>115.96</v>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>35.190.1100</t>
         </is>
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
+          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2122,11 +2122,11 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>271.25</v>
+        <v>237.4</v>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F40" s="20">
@@ -2142,31 +2142,31 @@
         <v/>
       </c>
       <c r="I40" s="13" t="n">
-        <v>227.85</v>
-      </c>
-    </row>
-    <row r="41" ht="22" customHeight="1">
+        <v>199.42</v>
+      </c>
+    </row>
+    <row r="41" ht="33" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>35.190.1100 (montaj)</t>
         </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>1035.88</v>
+        <v>46.09</v>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 35.190.1100 pozunun 01.06.2026 tarihli MONTAJ fiyatı 46,09 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 189,92 x 1,25 + montaj 46,09 = 283,49 TL</t>
         </is>
       </c>
       <c r="F41" s="20">
@@ -2182,31 +2182,31 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
-        <v>870.14</v>
+        <v>38.72</v>
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0175</t>
+          <t>35.190.1101</t>
         </is>
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>3199.68</v>
+        <v>193.3</v>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F42" s="20">
@@ -2222,31 +2222,31 @@
         <v/>
       </c>
       <c r="I42" s="13" t="n">
-        <v>2687.73</v>
-      </c>
-    </row>
-    <row r="43" ht="22" customHeight="1">
+        <v>162.37</v>
+      </c>
+    </row>
+    <row r="43" ht="33" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0177</t>
+          <t>35.190.1101 (montaj)</t>
         </is>
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>835.1</v>
+        <v>25.36</v>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 35.190.1101 pozunun 01.06.2026 tarihli MONTAJ fiyatı 25,36 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 154,64 x 1,25 + montaj 25,36 = 218,66 TL</t>
         </is>
       </c>
       <c r="F43" s="20">
@@ -2262,6 +2262,206 @@
         <v/>
       </c>
       <c r="I43" s="13" t="n">
+        <v>21.3</v>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>43.527.1001</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="inlineStr">
+        <is>
+          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>393.69</v>
+      </c>
+      <c r="E44" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F44" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G44" s="5">
+        <f>D44*(1-F44)</f>
+        <v/>
+      </c>
+      <c r="H44" s="5">
+        <f>D44*$D$3</f>
+        <v/>
+      </c>
+      <c r="I44" s="13" t="n">
+        <v>330.7</v>
+      </c>
+    </row>
+    <row r="45" ht="14" customHeight="1">
+      <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0115</t>
+        </is>
+      </c>
+      <c r="B45" s="18" t="inlineStr">
+        <is>
+          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>271.25</v>
+      </c>
+      <c r="E45" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F45" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G45" s="5">
+        <f>D45*(1-F45)</f>
+        <v/>
+      </c>
+      <c r="H45" s="5">
+        <f>D45*$D$3</f>
+        <v/>
+      </c>
+      <c r="I45" s="13" t="n">
+        <v>227.85</v>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0151</t>
+        </is>
+      </c>
+      <c r="B46" s="18" t="inlineStr">
+        <is>
+          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>1035.88</v>
+      </c>
+      <c r="E46" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F46" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G46" s="5">
+        <f>D46*(1-F46)</f>
+        <v/>
+      </c>
+      <c r="H46" s="5">
+        <f>D46*$D$3</f>
+        <v/>
+      </c>
+      <c r="I46" s="13" t="n">
+        <v>870.14</v>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0175</t>
+        </is>
+      </c>
+      <c r="B47" s="18" t="inlineStr">
+        <is>
+          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="n">
+        <v>3199.68</v>
+      </c>
+      <c r="E47" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F47" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G47" s="5">
+        <f>D47*(1-F47)</f>
+        <v/>
+      </c>
+      <c r="H47" s="5">
+        <f>D47*$D$3</f>
+        <v/>
+      </c>
+      <c r="I47" s="13" t="n">
+        <v>2687.73</v>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0177</t>
+        </is>
+      </c>
+      <c r="B48" s="18" t="inlineStr">
+        <is>
+          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="n">
+        <v>835.1</v>
+      </c>
+      <c r="E48" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F48" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G48" s="5">
+        <f>D48*(1-F48)</f>
+        <v/>
+      </c>
+      <c r="H48" s="5">
+        <f>D48*$D$3</f>
+        <v/>
+      </c>
+      <c r="I48" s="13" t="n">
         <v>701.48</v>
       </c>
     </row>
@@ -2280,7 +2480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3652,51 +3852,206 @@
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="7" t="n"/>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="24" t="inlineStr">
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100</t>
+        </is>
+      </c>
+      <c r="C48" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F48" s="23">
+        <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G48" s="5">
+        <f>ROUND(E48*F48,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100 (montaj)</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F49" s="23">
+        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="5">
+        <f>ROUND(E49*F49,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="14" customHeight="1">
+      <c r="A50" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F50" s="23">
+        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="5">
+        <f>ROUND(E50*F50,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101 (montaj)</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F51" s="23">
+        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="5">
+        <f>ROUND(E51*F51,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="14" customHeight="1">
+      <c r="A52" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" s="21" t="inlineStr">
+        <is>
+          <t>30.190.1304</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E52" s="22" t="n">
+        <v>123</v>
+      </c>
+      <c r="F52" s="23">
+        <f>IFERROR(VLOOKUP($B52,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G52" s="5">
+        <f>ROUND(E52*F52,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="n"/>
+      <c r="B53" s="7" t="n"/>
+      <c r="C53" s="24" t="inlineStr">
         <is>
           <t>ARA TOPLAM (KDV hariç)</t>
         </is>
       </c>
-      <c r="D48" s="7" t="n"/>
-      <c r="E48" s="7" t="n"/>
-      <c r="F48" s="7" t="n"/>
-      <c r="G48" s="9">
-        <f>SUM(G6:G47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="25" t="inlineStr">
+      <c r="D53" s="7" t="n"/>
+      <c r="E53" s="7" t="n"/>
+      <c r="F53" s="7" t="n"/>
+      <c r="G53" s="9">
+        <f>SUM(G6:G52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n"/>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="25" t="inlineStr">
         <is>
           <t>KDV</t>
         </is>
       </c>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="5">
-        <f>G48*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="11" t="n"/>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="26" t="inlineStr">
+      <c r="D54" s="4" t="n"/>
+      <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="5">
+        <f>G53*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="n"/>
+      <c r="B55" s="11" t="n"/>
+      <c r="C55" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="13">
-        <f>G48+G49</f>
+      <c r="D55" s="11" t="n"/>
+      <c r="E55" s="11" t="n"/>
+      <c r="F55" s="11" t="n"/>
+      <c r="G55" s="13">
+        <f>G53+G54</f>
         <v/>
       </c>
     </row>
@@ -3716,7 +4071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5088,51 +5443,206 @@
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="7" t="n"/>
-      <c r="B48" s="7" t="n"/>
-      <c r="C48" s="24" t="inlineStr">
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100</t>
+        </is>
+      </c>
+      <c r="C48" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F48" s="23">
+        <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G48" s="5">
+        <f>ROUND(E48*F48,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100 (montaj)</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F49" s="23">
+        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="5">
+        <f>ROUND(E49*F49,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="14" customHeight="1">
+      <c r="A50" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F50" s="23">
+        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="5">
+        <f>ROUND(E50*F50,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101 (montaj)</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F51" s="23">
+        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="5">
+        <f>ROUND(E51*F51,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="14" customHeight="1">
+      <c r="A52" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" s="21" t="inlineStr">
+        <is>
+          <t>30.190.1304</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E52" s="22" t="n">
+        <v>123</v>
+      </c>
+      <c r="F52" s="23">
+        <f>IFERROR(VLOOKUP($B52,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G52" s="5">
+        <f>ROUND(E52*F52,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="n"/>
+      <c r="B53" s="7" t="n"/>
+      <c r="C53" s="24" t="inlineStr">
         <is>
           <t>ARA TOPLAM (KDV hariç)</t>
         </is>
       </c>
-      <c r="D48" s="7" t="n"/>
-      <c r="E48" s="7" t="n"/>
-      <c r="F48" s="7" t="n"/>
-      <c r="G48" s="9">
-        <f>SUM(G6:G47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="25" t="inlineStr">
+      <c r="D53" s="7" t="n"/>
+      <c r="E53" s="7" t="n"/>
+      <c r="F53" s="7" t="n"/>
+      <c r="G53" s="9">
+        <f>SUM(G6:G52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n"/>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="25" t="inlineStr">
         <is>
           <t>KDV</t>
         </is>
       </c>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="5">
-        <f>G48*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="11" t="n"/>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="26" t="inlineStr">
+      <c r="D54" s="4" t="n"/>
+      <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="5">
+        <f>G53*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="11" t="n"/>
+      <c r="B55" s="11" t="n"/>
+      <c r="C55" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="13">
-        <f>G48+G49</f>
+      <c r="D55" s="11" t="n"/>
+      <c r="E55" s="11" t="n"/>
+      <c r="F55" s="11" t="n"/>
+      <c r="G55" s="13">
+        <f>G53+G54</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: teklif belgeleri keşif özetinin satırlarına hizalandı
Dört belge artık satır satır aynı: keşif özeti, teklif sunum formu,
yapı teklifleri ve teklif çalışma kitabı. Tutarlar değişmedi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>'01 Kümes A Blok'!$G$53</f>
+        <f>'01 Kümes A Blok'!$G$49</f>
         <v/>
       </c>
       <c r="D4" s="6">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>'02 Kümes B Blok'!$G$53</f>
+        <f>'02 Kümes B Blok'!$G$49</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -753,7 +753,7 @@
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Makine ile kazı yapılması — kümes A ve B blok</t>
+          <t>Makine ile yumuşak ve sert toprak kazılması</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -785,7 +785,7 @@
         <v>52.37</v>
       </c>
     </row>
-    <row r="7" ht="14" customHeight="1">
+    <row r="7" ht="33" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>15.150.1003</t>
@@ -793,7 +793,7 @@
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>C 16/20 hazır beton dökülmesi — kümes temel altı grobeton</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 16/20 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -825,7 +825,7 @@
         <v>2750.45</v>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
+    <row r="8" ht="33" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>15.150.1005</t>
@@ -833,7 +833,7 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>C 25/30 hazır beton dökülmesi — kümes şerit temel ve bağ kirişleri</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 25/30 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>Nervürlü çelik hasırın yerine konulması — kümes döşemeleri</t>
+          <t>Nervürlü çelik hasırın yerine konulması</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -905,7 +905,7 @@
         <v>36949.5</v>
       </c>
     </row>
-    <row r="10" ht="14" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>15.160.1003</t>
@@ -913,7 +913,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Ø8-Ø12 nervürlü beton çelik çubuğu — kümes temelleri</t>
+          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -945,7 +945,7 @@
         <v>39045.24</v>
       </c>
     </row>
-    <row r="11" ht="14" customHeight="1">
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>15.160.1004</t>
@@ -953,7 +953,7 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>Ø14-Ø28 nervürlü beton çelik çubuğu — kümes temelleri</t>
+          <t>Ø 14 - Ø 28 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>Her çeşit profil, çelik çubuk ve saclarla karkas (çerçeve) inşaat yapılması, yerine tespiti — kümes çelik taşıyıcı sistemi</t>
+          <t>Her çeşit profil, çelik çubuk ve çelik saclarla karkas (çerçeve) inşaat yapılması, yerine tespiti (boya bedeli hariç)</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Plywood ile düz yüzeyli betonarme kalıbı — kümes temelleri</t>
+          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>10 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile bölme duvar yapılması — servis bölümü</t>
+          <t>10 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>20 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile) — cephe duvarı</t>
+          <t>20 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>20 cm kalınlığındaki teçhizatlı gazbeton lento temini ve yerine konulması — boşluk üstü lento ve yatay hatıl</t>
+          <t>20 cm kalınlığındaki teçhizatlı gazbeton lento temini ve yerine konulması</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1185,7 +1185,7 @@
         <v>1777.52</v>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
+    <row r="17" ht="14" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>15.275.1116</t>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>250 kg çimento dozlu harç ile kaba sıva yapılması — cephe duvarı dış yüzü</t>
+          <t>250 kg çimento dozlu harç ile kaba sıva yapılması</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması (iç cephe) — cephe duvarı iç yüzü</t>
+          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması (iç cephe)</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1265,7 +1265,7 @@
         <v>381.49</v>
       </c>
     </row>
-    <row r="19" ht="14" customHeight="1">
+    <row r="19" ht="22" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>15.315.1001</t>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>Ø70 sert PVC yağmur suyu iniş borusu temini ve yerine tesbiti</t>
+          <t>Ø 70 mm çapında bir ucu muflu sert PVC yağmur borusu temini ve yerine tesbiti</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="B20" s="18" t="inlineStr">
         <is>
-          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası</t>
+          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası yapılması</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası</t>
+          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası yapılması</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="B22" s="18" t="inlineStr">
         <is>
-          <t>1,50 mm sacdan bükme kapı kasası yapılması ve yerine konulması — servis bölümü iç kapıları</t>
+          <t>1,50 mm kalınlığında sıcak haddelenmiş sacdan bükme kapı kasası yapılması ve yerine konulması</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>Lama ve profil demirlerden mahya, saçak ve köşe kapama profilleri</t>
+          <t>Lama ve profil demirlerden çeşitli demir işleri yapılması ve yerine konulması</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="B24" s="18" t="inlineStr">
         <is>
-          <t>Kümes dağıtım panosu (sıva üstü galvanizli sac tablo, 0,40-0,50 m²)</t>
+          <t>Kümes dağıtım panosu (sıva üstü galvanizli sac tablo, 0,40-0,50 m²) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>Termik-manyetik kompakt şalter 3x100 A, Icu 35 kA — kümes besleme</t>
+          <t>Termik-manyetik kompakt şalter 3x100 A, Icu 35 kA — kümes besleme (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1545,7 +1545,7 @@
         <v>3528.05</v>
       </c>
     </row>
-    <row r="26" ht="14" customHeight="1">
+    <row r="26" ht="22" customHeight="1">
       <c r="A26" s="17" t="inlineStr">
         <is>
           <t>30.115.1003</t>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="B26" s="18" t="inlineStr">
         <is>
-          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA</t>
+          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>Çıplak bakır tel 25 mm² — eşpotansiyel bara ve topraklama iletkeni</t>
+          <t>Çıplak bakır tel 25 mm² — eşpotansiyel bara ve topraklama iletkeni (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="B28" s="18" t="inlineStr">
         <is>
-          <t>YVV (NYY) 1 kV yeraltı kablosu ile kolon hattı tesisi — 1x25 mm²</t>
+          <t>YVV (NYY) 1 kV yeraltı kablosu ile kolon hattı tesisi — 1x25 mm² (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1665,7 +1665,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="29" ht="14" customHeight="1">
+    <row r="29" ht="22" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
           <t>30.150.1401</t>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>Halojensiz H07Z tipi iletken 1x1,5 mm² ile kumanda tesisatı</t>
+          <t>Halojensiz H07Z tipi iletken 1x1,5 mm² ile kumanda tesisatı (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1705,7 +1705,7 @@
         <v>12.22</v>
       </c>
     </row>
-    <row r="30" ht="14" customHeight="1">
+    <row r="30" ht="22" customHeight="1">
       <c r="A30" s="17" t="inlineStr">
         <is>
           <t>30.150.1402</t>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="B30" s="18" t="inlineStr">
         <is>
-          <t>Halojensiz H07Z tipi iletken 1x2,5 mm² ile tesisat</t>
+          <t>Halojensiz H07Z tipi iletken 1x2,5 mm² ile tesisat (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1745,7 +1745,7 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="31" ht="14" customHeight="1">
+    <row r="31" ht="22" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
           <t>30.160.6102</t>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>Boş boru döşemesi — 25-32 mm PVC boru</t>
+          <t>Boş boru döşemesi — 25-32 mm PVC boru (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="B32" s="18" t="inlineStr">
         <is>
-          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 1800 lm — servis bölümü</t>
+          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 1800 lm — servis bölümü (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1825,7 +1825,7 @@
         <v>1370.96</v>
       </c>
     </row>
-    <row r="33" ht="22" customHeight="1">
+    <row r="33" ht="33" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
           <t>30.170.1602</t>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 2700 lm — kümes genel aydınlatması</t>
+          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 2700 lm — kümes genel aydınlatması (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1865,7 +1865,7 @@
         <v>1996.08</v>
       </c>
     </row>
-    <row r="34" ht="14" customHeight="1">
+    <row r="34" ht="22" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
           <t>30.190.1304</t>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
-          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli</t>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1905,7 +1905,7 @@
         <v>233.28</v>
       </c>
     </row>
-    <row r="35" ht="22" customHeight="1">
+    <row r="35" ht="33" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
           <t>30.740.1106</t>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -1945,7 +1945,7 @@
         <v>467349.29</v>
       </c>
     </row>
-    <row r="36" ht="14" customHeight="1">
+    <row r="36" ht="22" customHeight="1">
       <c r="A36" s="17" t="inlineStr">
         <is>
           <t>30.740.5406</t>
@@ -1953,7 +1953,7 @@
       </c>
       <c r="B36" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -1985,7 +1985,7 @@
         <v>79653.55</v>
       </c>
     </row>
-    <row r="37" ht="14" customHeight="1">
+    <row r="37" ht="22" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
           <t>30.750.1502</t>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
+          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2113,7 +2113,7 @@
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
+          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2185,7 +2185,7 @@
         <v>38.72</v>
       </c>
     </row>
-    <row r="42" ht="22" customHeight="1">
+    <row r="42" ht="33" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
           <t>35.190.1101</t>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
+          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B44" s="18" t="inlineStr">
         <is>
-          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>Çapı 150 mm HDPE koruge boru döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
+          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -2345,7 +2345,7 @@
         <v>227.85</v>
       </c>
     </row>
-    <row r="46" ht="22" customHeight="1">
+    <row r="46" ht="33" customHeight="1">
       <c r="A46" s="17" t="inlineStr">
         <is>
           <t>TKDK-0151</t>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B46" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
+          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2385,7 +2385,7 @@
         <v>870.14</v>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
+    <row r="47" ht="33" customHeight="1">
       <c r="A47" s="17" t="inlineStr">
         <is>
           <t>TKDK-0175</t>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2425,7 +2425,7 @@
         <v>2687.73</v>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1">
+    <row r="48" ht="44" customHeight="1">
       <c r="A48" s="17" t="inlineStr">
         <is>
           <t>TKDK-0177</t>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="B48" s="18" t="inlineStr">
         <is>
-          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -2480,7 +2480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Makine ile kazı yapılması — kümes A ve B blok</t>
+          <t>Makine ile yumuşak ve sert toprak kazılması</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -2581,7 +2581,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="14" customHeight="1">
+    <row r="7" ht="33" customHeight="1">
       <c r="A7" s="3" t="n">
         <v>2</v>
       </c>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>C 16/20 hazır beton dökülmesi — kümes temel altı grobeton</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 16/20 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -2612,7 +2612,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="14" customHeight="1">
+    <row r="8" ht="33" customHeight="1">
       <c r="A8" s="3" t="n">
         <v>3</v>
       </c>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>C 25/30 hazır beton dökülmesi — kümes şerit temel ve bağ kirişleri</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 25/30 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -2632,7 +2632,7 @@
         </is>
       </c>
       <c r="E8" s="22" t="n">
-        <v>115.71</v>
+        <v>278.34</v>
       </c>
       <c r="F8" s="23">
         <f>IFERROR(VLOOKUP($B8,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2649,21 +2649,21 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>15.150.1005</t>
+          <t>15.180.1003</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>C 25/30 hazır beton dökülmesi — kümes zemin döşemeleri (15 cm)</t>
+          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E9" s="22" t="n">
-        <v>162.63</v>
+        <v>551.26</v>
       </c>
       <c r="F9" s="23">
         <f>IFERROR(VLOOKUP($B9,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2674,27 +2674,27 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="14" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="3" t="n">
         <v>5</v>
       </c>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>15.180.1003</t>
+          <t>15.160.1003</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>Plywood ile düz yüzeyli betonarme kalıbı — kümes temelleri</t>
+          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>ton</t>
         </is>
       </c>
       <c r="E10" s="22" t="n">
-        <v>551.26</v>
+        <v>4.16</v>
       </c>
       <c r="F10" s="23">
         <f>IFERROR(VLOOKUP($B10,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2705,18 +2705,18 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="14" customHeight="1">
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="3" t="n">
         <v>6</v>
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>15.160.1003</t>
+          <t>15.160.1004</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>Ø8-Ø12 nervürlü beton çelik çubuğu — kümes temelleri</t>
+          <t>Ø 14 - Ø 28 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -2725,7 +2725,7 @@
         </is>
       </c>
       <c r="E11" s="22" t="n">
-        <v>4.16</v>
+        <v>7.288</v>
       </c>
       <c r="F11" s="23">
         <f>IFERROR(VLOOKUP($B11,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2742,12 +2742,12 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>15.160.1004</t>
+          <t>15.160.1002</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>Ø14-Ø28 nervürlü beton çelik çubuğu — kümes temelleri</t>
+          <t>Nervürlü çelik hasırın yerine konulması</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -2756,7 +2756,7 @@
         </is>
       </c>
       <c r="E12" s="22" t="n">
-        <v>7.288</v>
+        <v>3.637</v>
       </c>
       <c r="F12" s="23">
         <f>IFERROR(VLOOKUP($B12,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2767,18 +2767,18 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="14" customHeight="1">
+    <row r="13" ht="22" customHeight="1">
       <c r="A13" s="3" t="n">
         <v>8</v>
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>15.160.1002</t>
+          <t>15.165.1003</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>Nervürlü çelik hasırın yerine konulması — kümes döşemeleri</t>
+          <t>Her çeşit profil, çelik çubuk ve çelik saclarla karkas (çerçeve) inşaat yapılması, yerine tespiti (boya bedeli hariç)</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -2787,7 +2787,7 @@
         </is>
       </c>
       <c r="E13" s="22" t="n">
-        <v>3.637</v>
+        <v>44.048</v>
       </c>
       <c r="F13" s="23">
         <f>IFERROR(VLOOKUP($B13,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2804,21 +2804,21 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>15.165.1003</t>
+          <t>15.225.1010</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>Her çeşit profil, çelik çubuk ve saclarla karkas (çerçeve) inşaat yapılması, yerine tespiti — kümes çelik taşıyıcı sistemi</t>
+          <t>20 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E14" s="22" t="n">
-        <v>44.048</v>
+        <v>507.91</v>
       </c>
       <c r="F14" s="23">
         <f>IFERROR(VLOOKUP($B14,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2829,18 +2829,18 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
+    <row r="15" ht="14" customHeight="1">
       <c r="A15" s="3" t="n">
         <v>10</v>
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>15.225.1010</t>
+          <t>15.225.1410</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>20 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile) — cephe duvarı</t>
+          <t>20 cm kalınlığındaki teçhizatlı gazbeton lento temini ve yerine konulması</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -2849,7 +2849,7 @@
         </is>
       </c>
       <c r="E15" s="22" t="n">
-        <v>507.91</v>
+        <v>49.85</v>
       </c>
       <c r="F15" s="23">
         <f>IFERROR(VLOOKUP($B15,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2860,18 +2860,18 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
+    <row r="16" ht="14" customHeight="1">
       <c r="A16" s="3" t="n">
         <v>11</v>
       </c>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>15.225.1410</t>
+          <t>15.275.1116</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>20 cm kalınlığındaki teçhizatlı gazbeton lento temini ve yerine konulması — boşluk üstü lento ve yatay hatıl</t>
+          <t>250 kg çimento dozlu harç ile kaba sıva yapılması</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -2880,7 +2880,7 @@
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>49.85</v>
+        <v>557.76</v>
       </c>
       <c r="F16" s="23">
         <f>IFERROR(VLOOKUP($B16,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2897,12 +2897,12 @@
       </c>
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>15.275.1116</t>
+          <t>15.275.1117</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>250 kg çimento dozlu harç ile kaba sıva yapılması — cephe duvarı dış yüzü</t>
+          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması (iç cephe)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>557.76</v>
+        <v>647.76</v>
       </c>
       <c r="F17" s="23">
         <f>IFERROR(VLOOKUP($B17,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2928,12 +2928,12 @@
       </c>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>15.275.1117</t>
+          <t>15.540.1606</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması (iç cephe) — cephe duvarı iç yüzü</t>
+          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası yapılması</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -2959,12 +2959,12 @@
       </c>
       <c r="B19" s="21" t="inlineStr">
         <is>
-          <t>15.540.1606</t>
+          <t>15.540.1537</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası</t>
+          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası yapılması</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -2973,7 +2973,7 @@
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>557.76</v>
+        <v>612.76</v>
       </c>
       <c r="F19" s="23">
         <f>IFERROR(VLOOKUP($B19,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2984,27 +2984,27 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
+    <row r="20" ht="14" customHeight="1">
       <c r="A20" s="3" t="n">
         <v>15</v>
       </c>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>15.540.1537</t>
+          <t>15.550.1202</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası</t>
+          <t>Lama ve profil demirlerden çeşitli demir işleri yapılması ve yerine konulması</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>557.76</v>
+        <v>674</v>
       </c>
       <c r="F20" s="23">
         <f>IFERROR(VLOOKUP($B20,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3021,12 +3021,12 @@
       </c>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>15.550.1202</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Lama ve profil demirlerden mahya, saçak ve köşe kapama profilleri</t>
+          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -3035,7 +3035,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>674</v>
+        <v>319.2</v>
       </c>
       <c r="F21" s="23">
         <f>IFERROR(VLOOKUP($B21,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3052,21 +3052,21 @@
       </c>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>15.315.1001</t>
         </is>
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
+          <t>Ø 70 mm çapında bir ucu muflu sert PVC yağmur borusu temini ve yerine tesbiti</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>319.2</v>
+        <v>51.2</v>
       </c>
       <c r="F22" s="23">
         <f>IFERROR(VLOOKUP($B22,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3077,27 +3077,27 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="14" customHeight="1">
+    <row r="23" ht="22" customHeight="1">
       <c r="A23" s="3" t="n">
         <v>18</v>
       </c>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>15.315.1001</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Ø70 sert PVC yağmur suyu iniş borusu temini ve yerine tesbiti</t>
+          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>51.2</v>
+        <v>13.4</v>
       </c>
       <c r="F23" s="23">
         <f>IFERROR(VLOOKUP($B23,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3114,12 +3114,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>15.225.1004</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
+          <t>10 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -3128,7 +3128,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>4.4</v>
+        <v>45</v>
       </c>
       <c r="F24" s="23">
         <f>IFERROR(VLOOKUP($B24,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3139,18 +3139,18 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
+    <row r="25" ht="33" customHeight="1">
       <c r="A25" s="3" t="n">
         <v>20</v>
       </c>
       <c r="B25" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>TKDK-0177</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — yükleme/temizlik kapısı 300/300 sürgülü</t>
+          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>9</v>
+        <v>60</v>
       </c>
       <c r="F25" s="23">
         <f>IFERROR(VLOOKUP($B25,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3176,12 +3176,12 @@
       </c>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>15.225.1004</t>
+          <t>TKDK-0175</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>10 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile bölme duvar yapılması — servis bölümü</t>
+          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -3190,7 +3190,7 @@
         </is>
       </c>
       <c r="E26" s="22" t="n">
-        <v>45</v>
+        <v>5.67</v>
       </c>
       <c r="F26" s="23">
         <f>IFERROR(VLOOKUP($B26,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3207,21 +3207,21 @@
       </c>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>15.275.1117</t>
+          <t>15.550.1002</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması — servis bölümü bölme duvarları</t>
+          <t>1,50 mm kalınlığında sıcak haddelenmiş sacdan bükme kapı kasası yapılması ve yerine konulması</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E27" s="22" t="n">
-        <v>90</v>
+        <v>54.315</v>
       </c>
       <c r="F27" s="23">
         <f>IFERROR(VLOOKUP($B27,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3232,27 +3232,27 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
+    <row r="28" ht="14" customHeight="1">
       <c r="A28" s="3" t="n">
         <v>23</v>
       </c>
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0177</t>
+          <t>43.527.1001</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
         <is>
-          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+          <t>Çapı 150 mm HDPE koruge boru döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E28" s="22" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="F28" s="23">
         <f>IFERROR(VLOOKUP($B28,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3269,21 +3269,21 @@
       </c>
       <c r="B29" s="21" t="inlineStr">
         <is>
-          <t>15.540.1537</t>
+          <t>30.100.2105</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel boya — servis bölümü</t>
+          <t>Kümes dağıtım panosu (sıva üstü galvanizli sac tablo, 0,40-0,50 m²) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="F29" s="23">
         <f>IFERROR(VLOOKUP($B29,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3300,21 +3300,21 @@
       </c>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0175</t>
+          <t>30.110.1102</t>
         </is>
       </c>
       <c r="C30" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+          <t>Termik-manyetik kompakt şalter 3x100 A, Icu 35 kA — kümes besleme (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E30" s="22" t="n">
-        <v>5.67</v>
+        <v>1</v>
       </c>
       <c r="F30" s="23">
         <f>IFERROR(VLOOKUP($B30,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3325,27 +3325,27 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="22" customHeight="1">
+    <row r="31" ht="14" customHeight="1">
       <c r="A31" s="3" t="n">
         <v>26</v>
       </c>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>15.550.1002</t>
+          <t>30.115.1003</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>1,50 mm sacdan bükme kapı kasası yapılması ve yerine konulması — servis bölümü iç kapıları</t>
+          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E31" s="22" t="n">
-        <v>54.315</v>
+        <v>2</v>
       </c>
       <c r="F31" s="23">
         <f>IFERROR(VLOOKUP($B31,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3362,12 +3362,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>30.140.3104</t>
         </is>
       </c>
       <c r="C32" s="18" t="inlineStr">
         <is>
-          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>YVV (NYY) 1 kV yeraltı kablosu ile kolon hattı tesisi — 1x25 mm² (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -3376,7 +3376,7 @@
         </is>
       </c>
       <c r="E32" s="22" t="n">
-        <v>25</v>
+        <v>300</v>
       </c>
       <c r="F32" s="23">
         <f>IFERROR(VLOOKUP($B32,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3387,18 +3387,18 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="14" customHeight="1">
+    <row r="33" ht="22" customHeight="1">
       <c r="A33" s="3" t="n">
         <v>28</v>
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>30.100.2105</t>
+          <t>30.170.1602</t>
         </is>
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>Kümes dağıtım panosu (sıva üstü galvanizli sac tablo, 0,40-0,50 m²)</t>
+          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 2700 lm — kümes genel aydınlatması (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -3407,7 +3407,7 @@
         </is>
       </c>
       <c r="E33" s="22" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="F33" s="23">
         <f>IFERROR(VLOOKUP($B33,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3418,18 +3418,18 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="14" customHeight="1">
+    <row r="34" ht="22" customHeight="1">
       <c r="A34" s="3" t="n">
         <v>29</v>
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>30.110.1102</t>
+          <t>30.170.1601</t>
         </is>
       </c>
       <c r="C34" s="18" t="inlineStr">
         <is>
-          <t>Termik-manyetik kompakt şalter 3x100 A, Icu 35 kA — kümes besleme</t>
+          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 1800 lm — servis bölümü (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -3438,7 +3438,7 @@
         </is>
       </c>
       <c r="E34" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F34" s="23">
         <f>IFERROR(VLOOKUP($B34,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3455,21 +3455,21 @@
       </c>
       <c r="B35" s="21" t="inlineStr">
         <is>
-          <t>30.115.1003</t>
+          <t>30.160.6102</t>
         </is>
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA</t>
+          <t>Boş boru döşemesi — 25-32 mm PVC boru (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E35" s="22" t="n">
-        <v>2</v>
+        <v>500</v>
       </c>
       <c r="F35" s="23">
         <f>IFERROR(VLOOKUP($B35,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3486,12 +3486,12 @@
       </c>
       <c r="B36" s="21" t="inlineStr">
         <is>
-          <t>30.140.3104</t>
+          <t>30.150.1402</t>
         </is>
       </c>
       <c r="C36" s="18" t="inlineStr">
         <is>
-          <t>YVV (NYY) 1 kV yeraltı kablosu ile kolon hattı tesisi — 1x25 mm²</t>
+          <t>Halojensiz H07Z tipi iletken 1x2,5 mm² ile tesisat (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -3500,7 +3500,7 @@
         </is>
       </c>
       <c r="E36" s="22" t="n">
-        <v>300</v>
+        <v>2000</v>
       </c>
       <c r="F36" s="23">
         <f>IFERROR(VLOOKUP($B36,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3517,21 +3517,21 @@
       </c>
       <c r="B37" s="21" t="inlineStr">
         <is>
-          <t>30.170.1602</t>
+          <t>30.150.1401</t>
         </is>
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 2700 lm — kümes genel aydınlatması</t>
+          <t>Halojensiz H07Z tipi iletken 1x1,5 mm² ile kumanda tesisatı (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E37" s="22" t="n">
-        <v>30</v>
+        <v>600</v>
       </c>
       <c r="F37" s="23">
         <f>IFERROR(VLOOKUP($B37,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3548,21 +3548,21 @@
       </c>
       <c r="B38" s="21" t="inlineStr">
         <is>
-          <t>30.170.1601</t>
+          <t>30.140.1105</t>
         </is>
       </c>
       <c r="C38" s="18" t="inlineStr">
         <is>
-          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 1800 lm — servis bölümü</t>
+          <t>Çıplak bakır tel 25 mm² — eşpotansiyel bara ve topraklama iletkeni (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E38" s="22" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="F38" s="23">
         <f>IFERROR(VLOOKUP($B38,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3573,18 +3573,18 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="14" customHeight="1">
+    <row r="39" ht="22" customHeight="1">
       <c r="A39" s="3" t="n">
         <v>34</v>
       </c>
       <c r="B39" s="21" t="inlineStr">
         <is>
-          <t>30.160.6102</t>
+          <t>30.750.3002</t>
         </is>
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>Boş boru döşemesi — 25-32 mm PVC boru</t>
+          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -3593,7 +3593,7 @@
         </is>
       </c>
       <c r="E39" s="22" t="n">
-        <v>500</v>
+        <v>186</v>
       </c>
       <c r="F39" s="23">
         <f>IFERROR(VLOOKUP($B39,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3610,21 +3610,21 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>30.150.1402</t>
+          <t>30.750.1502</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
-          <t>Halojensiz H07Z tipi iletken 1x2,5 mm² ile tesisat</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E40" s="22" t="n">
-        <v>2000</v>
+        <v>1</v>
       </c>
       <c r="F40" s="23">
         <f>IFERROR(VLOOKUP($B40,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3635,18 +3635,18 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="14" customHeight="1">
+    <row r="41" ht="22" customHeight="1">
       <c r="A41" s="3" t="n">
         <v>36</v>
       </c>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>30.150.1401</t>
+          <t>30.750.2001</t>
         </is>
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>Halojensiz H07Z tipi iletken 1x1,5 mm² ile kumanda tesisatı</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -3655,7 +3655,7 @@
         </is>
       </c>
       <c r="E41" s="22" t="n">
-        <v>600</v>
+        <v>16</v>
       </c>
       <c r="F41" s="23">
         <f>IFERROR(VLOOKUP($B41,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3666,27 +3666,27 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="14" customHeight="1">
+    <row r="42" ht="22" customHeight="1">
       <c r="A42" s="3" t="n">
         <v>37</v>
       </c>
       <c r="B42" s="21" t="inlineStr">
         <is>
-          <t>30.140.1105</t>
+          <t>30.740.1106</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
         <is>
-          <t>Çıplak bakır tel 25 mm² — eşpotansiyel bara ve topraklama iletkeni</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E42" s="22" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F42" s="23">
         <f>IFERROR(VLOOKUP($B42,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3703,21 +3703,21 @@
       </c>
       <c r="B43" s="21" t="inlineStr">
         <is>
-          <t>30.750.3002</t>
+          <t>30.740.5406</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E43" s="22" t="n">
-        <v>186</v>
+        <v>1</v>
       </c>
       <c r="F43" s="23">
         <f>IFERROR(VLOOKUP($B43,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3728,27 +3728,27 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="14" customHeight="1">
+    <row r="44" ht="22" customHeight="1">
       <c r="A44" s="3" t="n">
         <v>39</v>
       </c>
       <c r="B44" s="21" t="inlineStr">
         <is>
-          <t>30.750.1502</t>
+          <t>35.190.1100</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
+          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E44" s="22" t="n">
-        <v>1</v>
+        <v>502</v>
       </c>
       <c r="F44" s="23">
         <f>IFERROR(VLOOKUP($B44,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3759,27 +3759,27 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="14" customHeight="1">
+    <row r="45" ht="22" customHeight="1">
       <c r="A45" s="3" t="n">
         <v>40</v>
       </c>
       <c r="B45" s="21" t="inlineStr">
         <is>
-          <t>30.750.2001</t>
+          <t>35.190.1100 (montaj)</t>
         </is>
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E45" s="22" t="n">
-        <v>16</v>
+        <v>502</v>
       </c>
       <c r="F45" s="23">
         <f>IFERROR(VLOOKUP($B45,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3796,21 +3796,21 @@
       </c>
       <c r="B46" s="21" t="inlineStr">
         <is>
-          <t>30.740.1106</t>
+          <t>35.190.1101</t>
         </is>
       </c>
       <c r="C46" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
+          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E46" s="22" t="n">
-        <v>1</v>
+        <v>361.2</v>
       </c>
       <c r="F46" s="23">
         <f>IFERROR(VLOOKUP($B46,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3821,27 +3821,27 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="14" customHeight="1">
+    <row r="47" ht="22" customHeight="1">
       <c r="A47" s="3" t="n">
         <v>42</v>
       </c>
       <c r="B47" s="21" t="inlineStr">
         <is>
-          <t>30.740.5406</t>
+          <t>35.190.1101 (montaj)</t>
         </is>
       </c>
       <c r="C47" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E47" s="22" t="n">
-        <v>1</v>
+        <v>361.2</v>
       </c>
       <c r="F47" s="23">
         <f>IFERROR(VLOOKUP($B47,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3858,21 +3858,21 @@
       </c>
       <c r="B48" s="21" t="inlineStr">
         <is>
-          <t>35.190.1100</t>
+          <t>30.190.1304</t>
         </is>
       </c>
       <c r="C48" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E48" s="22" t="n">
-        <v>502</v>
+        <v>123</v>
       </c>
       <c r="F48" s="23">
         <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3883,175 +3883,51 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="3" t="n">
-        <v>44</v>
-      </c>
-      <c r="B49" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1100 (montaj)</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E49" s="22" t="n">
-        <v>502</v>
-      </c>
-      <c r="F49" s="23">
-        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G49" s="5">
-        <f>ROUND(E49*F49,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="14" customHeight="1">
-      <c r="A50" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="B50" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101</t>
-        </is>
-      </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E50" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F50" s="23">
-        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
+    <row r="49">
+      <c r="A49" s="7" t="n"/>
+      <c r="B49" s="7" t="n"/>
+      <c r="C49" s="24" t="inlineStr">
+        <is>
+          <t>ARA TOPLAM (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="n"/>
+      <c r="E49" s="7" t="n"/>
+      <c r="F49" s="7" t="n"/>
+      <c r="G49" s="9">
+        <f>SUM(G6:G48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n"/>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="25" t="inlineStr">
+        <is>
+          <t>KDV</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
       <c r="G50" s="5">
-        <f>ROUND(E50*F50,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="B51" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101 (montaj)</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E51" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F51" s="23">
-        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G51" s="5">
-        <f>ROUND(E51*F51,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" ht="14" customHeight="1">
-      <c r="A52" s="3" t="n">
-        <v>47</v>
-      </c>
-      <c r="B52" s="21" t="inlineStr">
-        <is>
-          <t>30.190.1304</t>
-        </is>
-      </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E52" s="22" t="n">
-        <v>123</v>
-      </c>
-      <c r="F52" s="23">
-        <f>IFERROR(VLOOKUP($B52,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G52" s="5">
-        <f>ROUND(E52*F52,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="7" t="n"/>
-      <c r="B53" s="7" t="n"/>
-      <c r="C53" s="24" t="inlineStr">
-        <is>
-          <t>ARA TOPLAM (KDV hariç)</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="n"/>
-      <c r="E53" s="7" t="n"/>
-      <c r="F53" s="7" t="n"/>
-      <c r="G53" s="9">
-        <f>SUM(G6:G52)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="n"/>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="25" t="inlineStr">
-        <is>
-          <t>KDV</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="5">
-        <f>G53*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="n"/>
-      <c r="B55" s="11" t="n"/>
-      <c r="C55" s="26" t="inlineStr">
+        <f>G49*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="n"/>
+      <c r="B51" s="11" t="n"/>
+      <c r="C51" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D55" s="11" t="n"/>
-      <c r="E55" s="11" t="n"/>
-      <c r="F55" s="11" t="n"/>
-      <c r="G55" s="13">
-        <f>G53+G54</f>
+      <c r="D51" s="11" t="n"/>
+      <c r="E51" s="11" t="n"/>
+      <c r="F51" s="11" t="n"/>
+      <c r="G51" s="13">
+        <f>G49+G50</f>
         <v/>
       </c>
     </row>
@@ -4071,7 +3947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4152,7 +4028,7 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Makine ile kazı yapılması — kümes A ve B blok</t>
+          <t>Makine ile yumuşak ve sert toprak kazılması</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -4172,7 +4048,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="14" customHeight="1">
+    <row r="7" ht="33" customHeight="1">
       <c r="A7" s="3" t="n">
         <v>2</v>
       </c>
@@ -4183,7 +4059,7 @@
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>C 16/20 hazır beton dökülmesi — kümes temel altı grobeton</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 16/20 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -4203,7 +4079,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="14" customHeight="1">
+    <row r="8" ht="33" customHeight="1">
       <c r="A8" s="3" t="n">
         <v>3</v>
       </c>
@@ -4214,7 +4090,7 @@
       </c>
       <c r="C8" s="18" t="inlineStr">
         <is>
-          <t>C 25/30 hazır beton dökülmesi — kümes şerit temel ve bağ kirişleri</t>
+          <t>Beton santralinde üretilen veya satın alınan ve beton pompasıyla basılan, C 25/30 basınç dayanım sınıfında, gri renkte, normal hazır beton dökülmesi (beton nakli dahil)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -4223,7 +4099,7 @@
         </is>
       </c>
       <c r="E8" s="22" t="n">
-        <v>115.71</v>
+        <v>278.34</v>
       </c>
       <c r="F8" s="23">
         <f>IFERROR(VLOOKUP($B8,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4240,21 +4116,21 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t>15.150.1005</t>
+          <t>15.180.1003</t>
         </is>
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>C 25/30 hazır beton dökülmesi — kümes zemin döşemeleri (15 cm)</t>
+          <t>Plywood ile düz yüzeyli betonarme kalıbı yapılması</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E9" s="22" t="n">
-        <v>162.63</v>
+        <v>551.26</v>
       </c>
       <c r="F9" s="23">
         <f>IFERROR(VLOOKUP($B9,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4265,27 +4141,27 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="14" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="A10" s="3" t="n">
         <v>5</v>
       </c>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>15.180.1003</t>
+          <t>15.160.1003</t>
         </is>
       </c>
       <c r="C10" s="18" t="inlineStr">
         <is>
-          <t>Plywood ile düz yüzeyli betonarme kalıbı — kümes temelleri</t>
+          <t>Ø 8 - Ø 12 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>ton</t>
         </is>
       </c>
       <c r="E10" s="22" t="n">
-        <v>551.26</v>
+        <v>4.16</v>
       </c>
       <c r="F10" s="23">
         <f>IFERROR(VLOOKUP($B10,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4296,18 +4172,18 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="14" customHeight="1">
+    <row r="11" ht="22" customHeight="1">
       <c r="A11" s="3" t="n">
         <v>6</v>
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>15.160.1003</t>
+          <t>15.160.1004</t>
         </is>
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>Ø8-Ø12 nervürlü beton çelik çubuğu — kümes temelleri</t>
+          <t>Ø 14 - Ø 28 mm nervürlü beton çelik çubuğu, çubukların kesilmesi, bükülmesi ve yerine konulması</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -4316,7 +4192,7 @@
         </is>
       </c>
       <c r="E11" s="22" t="n">
-        <v>4.16</v>
+        <v>7.288</v>
       </c>
       <c r="F11" s="23">
         <f>IFERROR(VLOOKUP($B11,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4333,12 +4209,12 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>15.160.1004</t>
+          <t>15.160.1002</t>
         </is>
       </c>
       <c r="C12" s="18" t="inlineStr">
         <is>
-          <t>Ø14-Ø28 nervürlü beton çelik çubuğu — kümes temelleri</t>
+          <t>Nervürlü çelik hasırın yerine konulması</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -4347,7 +4223,7 @@
         </is>
       </c>
       <c r="E12" s="22" t="n">
-        <v>7.288</v>
+        <v>3.637</v>
       </c>
       <c r="F12" s="23">
         <f>IFERROR(VLOOKUP($B12,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4358,18 +4234,18 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="14" customHeight="1">
+    <row r="13" ht="22" customHeight="1">
       <c r="A13" s="3" t="n">
         <v>8</v>
       </c>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>15.160.1002</t>
+          <t>15.165.1003</t>
         </is>
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>Nervürlü çelik hasırın yerine konulması — kümes döşemeleri</t>
+          <t>Her çeşit profil, çelik çubuk ve çelik saclarla karkas (çerçeve) inşaat yapılması, yerine tespiti (boya bedeli hariç)</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -4378,7 +4254,7 @@
         </is>
       </c>
       <c r="E13" s="22" t="n">
-        <v>3.637</v>
+        <v>44.048</v>
       </c>
       <c r="F13" s="23">
         <f>IFERROR(VLOOKUP($B13,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4395,21 +4271,21 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>15.165.1003</t>
+          <t>15.225.1010</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>Her çeşit profil, çelik çubuk ve saclarla karkas (çerçeve) inşaat yapılması, yerine tespiti — kümes çelik taşıyıcı sistemi</t>
+          <t>20 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>ton</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E14" s="22" t="n">
-        <v>44.048</v>
+        <v>507.91</v>
       </c>
       <c r="F14" s="23">
         <f>IFERROR(VLOOKUP($B14,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4420,18 +4296,18 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
+    <row r="15" ht="14" customHeight="1">
       <c r="A15" s="3" t="n">
         <v>10</v>
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>15.225.1010</t>
+          <t>15.225.1410</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>20 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile) — cephe duvarı</t>
+          <t>20 cm kalınlığındaki teçhizatlı gazbeton lento temini ve yerine konulması</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -4440,7 +4316,7 @@
         </is>
       </c>
       <c r="E15" s="22" t="n">
-        <v>507.91</v>
+        <v>49.85</v>
       </c>
       <c r="F15" s="23">
         <f>IFERROR(VLOOKUP($B15,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4451,18 +4327,18 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
+    <row r="16" ht="14" customHeight="1">
       <c r="A16" s="3" t="n">
         <v>11</v>
       </c>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>15.225.1410</t>
+          <t>15.275.1116</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>20 cm kalınlığındaki teçhizatlı gazbeton lento temini ve yerine konulması — boşluk üstü lento ve yatay hatıl</t>
+          <t>250 kg çimento dozlu harç ile kaba sıva yapılması</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -4471,7 +4347,7 @@
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>49.85</v>
+        <v>557.76</v>
       </c>
       <c r="F16" s="23">
         <f>IFERROR(VLOOKUP($B16,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4488,12 +4364,12 @@
       </c>
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>15.275.1116</t>
+          <t>15.275.1117</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>250 kg çimento dozlu harç ile kaba sıva yapılması — cephe duvarı dış yüzü</t>
+          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması (iç cephe)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -4502,7 +4378,7 @@
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>557.76</v>
+        <v>647.76</v>
       </c>
       <c r="F17" s="23">
         <f>IFERROR(VLOOKUP($B17,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4519,12 +4395,12 @@
       </c>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>15.275.1117</t>
+          <t>15.540.1606</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması (iç cephe) — cephe duvarı iç yüzü</t>
+          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası yapılması</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -4550,12 +4426,12 @@
       </c>
       <c r="B19" s="21" t="inlineStr">
         <is>
-          <t>15.540.1606</t>
+          <t>15.540.1537</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası</t>
+          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası yapılması</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -4564,7 +4440,7 @@
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>557.76</v>
+        <v>612.76</v>
       </c>
       <c r="F19" s="23">
         <f>IFERROR(VLOOKUP($B19,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4575,27 +4451,27 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
+    <row r="20" ht="14" customHeight="1">
       <c r="A20" s="3" t="n">
         <v>15</v>
       </c>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>15.540.1537</t>
+          <t>15.550.1202</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası</t>
+          <t>Lama ve profil demirlerden çeşitli demir işleri yapılması ve yerine konulması</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>557.76</v>
+        <v>674</v>
       </c>
       <c r="F20" s="23">
         <f>IFERROR(VLOOKUP($B20,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4612,12 +4488,12 @@
       </c>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>15.550.1202</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Lama ve profil demirlerden mahya, saçak ve köşe kapama profilleri</t>
+          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -4626,7 +4502,7 @@
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>674</v>
+        <v>319.2</v>
       </c>
       <c r="F21" s="23">
         <f>IFERROR(VLOOKUP($B21,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4643,21 +4519,21 @@
       </c>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>15.315.1001</t>
         </is>
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu yapılması — dere</t>
+          <t>Ø 70 mm çapında bir ucu muflu sert PVC yağmur borusu temini ve yerine tesbiti</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>319.2</v>
+        <v>51.2</v>
       </c>
       <c r="F22" s="23">
         <f>IFERROR(VLOOKUP($B22,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4668,27 +4544,27 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="14" customHeight="1">
+    <row r="23" ht="22" customHeight="1">
       <c r="A23" s="3" t="n">
         <v>18</v>
       </c>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>15.315.1001</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>Ø70 sert PVC yağmur suyu iniş borusu temini ve yerine tesbiti</t>
+          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>51.2</v>
+        <v>13.4</v>
       </c>
       <c r="F23" s="23">
         <f>IFERROR(VLOOKUP($B23,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4705,12 +4581,12 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>15.225.1004</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — kümes servis kapısı 100/220</t>
+          <t>10 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -4719,7 +4595,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>4.4</v>
+        <v>45</v>
       </c>
       <c r="F24" s="23">
         <f>IFERROR(VLOOKUP($B24,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4730,18 +4606,18 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
+    <row r="25" ht="33" customHeight="1">
       <c r="A25" s="3" t="n">
         <v>20</v>
       </c>
       <c r="B25" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>TKDK-0177</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu panel ile ısı yalıtımlı kapı yapılması — yükleme/temizlik kapısı 300/300 sürgülü</t>
+          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -4750,7 +4626,7 @@
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>9</v>
+        <v>60</v>
       </c>
       <c r="F25" s="23">
         <f>IFERROR(VLOOKUP($B25,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4767,12 +4643,12 @@
       </c>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>15.225.1004</t>
+          <t>TKDK-0175</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>10 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile bölme duvar yapılması — servis bölümü</t>
+          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -4781,7 +4657,7 @@
         </is>
       </c>
       <c r="E26" s="22" t="n">
-        <v>45</v>
+        <v>5.67</v>
       </c>
       <c r="F26" s="23">
         <f>IFERROR(VLOOKUP($B26,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4798,21 +4674,21 @@
       </c>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>15.275.1117</t>
+          <t>15.550.1002</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması — servis bölümü bölme duvarları</t>
+          <t>1,50 mm kalınlığında sıcak haddelenmiş sacdan bükme kapı kasası yapılması ve yerine konulması</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E27" s="22" t="n">
-        <v>90</v>
+        <v>54.315</v>
       </c>
       <c r="F27" s="23">
         <f>IFERROR(VLOOKUP($B27,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4823,27 +4699,27 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
+    <row r="28" ht="14" customHeight="1">
       <c r="A28" s="3" t="n">
         <v>23</v>
       </c>
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0177</t>
+          <t>43.527.1001</t>
         </is>
       </c>
       <c r="C28" s="18" t="inlineStr">
         <is>
-          <t>Duvar karosu ile 3 mm derz aralıklı döşeme ve duvar kaplaması yapılması — servis bölümü</t>
+          <t>Çapı 150 mm HDPE koruge boru döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E28" s="22" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="F28" s="23">
         <f>IFERROR(VLOOKUP($B28,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4860,21 +4736,21 @@
       </c>
       <c r="B29" s="21" t="inlineStr">
         <is>
-          <t>15.540.1537</t>
+          <t>30.100.2105</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel boya — servis bölümü</t>
+          <t>Kümes dağıtım panosu (sıva üstü galvanizli sac tablo, 0,40-0,50 m²) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E29" s="22" t="n">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="F29" s="23">
         <f>IFERROR(VLOOKUP($B29,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4891,21 +4767,21 @@
       </c>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0175</t>
+          <t>30.110.1102</t>
         </is>
       </c>
       <c r="C30" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı MDF presli iç kapı kanadı yapılması, yerinde takılması — servis bölümü</t>
+          <t>Termik-manyetik kompakt şalter 3x100 A, Icu 35 kA — kümes besleme (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E30" s="22" t="n">
-        <v>5.67</v>
+        <v>1</v>
       </c>
       <c r="F30" s="23">
         <f>IFERROR(VLOOKUP($B30,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4916,27 +4792,27 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="22" customHeight="1">
+    <row r="31" ht="14" customHeight="1">
       <c r="A31" s="3" t="n">
         <v>26</v>
       </c>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>15.550.1002</t>
+          <t>30.115.1003</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>1,50 mm sacdan bükme kapı kasası yapılması ve yerine konulması — servis bölümü iç kapıları</t>
+          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E31" s="22" t="n">
-        <v>54.315</v>
+        <v>2</v>
       </c>
       <c r="F31" s="23">
         <f>IFERROR(VLOOKUP($B31,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4953,12 +4829,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>30.140.3104</t>
         </is>
       </c>
       <c r="C32" s="18" t="inlineStr">
         <is>
-          <t>ø150 HDPE koruge boru ile pissu hattı döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>YVV (NYY) 1 kV yeraltı kablosu ile kolon hattı tesisi — 1x25 mm² (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -4967,7 +4843,7 @@
         </is>
       </c>
       <c r="E32" s="22" t="n">
-        <v>25</v>
+        <v>300</v>
       </c>
       <c r="F32" s="23">
         <f>IFERROR(VLOOKUP($B32,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4978,18 +4854,18 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="14" customHeight="1">
+    <row r="33" ht="22" customHeight="1">
       <c r="A33" s="3" t="n">
         <v>28</v>
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>30.100.2105</t>
+          <t>30.170.1602</t>
         </is>
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>Kümes dağıtım panosu (sıva üstü galvanizli sac tablo, 0,40-0,50 m²)</t>
+          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 2700 lm — kümes genel aydınlatması (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -4998,7 +4874,7 @@
         </is>
       </c>
       <c r="E33" s="22" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="F33" s="23">
         <f>IFERROR(VLOOKUP($B33,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5009,18 +4885,18 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="14" customHeight="1">
+    <row r="34" ht="22" customHeight="1">
       <c r="A34" s="3" t="n">
         <v>29</v>
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>30.110.1102</t>
+          <t>30.170.1601</t>
         </is>
       </c>
       <c r="C34" s="18" t="inlineStr">
         <is>
-          <t>Termik-manyetik kompakt şalter 3x100 A, Icu 35 kA — kümes besleme</t>
+          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 1800 lm — servis bölümü (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -5029,7 +4905,7 @@
         </is>
       </c>
       <c r="E34" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F34" s="23">
         <f>IFERROR(VLOOKUP($B34,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5046,21 +4922,21 @@
       </c>
       <c r="B35" s="21" t="inlineStr">
         <is>
-          <t>30.115.1003</t>
+          <t>30.160.6102</t>
         </is>
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>Kaçak akım koruma şalteri 2x63 A, 30 mA</t>
+          <t>Boş boru döşemesi — 25-32 mm PVC boru (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E35" s="22" t="n">
-        <v>2</v>
+        <v>500</v>
       </c>
       <c r="F35" s="23">
         <f>IFERROR(VLOOKUP($B35,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5077,12 +4953,12 @@
       </c>
       <c r="B36" s="21" t="inlineStr">
         <is>
-          <t>30.140.3104</t>
+          <t>30.150.1402</t>
         </is>
       </c>
       <c r="C36" s="18" t="inlineStr">
         <is>
-          <t>YVV (NYY) 1 kV yeraltı kablosu ile kolon hattı tesisi — 1x25 mm²</t>
+          <t>Halojensiz H07Z tipi iletken 1x2,5 mm² ile tesisat (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -5091,7 +4967,7 @@
         </is>
       </c>
       <c r="E36" s="22" t="n">
-        <v>300</v>
+        <v>2000</v>
       </c>
       <c r="F36" s="23">
         <f>IFERROR(VLOOKUP($B36,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5108,21 +4984,21 @@
       </c>
       <c r="B37" s="21" t="inlineStr">
         <is>
-          <t>30.170.1602</t>
+          <t>30.150.1401</t>
         </is>
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 2700 lm — kümes genel aydınlatması</t>
+          <t>Halojensiz H07Z tipi iletken 1x1,5 mm² ile kumanda tesisatı (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E37" s="22" t="n">
-        <v>30</v>
+        <v>600</v>
       </c>
       <c r="F37" s="23">
         <f>IFERROR(VLOOKUP($B37,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5139,21 +5015,21 @@
       </c>
       <c r="B38" s="21" t="inlineStr">
         <is>
-          <t>30.170.1601</t>
+          <t>30.140.1105</t>
         </is>
       </c>
       <c r="C38" s="18" t="inlineStr">
         <is>
-          <t>LED sıva üstü etanj armatür (polikarbon gövdeli), ışık akısı en az 1800 lm — servis bölümü</t>
+          <t>Çıplak bakır tel 25 mm² — eşpotansiyel bara ve topraklama iletkeni (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E38" s="22" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="F38" s="23">
         <f>IFERROR(VLOOKUP($B38,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5164,18 +5040,18 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="14" customHeight="1">
+    <row r="39" ht="22" customHeight="1">
       <c r="A39" s="3" t="n">
         <v>34</v>
       </c>
       <c r="B39" s="21" t="inlineStr">
         <is>
-          <t>30.160.6102</t>
+          <t>30.750.3002</t>
         </is>
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>Boş boru döşemesi — 25-32 mm PVC boru</t>
+          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -5184,7 +5060,7 @@
         </is>
       </c>
       <c r="E39" s="22" t="n">
-        <v>500</v>
+        <v>186</v>
       </c>
       <c r="F39" s="23">
         <f>IFERROR(VLOOKUP($B39,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5201,21 +5077,21 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>30.150.1402</t>
+          <t>30.750.1502</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
-          <t>Halojensiz H07Z tipi iletken 1x2,5 mm² ile tesisat</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E40" s="22" t="n">
-        <v>2000</v>
+        <v>1</v>
       </c>
       <c r="F40" s="23">
         <f>IFERROR(VLOOKUP($B40,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5226,18 +5102,18 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="14" customHeight="1">
+    <row r="41" ht="22" customHeight="1">
       <c r="A41" s="3" t="n">
         <v>36</v>
       </c>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>30.150.1401</t>
+          <t>30.750.2001</t>
         </is>
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>Halojensiz H07Z tipi iletken 1x1,5 mm² ile kumanda tesisatı</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -5246,7 +5122,7 @@
         </is>
       </c>
       <c r="E41" s="22" t="n">
-        <v>600</v>
+        <v>16</v>
       </c>
       <c r="F41" s="23">
         <f>IFERROR(VLOOKUP($B41,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5257,27 +5133,27 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="14" customHeight="1">
+    <row r="42" ht="22" customHeight="1">
       <c r="A42" s="3" t="n">
         <v>37</v>
       </c>
       <c r="B42" s="21" t="inlineStr">
         <is>
-          <t>30.140.1105</t>
+          <t>30.740.1106</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
         <is>
-          <t>Çıplak bakır tel 25 mm² — eşpotansiyel bara ve topraklama iletkeni</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E42" s="22" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F42" s="23">
         <f>IFERROR(VLOOKUP($B42,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5294,21 +5170,21 @@
       </c>
       <c r="B43" s="21" t="inlineStr">
         <is>
-          <t>30.750.3002</t>
+          <t>30.740.5406</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması)</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E43" s="22" t="n">
-        <v>186</v>
+        <v>1</v>
       </c>
       <c r="F43" s="23">
         <f>IFERROR(VLOOKUP($B43,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5319,27 +5195,27 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="14" customHeight="1">
+    <row r="44" ht="22" customHeight="1">
       <c r="A44" s="3" t="n">
         <v>39</v>
       </c>
       <c r="B44" s="21" t="inlineStr">
         <is>
-          <t>30.750.1502</t>
+          <t>35.190.1100</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m</t>
+          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E44" s="22" t="n">
-        <v>1</v>
+        <v>502</v>
       </c>
       <c r="F44" s="23">
         <f>IFERROR(VLOOKUP($B44,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5350,27 +5226,27 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="14" customHeight="1">
+    <row r="45" ht="22" customHeight="1">
       <c r="A45" s="3" t="n">
         <v>40</v>
       </c>
       <c r="B45" s="21" t="inlineStr">
         <is>
-          <t>30.750.2001</t>
+          <t>35.190.1100 (montaj)</t>
         </is>
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel</t>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E45" s="22" t="n">
-        <v>16</v>
+        <v>502</v>
       </c>
       <c r="F45" s="23">
         <f>IFERROR(VLOOKUP($B45,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5387,21 +5263,21 @@
       </c>
       <c r="B46" s="21" t="inlineStr">
         <is>
-          <t>30.740.1106</t>
+          <t>35.190.1101</t>
         </is>
       </c>
       <c r="C46" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak</t>
+          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E46" s="22" t="n">
-        <v>1</v>
+        <v>361.2</v>
       </c>
       <c r="F46" s="23">
         <f>IFERROR(VLOOKUP($B46,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5412,27 +5288,27 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="14" customHeight="1">
+    <row r="47" ht="22" customHeight="1">
       <c r="A47" s="3" t="n">
         <v>42</v>
       </c>
       <c r="B47" s="21" t="inlineStr">
         <is>
-          <t>30.740.5406</t>
+          <t>35.190.1101 (montaj)</t>
         </is>
       </c>
       <c r="C47" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA</t>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E47" s="22" t="n">
-        <v>1</v>
+        <v>361.2</v>
       </c>
       <c r="F47" s="23">
         <f>IFERROR(VLOOKUP($B47,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5449,21 +5325,21 @@
       </c>
       <c r="B48" s="21" t="inlineStr">
         <is>
-          <t>35.190.1100</t>
+          <t>30.190.1304</t>
         </is>
       </c>
       <c r="C48" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemi — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme)</t>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E48" s="22" t="n">
-        <v>502</v>
+        <v>123</v>
       </c>
       <c r="F48" s="23">
         <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5474,175 +5350,51 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="3" t="n">
-        <v>44</v>
-      </c>
-      <c r="B49" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1100 (montaj)</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E49" s="22" t="n">
-        <v>502</v>
-      </c>
-      <c r="F49" s="23">
-        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G49" s="5">
-        <f>ROUND(E49*F49,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="14" customHeight="1">
-      <c r="A50" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="B50" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101</t>
-        </is>
-      </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemi kapak sacı — 1,0 mm sıcak daldırma galvanizli (malzeme)</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E50" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F50" s="23">
-        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
+    <row r="49">
+      <c r="A49" s="7" t="n"/>
+      <c r="B49" s="7" t="n"/>
+      <c r="C49" s="24" t="inlineStr">
+        <is>
+          <t>ARA TOPLAM (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="n"/>
+      <c r="E49" s="7" t="n"/>
+      <c r="F49" s="7" t="n"/>
+      <c r="G49" s="9">
+        <f>SUM(G6:G48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n"/>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="25" t="inlineStr">
+        <is>
+          <t>KDV</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
       <c r="G50" s="5">
-        <f>ROUND(E50*F50,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="B51" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101 (montaj)</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E51" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F51" s="23">
-        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G51" s="5">
-        <f>ROUND(E51*F51,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" ht="14" customHeight="1">
-      <c r="A52" s="3" t="n">
-        <v>47</v>
-      </c>
-      <c r="B52" s="21" t="inlineStr">
-        <is>
-          <t>30.190.1304</t>
-        </is>
-      </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E52" s="22" t="n">
-        <v>123</v>
-      </c>
-      <c r="F52" s="23">
-        <f>IFERROR(VLOOKUP($B52,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G52" s="5">
-        <f>ROUND(E52*F52,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="7" t="n"/>
-      <c r="B53" s="7" t="n"/>
-      <c r="C53" s="24" t="inlineStr">
-        <is>
-          <t>ARA TOPLAM (KDV hariç)</t>
-        </is>
-      </c>
-      <c r="D53" s="7" t="n"/>
-      <c r="E53" s="7" t="n"/>
-      <c r="F53" s="7" t="n"/>
-      <c r="G53" s="9">
-        <f>SUM(G6:G52)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="n"/>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="25" t="inlineStr">
-        <is>
-          <t>KDV</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="5">
-        <f>G53*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="11" t="n"/>
-      <c r="B55" s="11" t="n"/>
-      <c r="C55" s="26" t="inlineStr">
+        <f>G49*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="n"/>
+      <c r="B51" s="11" t="n"/>
+      <c r="C51" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D55" s="11" t="n"/>
-      <c r="E55" s="11" t="n"/>
-      <c r="F55" s="11" t="n"/>
-      <c r="G55" s="13">
-        <f>G53+G54</f>
+      <c r="D51" s="11" t="n"/>
+      <c r="E51" s="11" t="n"/>
+      <c r="F51" s="11" t="n"/>
+      <c r="G51" s="13">
+        <f>G49+G50</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: iki blok eşitlendi, belge sırası keşif özetine sabitlendi
Kümes A = Kümes B = 7.887.227,25 TL. Keşif özeti, teklif sunum formu,
teklifler ve iki Excel satır satır örtüşüyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -2570,7 +2570,7 @@
         </is>
       </c>
       <c r="E6" s="22" t="n">
-        <v>1684.39</v>
+        <v>1684.385</v>
       </c>
       <c r="F6" s="23">
         <f>IFERROR(VLOOKUP($B6,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2798,27 +2798,27 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
+    <row r="14" ht="14" customHeight="1">
       <c r="A14" s="3" t="n">
         <v>9</v>
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>15.225.1010</t>
+          <t>15.550.1202</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>20 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
+          <t>Lama ve profil demirlerden çeşitli demir işleri yapılması ve yerine konulması</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E14" s="22" t="n">
-        <v>507.91</v>
+        <v>674</v>
       </c>
       <c r="F14" s="23">
         <f>IFERROR(VLOOKUP($B14,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2829,18 +2829,18 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="14" customHeight="1">
+    <row r="15" ht="22" customHeight="1">
       <c r="A15" s="3" t="n">
         <v>10</v>
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>15.225.1410</t>
+          <t>15.225.1010</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>20 cm kalınlığındaki teçhizatlı gazbeton lento temini ve yerine konulması</t>
+          <t>20 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -2849,7 +2849,7 @@
         </is>
       </c>
       <c r="E15" s="22" t="n">
-        <v>49.85</v>
+        <v>507.91</v>
       </c>
       <c r="F15" s="23">
         <f>IFERROR(VLOOKUP($B15,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2866,12 +2866,12 @@
       </c>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>15.275.1116</t>
+          <t>15.225.1410</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>250 kg çimento dozlu harç ile kaba sıva yapılması</t>
+          <t>20 cm kalınlığındaki teçhizatlı gazbeton lento temini ve yerine konulması</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -2880,7 +2880,7 @@
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>557.76</v>
+        <v>49.85</v>
       </c>
       <c r="F16" s="23">
         <f>IFERROR(VLOOKUP($B16,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2891,18 +2891,18 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="14" customHeight="1">
+    <row r="17" ht="22" customHeight="1">
       <c r="A17" s="3" t="n">
         <v>12</v>
       </c>
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>15.275.1117</t>
+          <t>15.225.1004</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması (iç cephe)</t>
+          <t>10 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -2911,7 +2911,7 @@
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>647.76</v>
+        <v>45</v>
       </c>
       <c r="F17" s="23">
         <f>IFERROR(VLOOKUP($B17,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2922,27 +2922,27 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
+    <row r="18" ht="14" customHeight="1">
       <c r="A18" s="3" t="n">
         <v>13</v>
       </c>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>15.540.1606</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası yapılması</t>
+          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>557.76</v>
+        <v>319.2</v>
       </c>
       <c r="F18" s="23">
         <f>IFERROR(VLOOKUP($B18,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2953,27 +2953,27 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
+    <row r="19" ht="14" customHeight="1">
       <c r="A19" s="3" t="n">
         <v>14</v>
       </c>
       <c r="B19" s="21" t="inlineStr">
         <is>
-          <t>15.540.1537</t>
+          <t>15.315.1001</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası yapılması</t>
+          <t>Ø 70 mm çapında bir ucu muflu sert PVC yağmur borusu temini ve yerine tesbiti</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>612.76</v>
+        <v>51.2</v>
       </c>
       <c r="F19" s="23">
         <f>IFERROR(VLOOKUP($B19,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -2984,27 +2984,27 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="14" customHeight="1">
+    <row r="20" ht="22" customHeight="1">
       <c r="A20" s="3" t="n">
         <v>15</v>
       </c>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>15.550.1202</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Lama ve profil demirlerden çeşitli demir işleri yapılması ve yerine konulması</t>
+          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>674</v>
+        <v>13.4</v>
       </c>
       <c r="F20" s="23">
         <f>IFERROR(VLOOKUP($B20,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3015,27 +3015,27 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="14" customHeight="1">
+    <row r="21" ht="22" customHeight="1">
       <c r="A21" s="3" t="n">
         <v>16</v>
       </c>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>TKDK-0175</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
+          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>319.2</v>
+        <v>5.67</v>
       </c>
       <c r="F21" s="23">
         <f>IFERROR(VLOOKUP($B21,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3046,27 +3046,27 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="14" customHeight="1">
+    <row r="22" ht="22" customHeight="1">
       <c r="A22" s="3" t="n">
         <v>17</v>
       </c>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>15.315.1001</t>
+          <t>15.550.1002</t>
         </is>
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>Ø 70 mm çapında bir ucu muflu sert PVC yağmur borusu temini ve yerine tesbiti</t>
+          <t>1,50 mm kalınlığında sıcak haddelenmiş sacdan bükme kapı kasası yapılması ve yerine konulması</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>51.2</v>
+        <v>54.315</v>
       </c>
       <c r="F22" s="23">
         <f>IFERROR(VLOOKUP($B22,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3077,18 +3077,18 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
+    <row r="23" ht="14" customHeight="1">
       <c r="A23" s="3" t="n">
         <v>18</v>
       </c>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>15.275.1116</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
+          <t>250 kg çimento dozlu harç ile kaba sıva yapılması</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -3097,7 +3097,7 @@
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>13.4</v>
+        <v>557.76</v>
       </c>
       <c r="F23" s="23">
         <f>IFERROR(VLOOKUP($B23,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3108,18 +3108,18 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1">
+    <row r="24" ht="14" customHeight="1">
       <c r="A24" s="3" t="n">
         <v>19</v>
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>15.225.1004</t>
+          <t>15.275.1117</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>10 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
+          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması (iç cephe)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -3128,7 +3128,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>45</v>
+        <v>647.76</v>
       </c>
       <c r="F24" s="23">
         <f>IFERROR(VLOOKUP($B24,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3139,18 +3139,18 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="33" customHeight="1">
+    <row r="25" ht="22" customHeight="1">
       <c r="A25" s="3" t="n">
         <v>20</v>
       </c>
       <c r="B25" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0177</t>
+          <t>15.540.1606</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
+          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası yapılması</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>60</v>
+        <v>557.76</v>
       </c>
       <c r="F25" s="23">
         <f>IFERROR(VLOOKUP($B25,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3176,12 +3176,12 @@
       </c>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0175</t>
+          <t>15.540.1537</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
+          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası yapılması</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -3190,7 +3190,7 @@
         </is>
       </c>
       <c r="E26" s="22" t="n">
-        <v>5.67</v>
+        <v>612.76</v>
       </c>
       <c r="F26" s="23">
         <f>IFERROR(VLOOKUP($B26,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3201,27 +3201,27 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="22" customHeight="1">
+    <row r="27" ht="33" customHeight="1">
       <c r="A27" s="3" t="n">
         <v>22</v>
       </c>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>15.550.1002</t>
+          <t>TKDK-0177</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>1,50 mm kalınlığında sıcak haddelenmiş sacdan bükme kapı kasası yapılması ve yerine konulması</t>
+          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E27" s="22" t="n">
-        <v>54.315</v>
+        <v>60</v>
       </c>
       <c r="F27" s="23">
         <f>IFERROR(VLOOKUP($B27,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="E6" s="22" t="n">
-        <v>1684.38</v>
+        <v>1684.385</v>
       </c>
       <c r="F6" s="23">
         <f>IFERROR(VLOOKUP($B6,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4265,27 +4265,27 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
+    <row r="14" ht="14" customHeight="1">
       <c r="A14" s="3" t="n">
         <v>9</v>
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>15.225.1010</t>
+          <t>15.550.1202</t>
         </is>
       </c>
       <c r="C14" s="18" t="inlineStr">
         <is>
-          <t>20 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
+          <t>Lama ve profil demirlerden çeşitli demir işleri yapılması ve yerine konulması</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E14" s="22" t="n">
-        <v>507.91</v>
+        <v>674</v>
       </c>
       <c r="F14" s="23">
         <f>IFERROR(VLOOKUP($B14,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4296,18 +4296,18 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="14" customHeight="1">
+    <row r="15" ht="22" customHeight="1">
       <c r="A15" s="3" t="n">
         <v>10</v>
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>15.225.1410</t>
+          <t>15.225.1010</t>
         </is>
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>20 cm kalınlığındaki teçhizatlı gazbeton lento temini ve yerine konulması</t>
+          <t>20 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -4316,7 +4316,7 @@
         </is>
       </c>
       <c r="E15" s="22" t="n">
-        <v>49.85</v>
+        <v>507.91</v>
       </c>
       <c r="F15" s="23">
         <f>IFERROR(VLOOKUP($B15,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4333,12 +4333,12 @@
       </c>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>15.275.1116</t>
+          <t>15.225.1410</t>
         </is>
       </c>
       <c r="C16" s="18" t="inlineStr">
         <is>
-          <t>250 kg çimento dozlu harç ile kaba sıva yapılması</t>
+          <t>20 cm kalınlığındaki teçhizatlı gazbeton lento temini ve yerine konulması</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -4347,7 +4347,7 @@
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>557.76</v>
+        <v>49.85</v>
       </c>
       <c r="F16" s="23">
         <f>IFERROR(VLOOKUP($B16,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4358,18 +4358,18 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="14" customHeight="1">
+    <row r="17" ht="22" customHeight="1">
       <c r="A17" s="3" t="n">
         <v>12</v>
       </c>
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>15.275.1117</t>
+          <t>15.225.1004</t>
         </is>
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması (iç cephe)</t>
+          <t>10 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -4378,7 +4378,7 @@
         </is>
       </c>
       <c r="E17" s="22" t="n">
-        <v>647.76</v>
+        <v>45</v>
       </c>
       <c r="F17" s="23">
         <f>IFERROR(VLOOKUP($B17,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4389,27 +4389,27 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
+    <row r="18" ht="14" customHeight="1">
       <c r="A18" s="3" t="n">
         <v>13</v>
       </c>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>15.540.1606</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="C18" s="18" t="inlineStr">
         <is>
-          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası yapılması</t>
+          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>557.76</v>
+        <v>319.2</v>
       </c>
       <c r="F18" s="23">
         <f>IFERROR(VLOOKUP($B18,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4420,27 +4420,27 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
+    <row r="19" ht="14" customHeight="1">
       <c r="A19" s="3" t="n">
         <v>14</v>
       </c>
       <c r="B19" s="21" t="inlineStr">
         <is>
-          <t>15.540.1537</t>
+          <t>15.315.1001</t>
         </is>
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası yapılması</t>
+          <t>Ø 70 mm çapında bir ucu muflu sert PVC yağmur borusu temini ve yerine tesbiti</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E19" s="22" t="n">
-        <v>612.76</v>
+        <v>51.2</v>
       </c>
       <c r="F19" s="23">
         <f>IFERROR(VLOOKUP($B19,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4451,27 +4451,27 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="14" customHeight="1">
+    <row r="20" ht="22" customHeight="1">
       <c r="A20" s="3" t="n">
         <v>15</v>
       </c>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>15.550.1202</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Lama ve profil demirlerden çeşitli demir işleri yapılması ve yerine konulması</t>
+          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>674</v>
+        <v>13.4</v>
       </c>
       <c r="F20" s="23">
         <f>IFERROR(VLOOKUP($B20,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4482,27 +4482,27 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="14" customHeight="1">
+    <row r="21" ht="22" customHeight="1">
       <c r="A21" s="3" t="n">
         <v>16</v>
       </c>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>TKDK-0175</t>
         </is>
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
+          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E21" s="22" t="n">
-        <v>319.2</v>
+        <v>5.67</v>
       </c>
       <c r="F21" s="23">
         <f>IFERROR(VLOOKUP($B21,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4513,27 +4513,27 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="14" customHeight="1">
+    <row r="22" ht="22" customHeight="1">
       <c r="A22" s="3" t="n">
         <v>17</v>
       </c>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>15.315.1001</t>
+          <t>15.550.1002</t>
         </is>
       </c>
       <c r="C22" s="18" t="inlineStr">
         <is>
-          <t>Ø 70 mm çapında bir ucu muflu sert PVC yağmur borusu temini ve yerine tesbiti</t>
+          <t>1,50 mm kalınlığında sıcak haddelenmiş sacdan bükme kapı kasası yapılması ve yerine konulması</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>51.2</v>
+        <v>54.315</v>
       </c>
       <c r="F22" s="23">
         <f>IFERROR(VLOOKUP($B22,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4544,18 +4544,18 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
+    <row r="23" ht="14" customHeight="1">
       <c r="A23" s="3" t="n">
         <v>18</v>
       </c>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>15.275.1116</t>
         </is>
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
+          <t>250 kg çimento dozlu harç ile kaba sıva yapılması</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -4564,7 +4564,7 @@
         </is>
       </c>
       <c r="E23" s="22" t="n">
-        <v>13.4</v>
+        <v>557.76</v>
       </c>
       <c r="F23" s="23">
         <f>IFERROR(VLOOKUP($B23,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4575,18 +4575,18 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1">
+    <row r="24" ht="14" customHeight="1">
       <c r="A24" s="3" t="n">
         <v>19</v>
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>15.225.1004</t>
+          <t>15.275.1117</t>
         </is>
       </c>
       <c r="C24" s="18" t="inlineStr">
         <is>
-          <t>10 cm kalınlığındaki teçhizatsız gazbeton duvar blokları ile duvar yapılması (gazbeton tutkalı ile)</t>
+          <t>200 kg çimento ve kireç karışımı harç ile kaba sıva yapılması (iç cephe)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -4595,7 +4595,7 @@
         </is>
       </c>
       <c r="E24" s="22" t="n">
-        <v>45</v>
+        <v>647.76</v>
       </c>
       <c r="F24" s="23">
         <f>IFERROR(VLOOKUP($B24,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4606,18 +4606,18 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="33" customHeight="1">
+    <row r="25" ht="22" customHeight="1">
       <c r="A25" s="3" t="n">
         <v>20</v>
       </c>
       <c r="B25" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0177</t>
+          <t>15.540.1606</t>
         </is>
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
+          <t>Brüt beton, sıvalı veya eski boyalı yüzeylere astar uygulanarak silikon esaslı su bazlı dış cephe boyası yapılması</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -4626,7 +4626,7 @@
         </is>
       </c>
       <c r="E25" s="22" t="n">
-        <v>60</v>
+        <v>557.76</v>
       </c>
       <c r="F25" s="23">
         <f>IFERROR(VLOOKUP($B25,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4643,12 +4643,12 @@
       </c>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>TKDK-0175</t>
+          <t>15.540.1537</t>
         </is>
       </c>
       <c r="C26" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
+          <t>Yeni sıva yüzeylere astar uygulanarak iki kat su bazlı plastik antibakteriyel iç cephe boyası yapılması</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -4657,7 +4657,7 @@
         </is>
       </c>
       <c r="E26" s="22" t="n">
-        <v>5.67</v>
+        <v>612.76</v>
       </c>
       <c r="F26" s="23">
         <f>IFERROR(VLOOKUP($B26,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4668,27 +4668,27 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="22" customHeight="1">
+    <row r="27" ht="33" customHeight="1">
       <c r="A27" s="3" t="n">
         <v>22</v>
       </c>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>15.550.1002</t>
+          <t>TKDK-0177</t>
         </is>
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>1,50 mm kalınlığında sıcak haddelenmiş sacdan bükme kapı kasası yapılması ve yerine konulması</t>
+          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E27" s="22" t="n">
-        <v>54.315</v>
+        <v>60</v>
       </c>
       <c r="F27" s="23">
         <f>IFERROR(VLOOKUP($B27,'Fiyatlar'!$A:$I,9,FALSE),0)</f>

</xml_diff>

<commit_message>
Yayın: elektrik pozları birim fiyat serisine (35.xxx) alındı
Uygun harcama 15.753.004,18 TL = 298.587 Avro; eşiğe kalan pay 1.413 Avro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>'01 Kümes A Blok'!$G$49</f>
+        <f>'01 Kümes A Blok'!$G$54</f>
         <v/>
       </c>
       <c r="D4" s="6">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>'02 Kümes B Blok'!$G$49</f>
+        <f>'02 Kümes B Blok'!$G$54</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1468,7 +1468,7 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>30.100.2105</t>
+          <t>35.100.2105</t>
         </is>
       </c>
       <c r="B24" s="18" t="inlineStr">
@@ -1508,7 +1508,7 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="17" t="inlineStr">
         <is>
-          <t>30.110.1102</t>
+          <t>35.110.1102</t>
         </is>
       </c>
       <c r="B25" s="18" t="inlineStr">
@@ -1548,7 +1548,7 @@
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="17" t="inlineStr">
         <is>
-          <t>30.115.1003</t>
+          <t>35.115.1003</t>
         </is>
       </c>
       <c r="B26" s="18" t="inlineStr">
@@ -1588,7 +1588,7 @@
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>30.140.1105</t>
+          <t>35.140.1105</t>
         </is>
       </c>
       <c r="B27" s="18" t="inlineStr">
@@ -1628,7 +1628,7 @@
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
         <is>
-          <t>30.140.3104</t>
+          <t>35.140.3104</t>
         </is>
       </c>
       <c r="B28" s="18" t="inlineStr">
@@ -1668,7 +1668,7 @@
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>30.150.1401</t>
+          <t>35.150.1401</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
@@ -1708,7 +1708,7 @@
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>30.150.1402</t>
+          <t>35.150.1402</t>
         </is>
       </c>
       <c r="B30" s="18" t="inlineStr">
@@ -1748,7 +1748,7 @@
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>30.160.6102</t>
+          <t>35.160.6102</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
@@ -1788,7 +1788,7 @@
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>30.170.1601</t>
+          <t>35.170.1601</t>
         </is>
       </c>
       <c r="B32" s="18" t="inlineStr">
@@ -1828,7 +1828,7 @@
     <row r="33" ht="33" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>30.170.1602</t>
+          <t>35.170.1602</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
@@ -1868,21 +1868,21 @@
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>30.190.1304</t>
+          <t>35.190.1100</t>
         </is>
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
-          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
+          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D34" s="5" t="n">
-        <v>277.71</v>
+        <v>237.4</v>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
@@ -1902,31 +1902,31 @@
         <v/>
       </c>
       <c r="I34" s="13" t="n">
-        <v>233.28</v>
+        <v>199.42</v>
       </c>
     </row>
     <row r="35" ht="33" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>30.740.1106</t>
+          <t>35.190.1100 (montaj)</t>
         </is>
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D35" s="5" t="n">
-        <v>556368.2</v>
+        <v>46.09</v>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>ÇŞB 35.190.1100 pozunun 01.06.2026 tarihli MONTAJ fiyatı 46,09 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 189,92 x 1,25 + montaj 46,09 = 283,49 TL</t>
         </is>
       </c>
       <c r="F35" s="20">
@@ -1942,27 +1942,27 @@
         <v/>
       </c>
       <c r="I35" s="13" t="n">
-        <v>467349.29</v>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
+        <v>38.72</v>
+      </c>
+    </row>
+    <row r="36" ht="33" customHeight="1">
       <c r="A36" s="17" t="inlineStr">
         <is>
-          <t>30.740.5406</t>
+          <t>35.190.1101</t>
         </is>
       </c>
       <c r="B36" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
+          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D36" s="5" t="n">
-        <v>94825.64999999999</v>
+        <v>193.3</v>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
@@ -1982,31 +1982,31 @@
         <v/>
       </c>
       <c r="I36" s="13" t="n">
-        <v>79653.55</v>
-      </c>
-    </row>
-    <row r="37" ht="22" customHeight="1">
+        <v>162.37</v>
+      </c>
+    </row>
+    <row r="37" ht="33" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>30.750.1502</t>
+          <t>35.190.1101 (montaj)</t>
         </is>
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>18566.2</v>
+        <v>25.36</v>
       </c>
       <c r="E37" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>ÇŞB 35.190.1101 pozunun 01.06.2026 tarihli MONTAJ fiyatı 25,36 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 154,64 x 1,25 + montaj 25,36 = 218,66 TL</t>
         </is>
       </c>
       <c r="F37" s="20">
@@ -2022,18 +2022,18 @@
         <v/>
       </c>
       <c r="I37" s="13" t="n">
-        <v>15595.61</v>
+        <v>21.3</v>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>30.750.2001</t>
+          <t>35.190.1304</t>
         </is>
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>508</v>
+        <v>277.71</v>
       </c>
       <c r="E38" s="19" t="inlineStr">
         <is>
@@ -2062,27 +2062,27 @@
         <v/>
       </c>
       <c r="I38" s="13" t="n">
-        <v>426.72</v>
-      </c>
-    </row>
-    <row r="39" ht="22" customHeight="1">
+        <v>233.28</v>
+      </c>
+    </row>
+    <row r="39" ht="33" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>30.750.3002</t>
+          <t>35.740.1106</t>
         </is>
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması) (%25 müteahhit kârı dahil)</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>138.05</v>
+        <v>504175</v>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
@@ -2102,31 +2102,31 @@
         <v/>
       </c>
       <c r="I39" s="13" t="n">
-        <v>115.96</v>
+        <v>423507</v>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>35.190.1100</t>
+          <t>35.740.1106 (montaj)</t>
         </is>
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
+          <t>Dizel elektrojen grubunun montajı — yerine konulması, bağlantıları ve işler hâlde teslimi</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>237.4</v>
+        <v>24847.84</v>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>ÇŞB 35.740.1106 pozunun 01.06.2026 tarihli MONTAJ fiyatı 24.847,84 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 403.340,00 x 1,25 + montaj 24.847,84 = 529.022,84 TL</t>
         </is>
       </c>
       <c r="F40" s="20">
@@ -2142,31 +2142,31 @@
         <v/>
       </c>
       <c r="I40" s="13" t="n">
-        <v>199.42</v>
-      </c>
-    </row>
-    <row r="41" ht="33" customHeight="1">
+        <v>20872.19</v>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>35.190.1100 (montaj)</t>
+          <t>35.740.5406</t>
         </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>46.09</v>
+        <v>85930</v>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 35.190.1100 pozunun 01.06.2026 tarihli MONTAJ fiyatı 46,09 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 189,92 x 1,25 + montaj 46,09 = 283,49 TL</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F41" s="20">
@@ -2182,31 +2182,31 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
-        <v>38.72</v>
-      </c>
-    </row>
-    <row r="42" ht="33" customHeight="1">
+        <v>72181.2</v>
+      </c>
+    </row>
+    <row r="42" ht="14" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>35.190.1101</t>
+          <t>35.740.5406 (montaj)</t>
         </is>
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
+          <t>Jeneratör ses izolasyon kabininin montajı</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>193.3</v>
+        <v>7391.38</v>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>ÇŞB 35.740.5406 pozunun 01.06.2026 tarihli MONTAJ fiyatı 7.391,38 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 68.744,00 x 1,25 + montaj 7.391,38 = 93.321,38 TL</t>
         </is>
       </c>
       <c r="F42" s="20">
@@ -2222,31 +2222,31 @@
         <v/>
       </c>
       <c r="I42" s="13" t="n">
-        <v>162.37</v>
-      </c>
-    </row>
-    <row r="43" ht="33" customHeight="1">
+        <v>6208.76</v>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>35.190.1101 (montaj)</t>
+          <t>35.750.1502</t>
         </is>
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>25.36</v>
+        <v>16824.5</v>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 35.190.1101 pozunun 01.06.2026 tarihli MONTAJ fiyatı 25,36 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 154,64 x 1,25 + montaj 25,36 = 218,66 TL</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F43" s="20">
@@ -2262,31 +2262,31 @@
         <v/>
       </c>
       <c r="I43" s="13" t="n">
-        <v>21.3</v>
+        <v>14132.58</v>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>43.527.1001</t>
+          <t>35.750.1502 (montaj)</t>
         </is>
       </c>
       <c r="B44" s="18" t="inlineStr">
         <is>
-          <t>Çapı 150 mm HDPE koruge boru döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+          <t>Aktif yakalama ucunun montajı — direk, taşıyıcı ve bağlantı elemanlarıyla yerine konulması</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>393.69</v>
+        <v>2537.5</v>
       </c>
       <c r="E44" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 35.750.1502 pozunun 01.06.2026 tarihli MONTAJ fiyatı 2.537,50 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 13.459,60 x 1,25 + montaj 2.537,50 = 19.362,00 TL</t>
         </is>
       </c>
       <c r="F44" s="20">
@@ -2302,31 +2302,31 @@
         <v/>
       </c>
       <c r="I44" s="13" t="n">
-        <v>330.7</v>
-      </c>
-    </row>
-    <row r="45" ht="14" customHeight="1">
+        <v>2131.5</v>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0115</t>
+          <t>35.750.2001</t>
         </is>
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>271.25</v>
+        <v>461.57</v>
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F45" s="20">
@@ -2342,31 +2342,31 @@
         <v/>
       </c>
       <c r="I45" s="13" t="n">
-        <v>227.85</v>
-      </c>
-    </row>
-    <row r="46" ht="33" customHeight="1">
+        <v>387.72</v>
+      </c>
+    </row>
+    <row r="46" ht="14" customHeight="1">
       <c r="A46" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0151</t>
+          <t>35.750.2001 (montaj)</t>
         </is>
       </c>
       <c r="B46" s="18" t="inlineStr">
         <is>
-          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatının montajı</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>1035.88</v>
+        <v>75.25</v>
       </c>
       <c r="E46" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 35.750.2001 pozunun 01.06.2026 tarihli MONTAJ fiyatı 75,25 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 369,26 x 1,25 + montaj 75,25 = 536,83 TL</t>
         </is>
       </c>
       <c r="F46" s="20">
@@ -2382,31 +2382,31 @@
         <v/>
       </c>
       <c r="I46" s="13" t="n">
-        <v>870.14</v>
-      </c>
-    </row>
-    <row r="47" ht="33" customHeight="1">
+        <v>63.21</v>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
       <c r="A47" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0175</t>
+          <t>35.750.3002</t>
         </is>
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
+          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>3199.68</v>
+        <v>125.44</v>
       </c>
       <c r="E47" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F47" s="20">
@@ -2422,31 +2422,31 @@
         <v/>
       </c>
       <c r="I47" s="13" t="n">
-        <v>2687.73</v>
-      </c>
-    </row>
-    <row r="48" ht="44" customHeight="1">
+        <v>105.37</v>
+      </c>
+    </row>
+    <row r="48" ht="14" customHeight="1">
       <c r="A48" s="17" t="inlineStr">
         <is>
-          <t>TKDK-0177</t>
+          <t>35.750.3002 (montaj)</t>
         </is>
       </c>
       <c r="B48" s="18" t="inlineStr">
         <is>
-          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
+          <t>Bina ihata iletkeni tesisatının montajı — temel topraklaması</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>835.1</v>
+        <v>92.31</v>
       </c>
       <c r="E48" s="19" t="inlineStr">
         <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+          <t>ÇŞB 35.750.3002 pozunun 01.06.2026 tarihli MONTAJ fiyatı 92,31 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 100,35 x 1,25 + montaj 92,31 = 217,75 TL</t>
         </is>
       </c>
       <c r="F48" s="20">
@@ -2462,6 +2462,206 @@
         <v/>
       </c>
       <c r="I48" s="13" t="n">
+        <v>77.54000000000001</v>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>43.527.1001</t>
+        </is>
+      </c>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>Çapı 150 mm HDPE koruge boru döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="n">
+        <v>393.69</v>
+      </c>
+      <c r="E49" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F49" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G49" s="5">
+        <f>D49*(1-F49)</f>
+        <v/>
+      </c>
+      <c r="H49" s="5">
+        <f>D49*$D$3</f>
+        <v/>
+      </c>
+      <c r="I49" s="13" t="n">
+        <v>330.7</v>
+      </c>
+    </row>
+    <row r="50" ht="14" customHeight="1">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0115</t>
+        </is>
+      </c>
+      <c r="B50" s="18" t="inlineStr">
+        <is>
+          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="n">
+        <v>271.25</v>
+      </c>
+      <c r="E50" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F50" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G50" s="5">
+        <f>D50*(1-F50)</f>
+        <v/>
+      </c>
+      <c r="H50" s="5">
+        <f>D50*$D$3</f>
+        <v/>
+      </c>
+      <c r="I50" s="13" t="n">
+        <v>227.85</v>
+      </c>
+    </row>
+    <row r="51" ht="33" customHeight="1">
+      <c r="A51" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0151</t>
+        </is>
+      </c>
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="n">
+        <v>1035.88</v>
+      </c>
+      <c r="E51" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F51" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G51" s="5">
+        <f>D51*(1-F51)</f>
+        <v/>
+      </c>
+      <c r="H51" s="5">
+        <f>D51*$D$3</f>
+        <v/>
+      </c>
+      <c r="I51" s="13" t="n">
+        <v>870.14</v>
+      </c>
+    </row>
+    <row r="52" ht="33" customHeight="1">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0175</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="n">
+        <v>3199.68</v>
+      </c>
+      <c r="E52" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F52" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G52" s="5">
+        <f>D52*(1-F52)</f>
+        <v/>
+      </c>
+      <c r="H52" s="5">
+        <f>D52*$D$3</f>
+        <v/>
+      </c>
+      <c r="I52" s="13" t="n">
+        <v>2687.73</v>
+      </c>
+    </row>
+    <row r="53" ht="44" customHeight="1">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>TKDK-0177</t>
+        </is>
+      </c>
+      <c r="B53" s="18" t="inlineStr">
+        <is>
+          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="n">
+        <v>835.1</v>
+      </c>
+      <c r="E53" s="19" t="inlineStr">
+        <is>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
+        </is>
+      </c>
+      <c r="F53" s="20">
+        <f>$B$3</f>
+        <v/>
+      </c>
+      <c r="G53" s="5">
+        <f>D53*(1-F53)</f>
+        <v/>
+      </c>
+      <c r="H53" s="5">
+        <f>D53*$D$3</f>
+        <v/>
+      </c>
+      <c r="I53" s="13" t="n">
         <v>701.48</v>
       </c>
     </row>
@@ -2480,7 +2680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3269,7 +3469,7 @@
       </c>
       <c r="B29" s="21" t="inlineStr">
         <is>
-          <t>30.100.2105</t>
+          <t>35.100.2105</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
@@ -3300,7 +3500,7 @@
       </c>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>30.110.1102</t>
+          <t>35.110.1102</t>
         </is>
       </c>
       <c r="C30" s="18" t="inlineStr">
@@ -3331,7 +3531,7 @@
       </c>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>30.115.1003</t>
+          <t>35.115.1003</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
@@ -3362,7 +3562,7 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>30.140.3104</t>
+          <t>35.140.3104</t>
         </is>
       </c>
       <c r="C32" s="18" t="inlineStr">
@@ -3393,7 +3593,7 @@
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>30.170.1602</t>
+          <t>35.170.1602</t>
         </is>
       </c>
       <c r="C33" s="18" t="inlineStr">
@@ -3424,7 +3624,7 @@
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>30.170.1601</t>
+          <t>35.170.1601</t>
         </is>
       </c>
       <c r="C34" s="18" t="inlineStr">
@@ -3455,7 +3655,7 @@
       </c>
       <c r="B35" s="21" t="inlineStr">
         <is>
-          <t>30.160.6102</t>
+          <t>35.160.6102</t>
         </is>
       </c>
       <c r="C35" s="18" t="inlineStr">
@@ -3486,7 +3686,7 @@
       </c>
       <c r="B36" s="21" t="inlineStr">
         <is>
-          <t>30.150.1402</t>
+          <t>35.150.1402</t>
         </is>
       </c>
       <c r="C36" s="18" t="inlineStr">
@@ -3517,7 +3717,7 @@
       </c>
       <c r="B37" s="21" t="inlineStr">
         <is>
-          <t>30.150.1401</t>
+          <t>35.150.1401</t>
         </is>
       </c>
       <c r="C37" s="18" t="inlineStr">
@@ -3548,7 +3748,7 @@
       </c>
       <c r="B38" s="21" t="inlineStr">
         <is>
-          <t>30.140.1105</t>
+          <t>35.140.1105</t>
         </is>
       </c>
       <c r="C38" s="18" t="inlineStr">
@@ -3579,7 +3779,7 @@
       </c>
       <c r="B39" s="21" t="inlineStr">
         <is>
-          <t>30.750.3002</t>
+          <t>35.750.3002</t>
         </is>
       </c>
       <c r="C39" s="18" t="inlineStr">
@@ -3610,21 +3810,21 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>30.750.1502</t>
+          <t>35.750.3002 (montaj)</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
+          <t>Bina ihata iletkeni tesisatının montajı — temel topraklaması</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E40" s="22" t="n">
-        <v>1</v>
+        <v>186</v>
       </c>
       <c r="F40" s="23">
         <f>IFERROR(VLOOKUP($B40,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3635,27 +3835,27 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1">
+    <row r="41" ht="14" customHeight="1">
       <c r="A41" s="3" t="n">
         <v>36</v>
       </c>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>30.750.2001</t>
+          <t>35.750.1502</t>
         </is>
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E41" s="22" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F41" s="23">
         <f>IFERROR(VLOOKUP($B41,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3672,12 +3872,12 @@
       </c>
       <c r="B42" s="21" t="inlineStr">
         <is>
-          <t>30.740.1106</t>
+          <t>35.750.1502 (montaj)</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
+          <t>Aktif yakalama ucunun montajı — direk, taşıyıcı ve bağlantı elemanlarıyla yerine konulması</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -3697,27 +3897,27 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="14" customHeight="1">
+    <row r="43" ht="22" customHeight="1">
       <c r="A43" s="3" t="n">
         <v>38</v>
       </c>
       <c r="B43" s="21" t="inlineStr">
         <is>
-          <t>30.740.5406</t>
+          <t>35.750.2001</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E43" s="22" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F43" s="23">
         <f>IFERROR(VLOOKUP($B43,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3728,27 +3928,27 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1">
+    <row r="44" ht="14" customHeight="1">
       <c r="A44" s="3" t="n">
         <v>39</v>
       </c>
       <c r="B44" s="21" t="inlineStr">
         <is>
-          <t>35.190.1100</t>
+          <t>35.750.2001 (montaj)</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatının montajı</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E44" s="22" t="n">
-        <v>502</v>
+        <v>16</v>
       </c>
       <c r="F44" s="23">
         <f>IFERROR(VLOOKUP($B44,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3765,21 +3965,21 @@
       </c>
       <c r="B45" s="21" t="inlineStr">
         <is>
-          <t>35.190.1100 (montaj)</t>
+          <t>35.740.1106</t>
         </is>
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E45" s="22" t="n">
-        <v>502</v>
+        <v>1</v>
       </c>
       <c r="F45" s="23">
         <f>IFERROR(VLOOKUP($B45,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3796,21 +3996,21 @@
       </c>
       <c r="B46" s="21" t="inlineStr">
         <is>
-          <t>35.190.1101</t>
+          <t>35.740.1106 (montaj)</t>
         </is>
       </c>
       <c r="C46" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
+          <t>Dizel elektrojen grubunun montajı — yerine konulması, bağlantıları ve işler hâlde teslimi</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E46" s="22" t="n">
-        <v>361.2</v>
+        <v>1</v>
       </c>
       <c r="F46" s="23">
         <f>IFERROR(VLOOKUP($B46,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3821,27 +4021,27 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
+    <row r="47" ht="14" customHeight="1">
       <c r="A47" s="3" t="n">
         <v>42</v>
       </c>
       <c r="B47" s="21" t="inlineStr">
         <is>
-          <t>35.190.1101 (montaj)</t>
+          <t>35.740.5406</t>
         </is>
       </c>
       <c r="C47" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E47" s="22" t="n">
-        <v>361.2</v>
+        <v>1</v>
       </c>
       <c r="F47" s="23">
         <f>IFERROR(VLOOKUP($B47,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3852,27 +4052,27 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1">
+    <row r="48" ht="14" customHeight="1">
       <c r="A48" s="3" t="n">
         <v>43</v>
       </c>
       <c r="B48" s="21" t="inlineStr">
         <is>
-          <t>30.190.1304</t>
+          <t>35.740.5406 (montaj)</t>
         </is>
       </c>
       <c r="C48" s="18" t="inlineStr">
         <is>
-          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
+          <t>Jeneratör ses izolasyon kabininin montajı</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E48" s="22" t="n">
-        <v>123</v>
+        <v>1</v>
       </c>
       <c r="F48" s="23">
         <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3883,51 +4083,206 @@
         <v/>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="7" t="n"/>
-      <c r="B49" s="7" t="n"/>
-      <c r="C49" s="24" t="inlineStr">
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F49" s="23">
+        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="5">
+        <f>ROUND(E49*F49,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100 (montaj)</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F50" s="23">
+        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="5">
+        <f>ROUND(E50*F50,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F51" s="23">
+        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="5">
+        <f>ROUND(E51*F51,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101 (montaj)</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E52" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F52" s="23">
+        <f>IFERROR(VLOOKUP($B52,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G52" s="5">
+        <f>ROUND(E52*F52,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1304</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E53" s="22" t="n">
+        <v>123</v>
+      </c>
+      <c r="F53" s="23">
+        <f>IFERROR(VLOOKUP($B53,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G53" s="5">
+        <f>ROUND(E53*F53,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="n"/>
+      <c r="B54" s="7" t="n"/>
+      <c r="C54" s="24" t="inlineStr">
         <is>
           <t>ARA TOPLAM (KDV hariç)</t>
         </is>
       </c>
-      <c r="D49" s="7" t="n"/>
-      <c r="E49" s="7" t="n"/>
-      <c r="F49" s="7" t="n"/>
-      <c r="G49" s="9">
-        <f>SUM(G6:G48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n"/>
-      <c r="B50" s="4" t="n"/>
-      <c r="C50" s="25" t="inlineStr">
+      <c r="D54" s="7" t="n"/>
+      <c r="E54" s="7" t="n"/>
+      <c r="F54" s="7" t="n"/>
+      <c r="G54" s="9">
+        <f>SUM(G6:G53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n"/>
+      <c r="B55" s="4" t="n"/>
+      <c r="C55" s="25" t="inlineStr">
         <is>
           <t>KDV</t>
         </is>
       </c>
-      <c r="D50" s="4" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="5">
-        <f>G49*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="11" t="n"/>
-      <c r="B51" s="11" t="n"/>
-      <c r="C51" s="26" t="inlineStr">
+      <c r="D55" s="4" t="n"/>
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="n"/>
+      <c r="G55" s="5">
+        <f>G54*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="n"/>
+      <c r="B56" s="11" t="n"/>
+      <c r="C56" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D51" s="11" t="n"/>
-      <c r="E51" s="11" t="n"/>
-      <c r="F51" s="11" t="n"/>
-      <c r="G51" s="13">
-        <f>G49+G50</f>
+      <c r="D56" s="11" t="n"/>
+      <c r="E56" s="11" t="n"/>
+      <c r="F56" s="11" t="n"/>
+      <c r="G56" s="13">
+        <f>G54+G55</f>
         <v/>
       </c>
     </row>
@@ -3947,7 +4302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4736,7 +5091,7 @@
       </c>
       <c r="B29" s="21" t="inlineStr">
         <is>
-          <t>30.100.2105</t>
+          <t>35.100.2105</t>
         </is>
       </c>
       <c r="C29" s="18" t="inlineStr">
@@ -4767,7 +5122,7 @@
       </c>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>30.110.1102</t>
+          <t>35.110.1102</t>
         </is>
       </c>
       <c r="C30" s="18" t="inlineStr">
@@ -4798,7 +5153,7 @@
       </c>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>30.115.1003</t>
+          <t>35.115.1003</t>
         </is>
       </c>
       <c r="C31" s="18" t="inlineStr">
@@ -4829,7 +5184,7 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>30.140.3104</t>
+          <t>35.140.3104</t>
         </is>
       </c>
       <c r="C32" s="18" t="inlineStr">
@@ -4860,7 +5215,7 @@
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>30.170.1602</t>
+          <t>35.170.1602</t>
         </is>
       </c>
       <c r="C33" s="18" t="inlineStr">
@@ -4891,7 +5246,7 @@
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>30.170.1601</t>
+          <t>35.170.1601</t>
         </is>
       </c>
       <c r="C34" s="18" t="inlineStr">
@@ -4922,7 +5277,7 @@
       </c>
       <c r="B35" s="21" t="inlineStr">
         <is>
-          <t>30.160.6102</t>
+          <t>35.160.6102</t>
         </is>
       </c>
       <c r="C35" s="18" t="inlineStr">
@@ -4953,7 +5308,7 @@
       </c>
       <c r="B36" s="21" t="inlineStr">
         <is>
-          <t>30.150.1402</t>
+          <t>35.150.1402</t>
         </is>
       </c>
       <c r="C36" s="18" t="inlineStr">
@@ -4984,7 +5339,7 @@
       </c>
       <c r="B37" s="21" t="inlineStr">
         <is>
-          <t>30.150.1401</t>
+          <t>35.150.1401</t>
         </is>
       </c>
       <c r="C37" s="18" t="inlineStr">
@@ -5015,7 +5370,7 @@
       </c>
       <c r="B38" s="21" t="inlineStr">
         <is>
-          <t>30.140.1105</t>
+          <t>35.140.1105</t>
         </is>
       </c>
       <c r="C38" s="18" t="inlineStr">
@@ -5046,7 +5401,7 @@
       </c>
       <c r="B39" s="21" t="inlineStr">
         <is>
-          <t>30.750.3002</t>
+          <t>35.750.3002</t>
         </is>
       </c>
       <c r="C39" s="18" t="inlineStr">
@@ -5077,21 +5432,21 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>30.750.1502</t>
+          <t>35.750.3002 (montaj)</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
+          <t>Bina ihata iletkeni tesisatının montajı — temel topraklaması</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E40" s="22" t="n">
-        <v>1</v>
+        <v>186</v>
       </c>
       <c r="F40" s="23">
         <f>IFERROR(VLOOKUP($B40,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5102,27 +5457,27 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="22" customHeight="1">
+    <row r="41" ht="14" customHeight="1">
       <c r="A41" s="3" t="n">
         <v>36</v>
       </c>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>30.750.2001</t>
+          <t>35.750.1502</t>
         </is>
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E41" s="22" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F41" s="23">
         <f>IFERROR(VLOOKUP($B41,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5139,12 +5494,12 @@
       </c>
       <c r="B42" s="21" t="inlineStr">
         <is>
-          <t>30.740.1106</t>
+          <t>35.750.1502 (montaj)</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
+          <t>Aktif yakalama ucunun montajı — direk, taşıyıcı ve bağlantı elemanlarıyla yerine konulması</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -5164,27 +5519,27 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="14" customHeight="1">
+    <row r="43" ht="22" customHeight="1">
       <c r="A43" s="3" t="n">
         <v>38</v>
       </c>
       <c r="B43" s="21" t="inlineStr">
         <is>
-          <t>30.740.5406</t>
+          <t>35.750.2001</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E43" s="22" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F43" s="23">
         <f>IFERROR(VLOOKUP($B43,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5195,27 +5550,27 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="22" customHeight="1">
+    <row r="44" ht="14" customHeight="1">
       <c r="A44" s="3" t="n">
         <v>39</v>
       </c>
       <c r="B44" s="21" t="inlineStr">
         <is>
-          <t>35.190.1100</t>
+          <t>35.750.2001 (montaj)</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatının montajı</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E44" s="22" t="n">
-        <v>502</v>
+        <v>16</v>
       </c>
       <c r="F44" s="23">
         <f>IFERROR(VLOOKUP($B44,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5232,21 +5587,21 @@
       </c>
       <c r="B45" s="21" t="inlineStr">
         <is>
-          <t>35.190.1100 (montaj)</t>
+          <t>35.740.1106</t>
         </is>
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E45" s="22" t="n">
-        <v>502</v>
+        <v>1</v>
       </c>
       <c r="F45" s="23">
         <f>IFERROR(VLOOKUP($B45,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5263,21 +5618,21 @@
       </c>
       <c r="B46" s="21" t="inlineStr">
         <is>
-          <t>35.190.1101</t>
+          <t>35.740.1106 (montaj)</t>
         </is>
       </c>
       <c r="C46" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
+          <t>Dizel elektrojen grubunun montajı — yerine konulması, bağlantıları ve işler hâlde teslimi</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E46" s="22" t="n">
-        <v>361.2</v>
+        <v>1</v>
       </c>
       <c r="F46" s="23">
         <f>IFERROR(VLOOKUP($B46,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5288,27 +5643,27 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="22" customHeight="1">
+    <row r="47" ht="14" customHeight="1">
       <c r="A47" s="3" t="n">
         <v>42</v>
       </c>
       <c r="B47" s="21" t="inlineStr">
         <is>
-          <t>35.190.1101 (montaj)</t>
+          <t>35.740.5406</t>
         </is>
       </c>
       <c r="C47" s="18" t="inlineStr">
         <is>
-          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E47" s="22" t="n">
-        <v>361.2</v>
+        <v>1</v>
       </c>
       <c r="F47" s="23">
         <f>IFERROR(VLOOKUP($B47,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5319,27 +5674,27 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="22" customHeight="1">
+    <row r="48" ht="14" customHeight="1">
       <c r="A48" s="3" t="n">
         <v>43</v>
       </c>
       <c r="B48" s="21" t="inlineStr">
         <is>
-          <t>30.190.1304</t>
+          <t>35.740.5406 (montaj)</t>
         </is>
       </c>
       <c r="C48" s="18" t="inlineStr">
         <is>
-          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
+          <t>Jeneratör ses izolasyon kabininin montajı</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E48" s="22" t="n">
-        <v>123</v>
+        <v>1</v>
       </c>
       <c r="F48" s="23">
         <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5350,51 +5705,206 @@
         <v/>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="7" t="n"/>
-      <c r="B49" s="7" t="n"/>
-      <c r="C49" s="24" t="inlineStr">
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100</t>
+        </is>
+      </c>
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F49" s="23">
+        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="5">
+        <f>ROUND(E49*F49,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1100 (montaj)</t>
+        </is>
+      </c>
+      <c r="C50" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="n">
+        <v>502</v>
+      </c>
+      <c r="F50" s="23">
+        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="5">
+        <f>ROUND(E50*F50,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101</t>
+        </is>
+      </c>
+      <c r="C51" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F51" s="23">
+        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="5">
+        <f>ROUND(E51*F51,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1101 (montaj)</t>
+        </is>
+      </c>
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E52" s="22" t="n">
+        <v>361.2</v>
+      </c>
+      <c r="F52" s="23">
+        <f>IFERROR(VLOOKUP($B52,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G52" s="5">
+        <f>ROUND(E52*F52,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" s="21" t="inlineStr">
+        <is>
+          <t>35.190.1304</t>
+        </is>
+      </c>
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E53" s="22" t="n">
+        <v>123</v>
+      </c>
+      <c r="F53" s="23">
+        <f>IFERROR(VLOOKUP($B53,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="G53" s="5">
+        <f>ROUND(E53*F53,2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="n"/>
+      <c r="B54" s="7" t="n"/>
+      <c r="C54" s="24" t="inlineStr">
         <is>
           <t>ARA TOPLAM (KDV hariç)</t>
         </is>
       </c>
-      <c r="D49" s="7" t="n"/>
-      <c r="E49" s="7" t="n"/>
-      <c r="F49" s="7" t="n"/>
-      <c r="G49" s="9">
-        <f>SUM(G6:G48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n"/>
-      <c r="B50" s="4" t="n"/>
-      <c r="C50" s="25" t="inlineStr">
+      <c r="D54" s="7" t="n"/>
+      <c r="E54" s="7" t="n"/>
+      <c r="F54" s="7" t="n"/>
+      <c r="G54" s="9">
+        <f>SUM(G6:G53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n"/>
+      <c r="B55" s="4" t="n"/>
+      <c r="C55" s="25" t="inlineStr">
         <is>
           <t>KDV</t>
         </is>
       </c>
-      <c r="D50" s="4" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="5">
-        <f>G49*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="11" t="n"/>
-      <c r="B51" s="11" t="n"/>
-      <c r="C51" s="26" t="inlineStr">
+      <c r="D55" s="4" t="n"/>
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="n"/>
+      <c r="G55" s="5">
+        <f>G54*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="11" t="n"/>
+      <c r="B56" s="11" t="n"/>
+      <c r="C56" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D51" s="11" t="n"/>
-      <c r="E51" s="11" t="n"/>
-      <c r="F51" s="11" t="n"/>
-      <c r="G51" s="13">
-        <f>G49+G50</f>
+      <c r="D56" s="11" t="n"/>
+      <c r="E56" s="11" t="n"/>
+      <c r="F56" s="11" t="n"/>
+      <c r="G56" s="13">
+        <f>G54+G55</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: elektrik pozları 35.xxx serisine geçti, tutar korundu
Uygun harcama 15.774.454,50 TL = 298.994 Avro, eşiğe kalan pay 1.006 Avro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/14_TEKLIFLER_MARFEN.xlsx
+++ b/belgeler/14_TEKLIFLER_MARFEN.xlsx
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="C4" s="5">
-        <f>'01 Kümes A Blok'!$G$54</f>
+        <f>'01 Kümes A Blok'!$G$49</f>
         <v/>
       </c>
       <c r="D4" s="6">
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>'02 Kümes B Blok'!$G$54</f>
+        <f>'02 Kümes B Blok'!$G$49</f>
         <v/>
       </c>
       <c r="D5" s="6">
@@ -644,7 +644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2082,7 +2082,7 @@
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>504175</v>
+        <v>556368.2</v>
       </c>
       <c r="E39" s="19" t="inlineStr">
         <is>
@@ -2102,18 +2102,18 @@
         <v/>
       </c>
       <c r="I39" s="13" t="n">
-        <v>423507</v>
+        <v>467349.29</v>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>35.740.1106 (montaj)</t>
+          <t>35.740.5406</t>
         </is>
       </c>
       <c r="B40" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubunun montajı — yerine konulması, bağlantıları ve işler hâlde teslimi</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2122,11 +2122,11 @@
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>24847.84</v>
+        <v>94825.64999999999</v>
       </c>
       <c r="E40" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 35.740.1106 pozunun 01.06.2026 tarihli MONTAJ fiyatı 24.847,84 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 403.340,00 x 1,25 + montaj 24.847,84 = 529.022,84 TL</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F40" s="20">
@@ -2142,18 +2142,18 @@
         <v/>
       </c>
       <c r="I40" s="13" t="n">
-        <v>20872.19</v>
+        <v>79653.55</v>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>35.740.5406</t>
+          <t>35.750.1502</t>
         </is>
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D41" s="5" t="n">
-        <v>85930</v>
+        <v>18566.2</v>
       </c>
       <c r="E41" s="19" t="inlineStr">
         <is>
@@ -2182,31 +2182,31 @@
         <v/>
       </c>
       <c r="I41" s="13" t="n">
-        <v>72181.2</v>
-      </c>
-    </row>
-    <row r="42" ht="14" customHeight="1">
+        <v>15595.61</v>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>35.740.5406 (montaj)</t>
+          <t>35.750.2001</t>
         </is>
       </c>
       <c r="B42" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabininin montajı</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D42" s="5" t="n">
-        <v>7391.38</v>
+        <v>508</v>
       </c>
       <c r="E42" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 35.740.5406 pozunun 01.06.2026 tarihli MONTAJ fiyatı 7.391,38 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 68.744,00 x 1,25 + montaj 7.391,38 = 93.321,38 TL</t>
+          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
         </is>
       </c>
       <c r="F42" s="20">
@@ -2222,27 +2222,27 @@
         <v/>
       </c>
       <c r="I42" s="13" t="n">
-        <v>6208.76</v>
+        <v>426.72</v>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>35.750.1502</t>
+          <t>35.750.3002</t>
         </is>
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
+          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D43" s="5" t="n">
-        <v>16824.5</v>
+        <v>138.05</v>
       </c>
       <c r="E43" s="19" t="inlineStr">
         <is>
@@ -2262,31 +2262,31 @@
         <v/>
       </c>
       <c r="I43" s="13" t="n">
-        <v>14132.58</v>
+        <v>115.96</v>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="17" t="inlineStr">
         <is>
-          <t>35.750.1502 (montaj)</t>
+          <t>43.527.1001</t>
         </is>
       </c>
       <c r="B44" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucunun montajı — direk, taşıyıcı ve bağlantı elemanlarıyla yerine konulması</t>
+          <t>Çapı 150 mm HDPE koruge boru döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D44" s="5" t="n">
-        <v>2537.5</v>
+        <v>393.69</v>
       </c>
       <c r="E44" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 35.750.1502 pozunun 01.06.2026 tarihli MONTAJ fiyatı 2.537,50 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 13.459,60 x 1,25 + montaj 2.537,50 = 19.362,00 TL</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F44" s="20">
@@ -2302,31 +2302,31 @@
         <v/>
       </c>
       <c r="I44" s="13" t="n">
-        <v>2131.5</v>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1">
+        <v>330.7</v>
+      </c>
+    </row>
+    <row r="45" ht="14" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>35.750.2001</t>
+          <t>TKDK-0115</t>
         </is>
       </c>
       <c r="B45" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
+          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="D45" s="5" t="n">
-        <v>461.57</v>
+        <v>271.25</v>
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F45" s="20">
@@ -2342,31 +2342,31 @@
         <v/>
       </c>
       <c r="I45" s="13" t="n">
-        <v>387.72</v>
-      </c>
-    </row>
-    <row r="46" ht="14" customHeight="1">
+        <v>227.85</v>
+      </c>
+    </row>
+    <row r="46" ht="33" customHeight="1">
       <c r="A46" s="17" t="inlineStr">
         <is>
-          <t>35.750.2001 (montaj)</t>
+          <t>TKDK-0151</t>
         </is>
       </c>
       <c r="B46" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatının montajı</t>
+          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D46" s="5" t="n">
-        <v>75.25</v>
+        <v>1035.88</v>
       </c>
       <c r="E46" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 35.750.2001 pozunun 01.06.2026 tarihli MONTAJ fiyatı 75,25 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 369,26 x 1,25 + montaj 75,25 = 536,83 TL</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F46" s="20">
@@ -2382,31 +2382,31 @@
         <v/>
       </c>
       <c r="I46" s="13" t="n">
-        <v>63.21</v>
-      </c>
-    </row>
-    <row r="47" ht="22" customHeight="1">
+        <v>870.14</v>
+      </c>
+    </row>
+    <row r="47" ht="33" customHeight="1">
       <c r="A47" s="17" t="inlineStr">
         <is>
-          <t>35.750.3002</t>
+          <t>TKDK-0175</t>
         </is>
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatı — 30x3,5 mm galvanizli çelik lama (temel topraklaması) (%25 müteahhit kârı dahil)</t>
+          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D47" s="5" t="n">
-        <v>125.44</v>
+        <v>3199.68</v>
       </c>
       <c r="E47" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 2026 Haziran elektrik rayici x 1,25</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F47" s="20">
@@ -2422,31 +2422,31 @@
         <v/>
       </c>
       <c r="I47" s="13" t="n">
-        <v>105.37</v>
-      </c>
-    </row>
-    <row r="48" ht="14" customHeight="1">
+        <v>2687.73</v>
+      </c>
+    </row>
+    <row r="48" ht="44" customHeight="1">
       <c r="A48" s="17" t="inlineStr">
         <is>
-          <t>35.750.3002 (montaj)</t>
+          <t>TKDK-0177</t>
         </is>
       </c>
       <c r="B48" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatının montajı — temel topraklaması</t>
+          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D48" s="5" t="n">
-        <v>92.31</v>
+        <v>835.1</v>
       </c>
       <c r="E48" s="19" t="inlineStr">
         <is>
-          <t>ÇŞB 35.750.3002 pozunun 01.06.2026 tarihli MONTAJ fiyatı 92,31 TL; kitabın kendi rakamıdır, kâr ve genel gider içindedir, ayrıca çarpılmamıştır. Kitabın birim fiyatı = malzeme 100,35 x 1,25 + montaj 92,31 = 217,75 TL</t>
+          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
         </is>
       </c>
       <c r="F48" s="20">
@@ -2462,206 +2462,6 @@
         <v/>
       </c>
       <c r="I48" s="13" t="n">
-        <v>77.54000000000001</v>
-      </c>
-    </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="17" t="inlineStr">
-        <is>
-          <t>43.527.1001</t>
-        </is>
-      </c>
-      <c r="B49" s="18" t="inlineStr">
-        <is>
-          <t>Çapı 150 mm HDPE koruge boru döşenmesi (SN 8, lastik conta ve boru bedeli dahil)</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="n">
-        <v>393.69</v>
-      </c>
-      <c r="E49" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F49" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G49" s="5">
-        <f>D49*(1-F49)</f>
-        <v/>
-      </c>
-      <c r="H49" s="5">
-        <f>D49*$D$3</f>
-        <v/>
-      </c>
-      <c r="I49" s="13" t="n">
-        <v>330.7</v>
-      </c>
-    </row>
-    <row r="50" ht="14" customHeight="1">
-      <c r="A50" s="17" t="inlineStr">
-        <is>
-          <t>TKDK-0115</t>
-        </is>
-      </c>
-      <c r="B50" s="18" t="inlineStr">
-        <is>
-          <t>Galvanizli düz sacdan yağmur oluğu veya iniş borusu yapılması</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="n">
-        <v>271.25</v>
-      </c>
-      <c r="E50" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F50" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G50" s="5">
-        <f>D50*(1-F50)</f>
-        <v/>
-      </c>
-      <c r="H50" s="5">
-        <f>D50*$D$3</f>
-        <v/>
-      </c>
-      <c r="I50" s="13" t="n">
-        <v>227.85</v>
-      </c>
-    </row>
-    <row r="51" ht="33" customHeight="1">
-      <c r="A51" s="17" t="inlineStr">
-        <is>
-          <t>TKDK-0151</t>
-        </is>
-      </c>
-      <c r="B51" s="18" t="inlineStr">
-        <is>
-          <t>5 cm poliüretan dolgulu (üst 0,50 mm düz, alt 0,40 mm düz) fabrikasyon rulo boyama sistemi ile boyanmış galvaniz levhalar ile ısı yalıtımlı kapı yapılması</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="n">
-        <v>1035.88</v>
-      </c>
-      <c r="E51" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F51" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G51" s="5">
-        <f>D51*(1-F51)</f>
-        <v/>
-      </c>
-      <c r="H51" s="5">
-        <f>D51*$D$3</f>
-        <v/>
-      </c>
-      <c r="I51" s="13" t="n">
-        <v>870.14</v>
-      </c>
-    </row>
-    <row r="52" ht="33" customHeight="1">
-      <c r="A52" s="17" t="inlineStr">
-        <is>
-          <t>TKDK-0175</t>
-        </is>
-      </c>
-      <c r="B52" s="18" t="inlineStr">
-        <is>
-          <t>PVC kaplamalı, iki yüzü odun lifinden yapılmış levhalarla (MDF) presli, kraft dolgulu iç kapı kanadı yapılması, yerinde takılması</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D52" s="5" t="n">
-        <v>3199.68</v>
-      </c>
-      <c r="E52" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F52" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G52" s="5">
-        <f>D52*(1-F52)</f>
-        <v/>
-      </c>
-      <c r="H52" s="5">
-        <f>D52*$D$3</f>
-        <v/>
-      </c>
-      <c r="I52" s="13" t="n">
-        <v>2687.73</v>
-      </c>
-    </row>
-    <row r="53" ht="44" customHeight="1">
-      <c r="A53" s="17" t="inlineStr">
-        <is>
-          <t>TKDK-0177</t>
-        </is>
-      </c>
-      <c r="B53" s="18" t="inlineStr">
-        <is>
-          <t>(25x70 - 25x75 - 40x80 cm) anma ebatlarında, her türlü desen ve yüzey özelliğinde, renkli duvar karosu ile 3 mm derz aralıklı döşeme, duvar ve cephe kaplaması yapılması (karo yapıştırıcısı ile)</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="n">
-        <v>835.1</v>
-      </c>
-      <c r="E53" s="19" t="inlineStr">
-        <is>
-          <t>TKDK 17.02.2026 Özel Poz Tablosu</t>
-        </is>
-      </c>
-      <c r="F53" s="20">
-        <f>$B$3</f>
-        <v/>
-      </c>
-      <c r="G53" s="5">
-        <f>D53*(1-F53)</f>
-        <v/>
-      </c>
-      <c r="H53" s="5">
-        <f>D53*$D$3</f>
-        <v/>
-      </c>
-      <c r="I53" s="13" t="n">
         <v>701.48</v>
       </c>
     </row>
@@ -2680,7 +2480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3810,21 +3610,21 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>35.750.3002 (montaj)</t>
+          <t>35.750.1502</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatının montajı — temel topraklaması</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E40" s="22" t="n">
-        <v>186</v>
+        <v>1</v>
       </c>
       <c r="F40" s="23">
         <f>IFERROR(VLOOKUP($B40,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3835,27 +3635,27 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="14" customHeight="1">
+    <row r="41" ht="22" customHeight="1">
       <c r="A41" s="3" t="n">
         <v>36</v>
       </c>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>35.750.1502</t>
+          <t>35.750.2001</t>
         </is>
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E41" s="22" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F41" s="23">
         <f>IFERROR(VLOOKUP($B41,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3872,12 +3672,12 @@
       </c>
       <c r="B42" s="21" t="inlineStr">
         <is>
-          <t>35.750.1502 (montaj)</t>
+          <t>35.740.1106</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucunun montajı — direk, taşıyıcı ve bağlantı elemanlarıyla yerine konulması</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -3897,27 +3697,27 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="22" customHeight="1">
+    <row r="43" ht="14" customHeight="1">
       <c r="A43" s="3" t="n">
         <v>38</v>
       </c>
       <c r="B43" s="21" t="inlineStr">
         <is>
-          <t>35.750.2001</t>
+          <t>35.740.5406</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E43" s="22" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F43" s="23">
         <f>IFERROR(VLOOKUP($B43,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3928,27 +3728,27 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="14" customHeight="1">
+    <row r="44" ht="22" customHeight="1">
       <c r="A44" s="3" t="n">
         <v>39</v>
       </c>
       <c r="B44" s="21" t="inlineStr">
         <is>
-          <t>35.750.2001 (montaj)</t>
+          <t>35.190.1100</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatının montajı</t>
+          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E44" s="22" t="n">
-        <v>16</v>
+        <v>502</v>
       </c>
       <c r="F44" s="23">
         <f>IFERROR(VLOOKUP($B44,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3965,21 +3765,21 @@
       </c>
       <c r="B45" s="21" t="inlineStr">
         <is>
-          <t>35.740.1106</t>
+          <t>35.190.1100 (montaj)</t>
         </is>
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E45" s="22" t="n">
-        <v>1</v>
+        <v>502</v>
       </c>
       <c r="F45" s="23">
         <f>IFERROR(VLOOKUP($B45,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -3996,21 +3796,21 @@
       </c>
       <c r="B46" s="21" t="inlineStr">
         <is>
-          <t>35.740.1106 (montaj)</t>
+          <t>35.190.1101</t>
         </is>
       </c>
       <c r="C46" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubunun montajı — yerine konulması, bağlantıları ve işler hâlde teslimi</t>
+          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E46" s="22" t="n">
-        <v>1</v>
+        <v>361.2</v>
       </c>
       <c r="F46" s="23">
         <f>IFERROR(VLOOKUP($B46,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4021,27 +3821,27 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="14" customHeight="1">
+    <row r="47" ht="22" customHeight="1">
       <c r="A47" s="3" t="n">
         <v>42</v>
       </c>
       <c r="B47" s="21" t="inlineStr">
         <is>
-          <t>35.740.5406</t>
+          <t>35.190.1101 (montaj)</t>
         </is>
       </c>
       <c r="C47" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E47" s="22" t="n">
-        <v>1</v>
+        <v>361.2</v>
       </c>
       <c r="F47" s="23">
         <f>IFERROR(VLOOKUP($B47,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4052,27 +3852,27 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="14" customHeight="1">
+    <row r="48" ht="22" customHeight="1">
       <c r="A48" s="3" t="n">
         <v>43</v>
       </c>
       <c r="B48" s="21" t="inlineStr">
         <is>
-          <t>35.740.5406 (montaj)</t>
+          <t>35.190.1304</t>
         </is>
       </c>
       <c r="C48" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabininin montajı</t>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E48" s="22" t="n">
-        <v>1</v>
+        <v>123</v>
       </c>
       <c r="F48" s="23">
         <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -4083,206 +3883,51 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="3" t="n">
-        <v>44</v>
-      </c>
-      <c r="B49" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1100</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E49" s="22" t="n">
-        <v>502</v>
-      </c>
-      <c r="F49" s="23">
-        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G49" s="5">
-        <f>ROUND(E49*F49,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="B50" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1100 (montaj)</t>
-        </is>
-      </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E50" s="22" t="n">
-        <v>502</v>
-      </c>
-      <c r="F50" s="23">
-        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
+    <row r="49">
+      <c r="A49" s="7" t="n"/>
+      <c r="B49" s="7" t="n"/>
+      <c r="C49" s="24" t="inlineStr">
+        <is>
+          <t>ARA TOPLAM (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="n"/>
+      <c r="E49" s="7" t="n"/>
+      <c r="F49" s="7" t="n"/>
+      <c r="G49" s="9">
+        <f>SUM(G6:G48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n"/>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="25" t="inlineStr">
+        <is>
+          <t>KDV</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
       <c r="G50" s="5">
-        <f>ROUND(E50*F50,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="B51" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E51" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F51" s="23">
-        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G51" s="5">
-        <f>ROUND(E51*F51,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="3" t="n">
-        <v>47</v>
-      </c>
-      <c r="B52" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101 (montaj)</t>
-        </is>
-      </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E52" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F52" s="23">
-        <f>IFERROR(VLOOKUP($B52,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G52" s="5">
-        <f>ROUND(E52*F52,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="B53" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1304</t>
-        </is>
-      </c>
-      <c r="C53" s="18" t="inlineStr">
-        <is>
-          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E53" s="22" t="n">
-        <v>123</v>
-      </c>
-      <c r="F53" s="23">
-        <f>IFERROR(VLOOKUP($B53,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G53" s="5">
-        <f>ROUND(E53*F53,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="n"/>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="24" t="inlineStr">
-        <is>
-          <t>ARA TOPLAM (KDV hariç)</t>
-        </is>
-      </c>
-      <c r="D54" s="7" t="n"/>
-      <c r="E54" s="7" t="n"/>
-      <c r="F54" s="7" t="n"/>
-      <c r="G54" s="9">
-        <f>SUM(G6:G53)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="n"/>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="25" t="inlineStr">
-        <is>
-          <t>KDV</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="5">
-        <f>G54*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="11" t="n"/>
-      <c r="B56" s="11" t="n"/>
-      <c r="C56" s="26" t="inlineStr">
+        <f>G49*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="n"/>
+      <c r="B51" s="11" t="n"/>
+      <c r="C51" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D56" s="11" t="n"/>
-      <c r="E56" s="11" t="n"/>
-      <c r="F56" s="11" t="n"/>
-      <c r="G56" s="13">
-        <f>G54+G55</f>
+      <c r="D51" s="11" t="n"/>
+      <c r="E51" s="11" t="n"/>
+      <c r="F51" s="11" t="n"/>
+      <c r="G51" s="13">
+        <f>G49+G50</f>
         <v/>
       </c>
     </row>
@@ -4302,7 +3947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5432,21 +5077,21 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>35.750.3002 (montaj)</t>
+          <t>35.750.1502</t>
         </is>
       </c>
       <c r="C40" s="18" t="inlineStr">
         <is>
-          <t>Bina ihata iletkeni tesisatının montajı — temel topraklaması</t>
+          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E40" s="22" t="n">
-        <v>186</v>
+        <v>1</v>
       </c>
       <c r="F40" s="23">
         <f>IFERROR(VLOOKUP($B40,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5457,27 +5102,27 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="14" customHeight="1">
+    <row r="41" ht="22" customHeight="1">
       <c r="A41" s="3" t="n">
         <v>36</v>
       </c>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>35.750.1502</t>
+          <t>35.750.2001</t>
         </is>
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucu, ortalama uyarım yolu DL = 30-40 m (%25 müteahhit kârı dahil)</t>
+          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E41" s="22" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="F41" s="23">
         <f>IFERROR(VLOOKUP($B41,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5494,12 +5139,12 @@
       </c>
       <c r="B42" s="21" t="inlineStr">
         <is>
-          <t>35.750.1502 (montaj)</t>
+          <t>35.740.1106</t>
         </is>
       </c>
       <c r="C42" s="18" t="inlineStr">
         <is>
-          <t>Aktif yakalama ucunun montajı — direk, taşıyıcı ve bağlantı elemanlarıyla yerine konulması</t>
+          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -5519,27 +5164,27 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="22" customHeight="1">
+    <row r="43" ht="14" customHeight="1">
       <c r="A43" s="3" t="n">
         <v>38</v>
       </c>
       <c r="B43" s="21" t="inlineStr">
         <is>
-          <t>35.750.2001</t>
+          <t>35.740.5406</t>
         </is>
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatı — 50 mm² elektrolitik bakır tel (%25 müteahhit kârı dahil)</t>
+          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ad</t>
         </is>
       </c>
       <c r="E43" s="22" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F43" s="23">
         <f>IFERROR(VLOOKUP($B43,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5550,27 +5195,27 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="14" customHeight="1">
+    <row r="44" ht="22" customHeight="1">
       <c r="A44" s="3" t="n">
         <v>39</v>
       </c>
       <c r="B44" s="21" t="inlineStr">
         <is>
-          <t>35.750.2001 (montaj)</t>
+          <t>35.190.1100</t>
         </is>
       </c>
       <c r="C44" s="18" t="inlineStr">
         <is>
-          <t>Çatı ihata ve indirme iletkeni tesisatının montajı</t>
+          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E44" s="22" t="n">
-        <v>16</v>
+        <v>502</v>
       </c>
       <c r="F44" s="23">
         <f>IFERROR(VLOOKUP($B44,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5587,21 +5232,21 @@
       </c>
       <c r="B45" s="21" t="inlineStr">
         <is>
-          <t>35.740.1106</t>
+          <t>35.190.1100 (montaj)</t>
         </is>
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubu (jeneratör) 63 kVA / 50 kW — dizel motoru su veya hava ile soğuyan cinsten, 1500 d/dak (%25 müteahhit kârı dahil)</t>
+          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E45" s="22" t="n">
-        <v>1</v>
+        <v>502</v>
       </c>
       <c r="F45" s="23">
         <f>IFERROR(VLOOKUP($B45,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5618,21 +5263,21 @@
       </c>
       <c r="B46" s="21" t="inlineStr">
         <is>
-          <t>35.740.1106 (montaj)</t>
+          <t>35.190.1101</t>
         </is>
       </c>
       <c r="C46" s="18" t="inlineStr">
         <is>
-          <t>Dizel elektrojen grubunun montajı — yerine konulması, bağlantıları ve işler hâlde teslimi</t>
+          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E46" s="22" t="n">
-        <v>1</v>
+        <v>361.2</v>
       </c>
       <c r="F46" s="23">
         <f>IFERROR(VLOOKUP($B46,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5643,27 +5288,27 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="14" customHeight="1">
+    <row r="47" ht="22" customHeight="1">
       <c r="A47" s="3" t="n">
         <v>42</v>
       </c>
       <c r="B47" s="21" t="inlineStr">
         <is>
-          <t>35.740.5406</t>
+          <t>35.190.1101 (montaj)</t>
         </is>
       </c>
       <c r="C47" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabini — 63 kVA (%25 müteahhit kârı dahil)</t>
+          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E47" s="22" t="n">
-        <v>1</v>
+        <v>361.2</v>
       </c>
       <c r="F47" s="23">
         <f>IFERROR(VLOOKUP($B47,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5674,27 +5319,27 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="14" customHeight="1">
+    <row r="48" ht="22" customHeight="1">
       <c r="A48" s="3" t="n">
         <v>43</v>
       </c>
       <c r="B48" s="21" t="inlineStr">
         <is>
-          <t>35.740.5406 (montaj)</t>
+          <t>35.190.1304</t>
         </is>
       </c>
       <c r="C48" s="18" t="inlineStr">
         <is>
-          <t>Jeneratör ses izolasyon kabininin montajı</t>
+          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E48" s="22" t="n">
-        <v>1</v>
+        <v>123</v>
       </c>
       <c r="F48" s="23">
         <f>IFERROR(VLOOKUP($B48,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
@@ -5705,206 +5350,51 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="3" t="n">
-        <v>44</v>
-      </c>
-      <c r="B49" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1100</t>
-        </is>
-      </c>
-      <c r="C49" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemleri — 200x60x1,0 mm sıcak daldırma galvanizli perfore kablo tavası (malzeme) (%25 müteahhit kârı dahil)</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E49" s="22" t="n">
-        <v>502</v>
-      </c>
-      <c r="F49" s="23">
-        <f>IFERROR(VLOOKUP($B49,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G49" s="5">
-        <f>ROUND(E49*F49,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1">
-      <c r="A50" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="B50" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1100 (montaj)</t>
-        </is>
-      </c>
-      <c r="C50" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemlerinin montajı — askı ve konsollarla tavana veya duvara tespiti; ek parça, konsol, askı tiji, vida ve somun bedelleri dâhildir, ayrıca ödenmez</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E50" s="22" t="n">
-        <v>502</v>
-      </c>
-      <c r="F50" s="23">
-        <f>IFERROR(VLOOKUP($B50,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
+    <row r="49">
+      <c r="A49" s="7" t="n"/>
+      <c r="B49" s="7" t="n"/>
+      <c r="C49" s="24" t="inlineStr">
+        <is>
+          <t>ARA TOPLAM (KDV hariç)</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="n"/>
+      <c r="E49" s="7" t="n"/>
+      <c r="F49" s="7" t="n"/>
+      <c r="G49" s="9">
+        <f>SUM(G6:G48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n"/>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="25" t="inlineStr">
+        <is>
+          <t>KDV</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="n"/>
+      <c r="F50" s="4" t="n"/>
       <c r="G50" s="5">
-        <f>ROUND(E50*F50,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1">
-      <c r="A51" s="3" t="n">
-        <v>46</v>
-      </c>
-      <c r="B51" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101</t>
-        </is>
-      </c>
-      <c r="C51" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemleri kapak sacı — 35.190.1100 pozuna uygun özellikte, 1,0 mm sıcak daldırma galvanizli (malzeme) (%25 müteahhit kârı dahil)</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E51" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F51" s="23">
-        <f>IFERROR(VLOOKUP($B51,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G51" s="5">
-        <f>ROUND(E51*F51,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" ht="22" customHeight="1">
-      <c r="A52" s="3" t="n">
-        <v>47</v>
-      </c>
-      <c r="B52" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1101 (montaj)</t>
-        </is>
-      </c>
-      <c r="C52" s="18" t="inlineStr">
-        <is>
-          <t>Kablo tava sistemleri kapak sacının montajı — onaylı projesinde belirtilen kanalların kapatılması; her türlü işçilik ve malzeme dâhil, işler hâlde teslim</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E52" s="22" t="n">
-        <v>361.2</v>
-      </c>
-      <c r="F52" s="23">
-        <f>IFERROR(VLOOKUP($B52,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G52" s="5">
-        <f>ROUND(E52*F52,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53" ht="22" customHeight="1">
-      <c r="A53" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="B53" s="21" t="inlineStr">
-        <is>
-          <t>35.190.1304</t>
-        </is>
-      </c>
-      <c r="C53" s="18" t="inlineStr">
-        <is>
-          <t>Sıva üstü PVC kablo kanalı — en az 100 x 35 mm, üç bölmeli (%25 müteahhit kârı dahil)</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E53" s="22" t="n">
-        <v>123</v>
-      </c>
-      <c r="F53" s="23">
-        <f>IFERROR(VLOOKUP($B53,'Fiyatlar'!$A:$I,9,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="G53" s="5">
-        <f>ROUND(E53*F53,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="n"/>
-      <c r="B54" s="7" t="n"/>
-      <c r="C54" s="24" t="inlineStr">
-        <is>
-          <t>ARA TOPLAM (KDV hariç)</t>
-        </is>
-      </c>
-      <c r="D54" s="7" t="n"/>
-      <c r="E54" s="7" t="n"/>
-      <c r="F54" s="7" t="n"/>
-      <c r="G54" s="9">
-        <f>SUM(G6:G53)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="n"/>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="25" t="inlineStr">
-        <is>
-          <t>KDV</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="5">
-        <f>G54*'Fiyatlar'!$F$3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="11" t="n"/>
-      <c r="B56" s="11" t="n"/>
-      <c r="C56" s="26" t="inlineStr">
+        <f>G49*'Fiyatlar'!$F$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="11" t="n"/>
+      <c r="B51" s="11" t="n"/>
+      <c r="C51" s="26" t="inlineStr">
         <is>
           <t>TEKLİF BEDELİ (KDV dâhil)</t>
         </is>
       </c>
-      <c r="D56" s="11" t="n"/>
-      <c r="E56" s="11" t="n"/>
-      <c r="F56" s="11" t="n"/>
-      <c r="G56" s="13">
-        <f>G54+G55</f>
+      <c r="D51" s="11" t="n"/>
+      <c r="E51" s="11" t="n"/>
+      <c r="F51" s="11" t="n"/>
+      <c r="G51" s="13">
+        <f>G49+G50</f>
         <v/>
       </c>
     </row>

</xml_diff>